<commit_message>
Sync monthly workload dashboard (2026-09-09 09:06)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C6267D6-D2CB-4CB3-9BBB-8258EE5E98DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0984B9B1-EF6B-4EDE-8BE5-7A1CFAB4EA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{17053454-EC3A-47CE-B50C-DF650D041A62}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{69867AB3-535F-423D-B17F-9FE4BD9A313D}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (21 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-03</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-09</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -697,7 +697,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3855F1D-1623-4716-99ED-5EDC912ED3C7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13AB372C-A7F1-4253-884A-E57D46E9EA71}">
   <dimension ref="A1:AF54"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2451,7 +2451,7 @@
         <v>43</v>
       </c>
       <c r="B39" s="10">
-        <v>327103</v>
+        <v>338679</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -2469,14 +2469,14 @@
       <c r="P39" s="8"/>
       <c r="Q39" s="8"/>
       <c r="R39" s="8">
-        <v>130841</v>
+        <v>136629</v>
       </c>
       <c r="S39" s="8"/>
       <c r="T39" s="8"/>
       <c r="U39" s="8"/>
       <c r="V39" s="8"/>
       <c r="W39" s="8">
-        <v>130841</v>
+        <v>136629</v>
       </c>
       <c r="X39" s="8"/>
       <c r="Y39" s="8"/>
@@ -2489,7 +2489,7 @@
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
       <c r="AF39" s="10">
-        <v>327103</v>
+        <v>338679</v>
       </c>
     </row>
     <row r="40" spans="1:32" ht="69" x14ac:dyDescent="0.25">
@@ -3043,7 +3043,7 @@
         <v>56</v>
       </c>
       <c r="B52" s="12">
-        <v>11573216</v>
+        <v>11584792</v>
       </c>
       <c r="C52" s="12">
         <v>403175</v>
@@ -3091,7 +3091,7 @@
         <v>180000</v>
       </c>
       <c r="R52" s="12">
-        <v>1133379</v>
+        <v>1139167</v>
       </c>
       <c r="S52" s="12">
         <v>1539976</v>
@@ -3106,7 +3106,7 @@
         <v>100926</v>
       </c>
       <c r="W52" s="12">
-        <v>1498838</v>
+        <v>1504626</v>
       </c>
       <c r="X52" s="12">
         <v>349950</v>
@@ -3133,7 +3133,7 @@
         <v>92000</v>
       </c>
       <c r="AF52" s="12">
-        <v>11573216</v>
+        <v>11584792</v>
       </c>
     </row>
     <row r="54" spans="1:32" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-09 10:17)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0984B9B1-EF6B-4EDE-8BE5-7A1CFAB4EA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{53458D76-64F9-4404-8FAB-CEDFC51536CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{69867AB3-535F-423D-B17F-9FE4BD9A313D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A77E88AE-6544-4B2B-B48E-925DB25E7F96}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,9 +39,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="59">
-  <si>
-    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (21 โครงการ PO)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="60">
+  <si>
+    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (22 โครงการ PO)</t>
   </si>
   <si>
     <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-09</t>
@@ -204,6 +204,9 @@
   </si>
   <si>
     <t>CRLEV-26-025  Achalaboon Residence</t>
+  </si>
+  <si>
+    <t>CRLEV-26-030  Peter KohLanta Residence</t>
   </si>
   <si>
     <t>K'Ink &amp; K'Cody Residence</t>
@@ -697,8 +700,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13AB372C-A7F1-4253-884A-E57D46E9EA71}">
-  <dimension ref="A1:AF54"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD617BA-78FA-484D-A319-00766E2BB694}">
+  <dimension ref="A1:AF56"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -1806,12 +1809,12 @@
         <v>341476</v>
       </c>
     </row>
-    <row r="26" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>55</v>
       </c>
       <c r="B26" s="10">
-        <v>164242</v>
+        <v>176436</v>
       </c>
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
@@ -1833,14 +1836,12 @@
       <c r="T26" s="8"/>
       <c r="U26" s="8"/>
       <c r="V26" s="8">
-        <v>50341</v>
+        <v>52931</v>
       </c>
       <c r="W26" s="8">
-        <v>83901</v>
-      </c>
-      <c r="X26" s="8">
-        <v>30000</v>
-      </c>
+        <v>123505</v>
+      </c>
+      <c r="X26" s="8"/>
       <c r="Y26" s="8"/>
       <c r="Z26" s="8"/>
       <c r="AA26" s="8"/>
@@ -1849,293 +1850,293 @@
       <c r="AD26" s="8"/>
       <c r="AE26" s="8"/>
       <c r="AF26" s="10">
+        <v>176436</v>
+      </c>
+    </row>
+    <row r="27" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A27" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="10">
         <v>164242</v>
       </c>
-    </row>
-    <row r="27" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" s="12">
-        <v>4484440</v>
-      </c>
-      <c r="C27" s="12">
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="8"/>
+      <c r="R27" s="8"/>
+      <c r="S27" s="8"/>
+      <c r="T27" s="8"/>
+      <c r="U27" s="8"/>
+      <c r="V27" s="8">
+        <v>50341</v>
+      </c>
+      <c r="W27" s="8">
+        <v>83901</v>
+      </c>
+      <c r="X27" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Y27" s="8"/>
+      <c r="Z27" s="8"/>
+      <c r="AA27" s="8"/>
+      <c r="AB27" s="8"/>
+      <c r="AC27" s="8"/>
+      <c r="AD27" s="8"/>
+      <c r="AE27" s="8"/>
+      <c r="AF27" s="10">
+        <v>164242</v>
+      </c>
+    </row>
+    <row r="28" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="12">
+        <v>4660876</v>
+      </c>
+      <c r="C28" s="12">
         <v>139012</v>
       </c>
-      <c r="D27" s="12">
+      <c r="D28" s="12">
         <v>231688</v>
       </c>
-      <c r="E27" s="12">
+      <c r="E28" s="12">
         <v>0</v>
       </c>
-      <c r="F27" s="12">
+      <c r="F28" s="12">
         <v>0</v>
       </c>
-      <c r="G27" s="12">
+      <c r="G28" s="12">
         <v>0</v>
       </c>
-      <c r="H27" s="12">
+      <c r="H28" s="12">
         <v>0</v>
       </c>
-      <c r="I27" s="12">
+      <c r="I28" s="12">
         <v>0</v>
       </c>
-      <c r="J27" s="12">
+      <c r="J28" s="12">
         <v>0</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K28" s="12">
         <v>0</v>
       </c>
-      <c r="L27" s="12">
+      <c r="L28" s="12">
         <v>0</v>
       </c>
-      <c r="M27" s="12">
+      <c r="M28" s="12">
         <v>0</v>
       </c>
-      <c r="N27" s="12">
+      <c r="N28" s="12">
         <v>0</v>
       </c>
-      <c r="O27" s="12">
+      <c r="O28" s="12">
         <v>229452</v>
       </c>
-      <c r="P27" s="12">
+      <c r="P28" s="12">
         <v>223986</v>
       </c>
-      <c r="Q27" s="12">
+      <c r="Q28" s="12">
         <v>229402</v>
       </c>
-      <c r="R27" s="12">
+      <c r="R28" s="12">
         <v>272600</v>
       </c>
-      <c r="S27" s="12">
+      <c r="S28" s="12">
         <v>337404</v>
       </c>
-      <c r="T27" s="12">
+      <c r="T28" s="12">
         <v>739676</v>
       </c>
-      <c r="U27" s="12">
+      <c r="U28" s="12">
         <v>327000</v>
       </c>
-      <c r="V27" s="12">
-        <v>353558</v>
-      </c>
-      <c r="W27" s="12">
-        <v>716892</v>
-      </c>
-      <c r="X27" s="12">
+      <c r="V28" s="12">
+        <v>406489</v>
+      </c>
+      <c r="W28" s="12">
+        <v>840397</v>
+      </c>
+      <c r="X28" s="12">
         <v>296922</v>
       </c>
-      <c r="Y27" s="12">
+      <c r="Y28" s="12">
         <v>155974</v>
       </c>
-      <c r="Z27" s="12">
+      <c r="Z28" s="12">
         <v>187274</v>
       </c>
-      <c r="AA27" s="12">
+      <c r="AA28" s="12">
         <v>0</v>
       </c>
-      <c r="AB27" s="12">
+      <c r="AB28" s="12">
         <v>0</v>
       </c>
-      <c r="AC27" s="12">
+      <c r="AC28" s="12">
         <v>0</v>
       </c>
-      <c r="AD27" s="12">
+      <c r="AD28" s="12">
         <v>43600</v>
       </c>
-      <c r="AE27" s="12">
+      <c r="AE28" s="12">
         <v>0</v>
       </c>
-      <c r="AF27" s="12">
-        <v>4484440</v>
-      </c>
-    </row>
-    <row r="29" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5"/>
-      <c r="O29" s="5"/>
-      <c r="P29" s="5"/>
-      <c r="Q29" s="5"/>
-      <c r="R29" s="5"/>
-      <c r="S29" s="5"/>
-      <c r="T29" s="5"/>
-      <c r="U29" s="5"/>
-      <c r="V29" s="5"/>
-      <c r="W29" s="5"/>
-      <c r="X29" s="5"/>
-      <c r="Y29" s="5"/>
-      <c r="Z29" s="5"/>
-      <c r="AA29" s="5"/>
-      <c r="AB29" s="5"/>
-      <c r="AC29" s="5"/>
-      <c r="AD29" s="5"/>
-      <c r="AE29" s="5"/>
-      <c r="AF29" s="5"/>
-    </row>
-    <row r="30" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="AF28" s="12">
+        <v>4660876</v>
+      </c>
+    </row>
+    <row r="30" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="5"/>
+      <c r="C30" s="5"/>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="5"/>
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+      <c r="N30" s="5"/>
+      <c r="O30" s="5"/>
+      <c r="P30" s="5"/>
+      <c r="Q30" s="5"/>
+      <c r="R30" s="5"/>
+      <c r="S30" s="5"/>
+      <c r="T30" s="5"/>
+      <c r="U30" s="5"/>
+      <c r="V30" s="5"/>
+      <c r="W30" s="5"/>
+      <c r="X30" s="5"/>
+      <c r="Y30" s="5"/>
+      <c r="Z30" s="5"/>
+      <c r="AA30" s="5"/>
+      <c r="AB30" s="5"/>
+      <c r="AC30" s="5"/>
+      <c r="AD30" s="5"/>
+      <c r="AE30" s="5"/>
+      <c r="AF30" s="5"/>
+    </row>
+    <row r="31" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C31" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D31" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="E31" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F31" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G31" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H31" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="I31" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J30" s="7" t="s">
+      <c r="J31" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K30" s="7" t="s">
+      <c r="K31" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="L30" s="7" t="s">
+      <c r="L31" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="M30" s="7" t="s">
+      <c r="M31" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N30" s="7" t="s">
+      <c r="N31" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="O30" s="7" t="s">
+      <c r="O31" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="P30" s="7" t="s">
+      <c r="P31" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Q30" s="7" t="s">
+      <c r="Q31" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="R30" s="7" t="s">
+      <c r="R31" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="S30" s="7" t="s">
+      <c r="S31" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="T30" s="7" t="s">
+      <c r="T31" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="U30" s="7" t="s">
+      <c r="U31" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="V30" s="7" t="s">
+      <c r="V31" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="W30" s="7" t="s">
+      <c r="W31" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="X30" s="7" t="s">
+      <c r="X31" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="Y30" s="7" t="s">
+      <c r="Y31" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="Z30" s="7" t="s">
+      <c r="Z31" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="AA30" s="7" t="s">
+      <c r="AA31" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AB30" s="7" t="s">
+      <c r="AB31" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="AC30" s="7" t="s">
+      <c r="AC31" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AD30" s="7" t="s">
+      <c r="AD31" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AE30" s="7" t="s">
+      <c r="AE31" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF30" s="6" t="s">
+      <c r="AF31" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A31" s="9" t="s">
+    <row r="32" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="10">
+      <c r="B32" s="10">
         <v>294109</v>
-      </c>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8"/>
-      <c r="I31" s="8"/>
-      <c r="J31" s="8"/>
-      <c r="K31" s="8"/>
-      <c r="L31" s="8"/>
-      <c r="M31" s="8"/>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8">
-        <v>130715</v>
-      </c>
-      <c r="P31" s="8"/>
-      <c r="Q31" s="8"/>
-      <c r="R31" s="8"/>
-      <c r="S31" s="8"/>
-      <c r="T31" s="8">
-        <v>130715</v>
-      </c>
-      <c r="U31" s="8"/>
-      <c r="V31" s="8">
-        <v>32679</v>
-      </c>
-      <c r="W31" s="8"/>
-      <c r="X31" s="8"/>
-      <c r="Y31" s="8"/>
-      <c r="Z31" s="8"/>
-      <c r="AA31" s="8"/>
-      <c r="AB31" s="8"/>
-      <c r="AC31" s="8"/>
-      <c r="AD31" s="8"/>
-      <c r="AE31" s="8"/>
-      <c r="AF31" s="10">
-        <v>294109</v>
-      </c>
-    </row>
-    <row r="32" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B32" s="10">
-        <v>409600</v>
       </c>
       <c r="C32" s="8"/>
       <c r="D32" s="8"/>
@@ -2149,23 +2150,23 @@
       <c r="L32" s="8"/>
       <c r="M32" s="8"/>
       <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="8">
-        <v>163840</v>
-      </c>
+      <c r="O32" s="8">
+        <v>130715</v>
+      </c>
+      <c r="P32" s="8"/>
       <c r="Q32" s="8"/>
       <c r="R32" s="8"/>
       <c r="S32" s="8"/>
-      <c r="T32" s="8"/>
+      <c r="T32" s="8">
+        <v>130715</v>
+      </c>
       <c r="U32" s="8"/>
-      <c r="V32" s="8"/>
-      <c r="W32" s="8">
-        <v>163840</v>
-      </c>
+      <c r="V32" s="8">
+        <v>32679</v>
+      </c>
+      <c r="W32" s="8"/>
       <c r="X32" s="8"/>
-      <c r="Y32" s="8">
-        <v>81920</v>
-      </c>
+      <c r="Y32" s="8"/>
       <c r="Z32" s="8"/>
       <c r="AA32" s="8"/>
       <c r="AB32" s="8"/>
@@ -2173,15 +2174,15 @@
       <c r="AD32" s="8"/>
       <c r="AE32" s="8"/>
       <c r="AF32" s="10">
+        <v>294109</v>
+      </c>
+    </row>
+    <row r="33" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A33" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B33" s="10">
         <v>409600</v>
-      </c>
-    </row>
-    <row r="33" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" s="10">
-        <v>576318</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -2195,23 +2196,23 @@
       <c r="L33" s="8"/>
       <c r="M33" s="8"/>
       <c r="N33" s="8"/>
-      <c r="O33" s="8">
-        <v>230527</v>
-      </c>
+      <c r="O33" s="8"/>
       <c r="P33" s="8">
-        <v>230527</v>
+        <v>163840</v>
       </c>
       <c r="Q33" s="8"/>
       <c r="R33" s="8"/>
       <c r="S33" s="8"/>
-      <c r="T33" s="8">
-        <v>115264</v>
-      </c>
+      <c r="T33" s="8"/>
       <c r="U33" s="8"/>
       <c r="V33" s="8"/>
-      <c r="W33" s="8"/>
+      <c r="W33" s="8">
+        <v>163840</v>
+      </c>
       <c r="X33" s="8"/>
-      <c r="Y33" s="8"/>
+      <c r="Y33" s="8">
+        <v>81920</v>
+      </c>
       <c r="Z33" s="8"/>
       <c r="AA33" s="8"/>
       <c r="AB33" s="8"/>
@@ -2219,15 +2220,15 @@
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
       <c r="AF33" s="10">
+        <v>409600</v>
+      </c>
+    </row>
+    <row r="34" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B34" s="10">
         <v>576318</v>
-      </c>
-    </row>
-    <row r="34" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B34" s="10">
-        <v>322960</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -2241,16 +2242,18 @@
       <c r="L34" s="8"/>
       <c r="M34" s="8"/>
       <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
+      <c r="O34" s="8">
+        <v>230527</v>
+      </c>
+      <c r="P34" s="8">
+        <v>230527</v>
+      </c>
       <c r="Q34" s="8"/>
-      <c r="R34" s="8">
-        <v>129184</v>
-      </c>
-      <c r="S34" s="8">
-        <v>193776</v>
-      </c>
-      <c r="T34" s="8"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="8"/>
+      <c r="T34" s="8">
+        <v>115264</v>
+      </c>
       <c r="U34" s="8"/>
       <c r="V34" s="8"/>
       <c r="W34" s="8"/>
@@ -2263,15 +2266,15 @@
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
       <c r="AF34" s="10">
+        <v>576318</v>
+      </c>
+    </row>
+    <row r="35" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B35" s="10">
         <v>322960</v>
-      </c>
-    </row>
-    <row r="35" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B35" s="10">
-        <v>252248</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -2288,16 +2291,18 @@
       <c r="O35" s="8"/>
       <c r="P35" s="8"/>
       <c r="Q35" s="8"/>
-      <c r="R35" s="8"/>
-      <c r="S35" s="8"/>
+      <c r="R35" s="8">
+        <v>129184</v>
+      </c>
+      <c r="S35" s="8">
+        <v>193776</v>
+      </c>
       <c r="T35" s="8"/>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
       <c r="W35" s="8"/>
       <c r="X35" s="8"/>
-      <c r="Y35" s="8">
-        <v>252248</v>
-      </c>
+      <c r="Y35" s="8"/>
       <c r="Z35" s="8"/>
       <c r="AA35" s="8"/>
       <c r="AB35" s="8"/>
@@ -2305,15 +2310,15 @@
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
       <c r="AF35" s="10">
-        <v>252248</v>
+        <v>322960</v>
       </c>
     </row>
     <row r="36" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B36" s="10">
-        <v>338450</v>
+        <v>252248</v>
       </c>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
@@ -2330,20 +2335,16 @@
       <c r="O36" s="8"/>
       <c r="P36" s="8"/>
       <c r="Q36" s="8"/>
-      <c r="R36" s="8">
-        <v>135380</v>
-      </c>
-      <c r="S36" s="8">
-        <v>135380</v>
-      </c>
-      <c r="T36" s="8">
-        <v>67690</v>
-      </c>
+      <c r="R36" s="8"/>
+      <c r="S36" s="8"/>
+      <c r="T36" s="8"/>
       <c r="U36" s="8"/>
       <c r="V36" s="8"/>
       <c r="W36" s="8"/>
       <c r="X36" s="8"/>
-      <c r="Y36" s="8"/>
+      <c r="Y36" s="8">
+        <v>252248</v>
+      </c>
       <c r="Z36" s="8"/>
       <c r="AA36" s="8"/>
       <c r="AB36" s="8"/>
@@ -2351,15 +2352,15 @@
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
       <c r="AF36" s="10">
+        <v>252248</v>
+      </c>
+    </row>
+    <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A37" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="10">
         <v>338450</v>
-      </c>
-    </row>
-    <row r="37" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B37" s="10">
-        <v>1156110</v>
       </c>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
@@ -2377,17 +2378,17 @@
       <c r="P37" s="8"/>
       <c r="Q37" s="8"/>
       <c r="R37" s="8">
-        <v>462444</v>
-      </c>
-      <c r="S37" s="8"/>
+        <v>135380</v>
+      </c>
+      <c r="S37" s="8">
+        <v>135380</v>
+      </c>
       <c r="T37" s="8">
-        <v>346833</v>
+        <v>67690</v>
       </c>
       <c r="U37" s="8"/>
       <c r="V37" s="8"/>
-      <c r="W37" s="8">
-        <v>346833</v>
-      </c>
+      <c r="W37" s="8"/>
       <c r="X37" s="8"/>
       <c r="Y37" s="8"/>
       <c r="Z37" s="8"/>
@@ -2397,15 +2398,15 @@
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
       <c r="AF37" s="10">
+        <v>338450</v>
+      </c>
+    </row>
+    <row r="38" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="10">
         <v>1156110</v>
-      </c>
-    </row>
-    <row r="38" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B38" s="10">
-        <v>594115</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2422,36 +2423,36 @@
       <c r="O38" s="8"/>
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
-      <c r="R38" s="8"/>
+      <c r="R38" s="8">
+        <v>462444</v>
+      </c>
       <c r="S38" s="8"/>
-      <c r="T38" s="8"/>
+      <c r="T38" s="8">
+        <v>346833</v>
+      </c>
       <c r="U38" s="8"/>
       <c r="V38" s="8"/>
-      <c r="W38" s="8"/>
+      <c r="W38" s="8">
+        <v>346833</v>
+      </c>
       <c r="X38" s="8"/>
-      <c r="Y38" s="8">
-        <v>237646</v>
-      </c>
-      <c r="Z38" s="8">
-        <v>237646</v>
-      </c>
-      <c r="AA38" s="8">
-        <v>118823</v>
-      </c>
+      <c r="Y38" s="8"/>
+      <c r="Z38" s="8"/>
+      <c r="AA38" s="8"/>
       <c r="AB38" s="8"/>
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
       <c r="AF38" s="10">
+        <v>1156110</v>
+      </c>
+    </row>
+    <row r="39" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="10">
         <v>594115</v>
-      </c>
-    </row>
-    <row r="39" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A39" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B39" s="10">
-        <v>338679</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -2468,36 +2469,36 @@
       <c r="O39" s="8"/>
       <c r="P39" s="8"/>
       <c r="Q39" s="8"/>
-      <c r="R39" s="8">
-        <v>136629</v>
-      </c>
+      <c r="R39" s="8"/>
       <c r="S39" s="8"/>
       <c r="T39" s="8"/>
       <c r="U39" s="8"/>
       <c r="V39" s="8"/>
-      <c r="W39" s="8">
-        <v>136629</v>
-      </c>
+      <c r="W39" s="8"/>
       <c r="X39" s="8"/>
-      <c r="Y39" s="8"/>
-      <c r="Z39" s="8"/>
+      <c r="Y39" s="8">
+        <v>237646</v>
+      </c>
+      <c r="Z39" s="8">
+        <v>237646</v>
+      </c>
       <c r="AA39" s="8">
-        <v>65421</v>
+        <v>118823</v>
       </c>
       <c r="AB39" s="8"/>
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
       <c r="AF39" s="10">
+        <v>594115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="10">
         <v>338679</v>
-      </c>
-    </row>
-    <row r="40" spans="1:32" ht="69" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B40" s="10">
-        <v>1707090</v>
       </c>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
@@ -2514,36 +2515,36 @@
       <c r="O40" s="8"/>
       <c r="P40" s="8"/>
       <c r="Q40" s="8"/>
-      <c r="R40" s="8"/>
-      <c r="S40" s="8">
-        <v>682836</v>
-      </c>
-      <c r="T40" s="8">
-        <v>682836</v>
-      </c>
-      <c r="U40" s="8">
-        <v>341418</v>
-      </c>
+      <c r="R40" s="8">
+        <v>136629</v>
+      </c>
+      <c r="S40" s="8"/>
+      <c r="T40" s="8"/>
+      <c r="U40" s="8"/>
       <c r="V40" s="8"/>
-      <c r="W40" s="8"/>
+      <c r="W40" s="8">
+        <v>136629</v>
+      </c>
       <c r="X40" s="8"/>
       <c r="Y40" s="8"/>
       <c r="Z40" s="8"/>
-      <c r="AA40" s="8"/>
+      <c r="AA40" s="8">
+        <v>65421</v>
+      </c>
       <c r="AB40" s="8"/>
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
       <c r="AF40" s="10">
-        <v>1707090</v>
+        <v>338679</v>
       </c>
     </row>
     <row r="41" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B41" s="10">
-        <v>80000</v>
+        <v>1707090</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
@@ -2560,14 +2561,16 @@
       <c r="O41" s="8"/>
       <c r="P41" s="8"/>
       <c r="Q41" s="8"/>
-      <c r="R41" s="8">
-        <v>32000</v>
-      </c>
+      <c r="R41" s="8"/>
       <c r="S41" s="8">
-        <v>48000</v>
-      </c>
-      <c r="T41" s="8"/>
-      <c r="U41" s="8"/>
+        <v>682836</v>
+      </c>
+      <c r="T41" s="8">
+        <v>682836</v>
+      </c>
+      <c r="U41" s="8">
+        <v>341418</v>
+      </c>
       <c r="V41" s="8"/>
       <c r="W41" s="8"/>
       <c r="X41" s="8"/>
@@ -2579,15 +2582,15 @@
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
       <c r="AF41" s="10">
-        <v>80000</v>
+        <v>1707090</v>
       </c>
     </row>
     <row r="42" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B42" s="10">
-        <v>1199960</v>
+        <v>80000</v>
       </c>
       <c r="C42" s="8"/>
       <c r="D42" s="8"/>
@@ -2604,36 +2607,34 @@
       <c r="O42" s="8"/>
       <c r="P42" s="8"/>
       <c r="Q42" s="8"/>
-      <c r="R42" s="8"/>
+      <c r="R42" s="8">
+        <v>32000</v>
+      </c>
       <c r="S42" s="8">
-        <v>479984</v>
+        <v>48000</v>
       </c>
       <c r="T42" s="8"/>
       <c r="U42" s="8"/>
       <c r="V42" s="8"/>
-      <c r="W42" s="8">
-        <v>479984</v>
-      </c>
+      <c r="W42" s="8"/>
       <c r="X42" s="8"/>
       <c r="Y42" s="8"/>
-      <c r="Z42" s="8">
-        <v>239992</v>
-      </c>
+      <c r="Z42" s="8"/>
       <c r="AA42" s="8"/>
       <c r="AB42" s="8"/>
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
       <c r="AF42" s="10">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+      <c r="A43" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="10">
         <v>1199960</v>
-      </c>
-    </row>
-    <row r="43" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A43" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B43" s="10">
-        <v>600000</v>
       </c>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
@@ -2647,39 +2648,39 @@
       <c r="L43" s="8"/>
       <c r="M43" s="8"/>
       <c r="N43" s="8"/>
-      <c r="O43" s="8">
-        <v>240000</v>
-      </c>
+      <c r="O43" s="8"/>
       <c r="P43" s="8"/>
-      <c r="Q43" s="8">
-        <v>180000</v>
-      </c>
-      <c r="R43" s="8">
-        <v>180000</v>
-      </c>
-      <c r="S43" s="8"/>
+      <c r="Q43" s="8"/>
+      <c r="R43" s="8"/>
+      <c r="S43" s="8">
+        <v>479984</v>
+      </c>
       <c r="T43" s="8"/>
       <c r="U43" s="8"/>
       <c r="V43" s="8"/>
-      <c r="W43" s="8"/>
+      <c r="W43" s="8">
+        <v>479984</v>
+      </c>
       <c r="X43" s="8"/>
       <c r="Y43" s="8"/>
-      <c r="Z43" s="8"/>
+      <c r="Z43" s="8">
+        <v>239992</v>
+      </c>
       <c r="AA43" s="8"/>
       <c r="AB43" s="8"/>
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
       <c r="AF43" s="10">
+        <v>1199960</v>
+      </c>
+    </row>
+    <row r="44" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B44" s="10">
         <v>600000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A44" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B44" s="10">
-        <v>317648</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -2694,14 +2695,14 @@
       <c r="M44" s="8"/>
       <c r="N44" s="8"/>
       <c r="O44" s="8">
-        <v>127059</v>
-      </c>
-      <c r="P44" s="8">
-        <v>127059</v>
-      </c>
-      <c r="Q44" s="8"/>
+        <v>240000</v>
+      </c>
+      <c r="P44" s="8"/>
+      <c r="Q44" s="8">
+        <v>180000</v>
+      </c>
       <c r="R44" s="8">
-        <v>63530</v>
+        <v>180000</v>
       </c>
       <c r="S44" s="8"/>
       <c r="T44" s="8"/>
@@ -2717,15 +2718,15 @@
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
       <c r="AF44" s="10">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B45" s="10">
         <v>317648</v>
-      </c>
-    </row>
-    <row r="45" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A45" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B45" s="10">
-        <v>832813</v>
       </c>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
@@ -2739,23 +2740,23 @@
       <c r="L45" s="8"/>
       <c r="M45" s="8"/>
       <c r="N45" s="8"/>
-      <c r="O45" s="8"/>
-      <c r="P45" s="8"/>
+      <c r="O45" s="8">
+        <v>127059</v>
+      </c>
+      <c r="P45" s="8">
+        <v>127059</v>
+      </c>
       <c r="Q45" s="8"/>
-      <c r="R45" s="8"/>
+      <c r="R45" s="8">
+        <v>63530</v>
+      </c>
       <c r="S45" s="8"/>
-      <c r="T45" s="8">
-        <v>333125</v>
-      </c>
-      <c r="U45" s="8">
-        <v>249844</v>
-      </c>
+      <c r="T45" s="8"/>
+      <c r="U45" s="8"/>
       <c r="V45" s="8"/>
       <c r="W45" s="8"/>
       <c r="X45" s="8"/>
-      <c r="Y45" s="8">
-        <v>249844</v>
-      </c>
+      <c r="Y45" s="8"/>
       <c r="Z45" s="8"/>
       <c r="AA45" s="8"/>
       <c r="AB45" s="8"/>
@@ -2763,22 +2764,18 @@
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
       <c r="AF45" s="10">
+        <v>317648</v>
+      </c>
+    </row>
+    <row r="46" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B46" s="10">
         <v>832813</v>
       </c>
-    </row>
-    <row r="46" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A46" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B46" s="10">
-        <v>341237</v>
-      </c>
-      <c r="C46" s="8">
-        <v>136495</v>
-      </c>
-      <c r="D46" s="8">
-        <v>136495</v>
-      </c>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
       <c r="E46" s="8"/>
       <c r="F46" s="8"/>
       <c r="G46" s="8"/>
@@ -2794,14 +2791,18 @@
       <c r="Q46" s="8"/>
       <c r="R46" s="8"/>
       <c r="S46" s="8"/>
-      <c r="T46" s="8"/>
-      <c r="U46" s="8"/>
-      <c r="V46" s="8">
-        <v>68247</v>
-      </c>
+      <c r="T46" s="8">
+        <v>333125</v>
+      </c>
+      <c r="U46" s="8">
+        <v>249844</v>
+      </c>
+      <c r="V46" s="8"/>
       <c r="W46" s="8"/>
       <c r="X46" s="8"/>
-      <c r="Y46" s="8"/>
+      <c r="Y46" s="8">
+        <v>249844</v>
+      </c>
       <c r="Z46" s="8"/>
       <c r="AA46" s="8"/>
       <c r="AB46" s="8"/>
@@ -2809,21 +2810,21 @@
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
       <c r="AF46" s="10">
+        <v>832813</v>
+      </c>
+    </row>
+    <row r="47" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B47" s="10">
         <v>341237</v>
       </c>
-    </row>
-    <row r="47" spans="1:32" ht="69" x14ac:dyDescent="0.25">
-      <c r="A47" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B47" s="10">
-        <v>666700</v>
-      </c>
       <c r="C47" s="8">
-        <v>266680</v>
+        <v>136495</v>
       </c>
       <c r="D47" s="8">
-        <v>266680</v>
+        <v>136495</v>
       </c>
       <c r="E47" s="8"/>
       <c r="F47" s="8"/>
@@ -2842,10 +2843,10 @@
       <c r="S47" s="8"/>
       <c r="T47" s="8"/>
       <c r="U47" s="8"/>
-      <c r="V47" s="8"/>
-      <c r="W47" s="8">
-        <v>133340</v>
-      </c>
+      <c r="V47" s="8">
+        <v>68247</v>
+      </c>
+      <c r="W47" s="8"/>
       <c r="X47" s="8"/>
       <c r="Y47" s="8"/>
       <c r="Z47" s="8"/>
@@ -2855,18 +2856,22 @@
       <c r="AD47" s="8"/>
       <c r="AE47" s="8"/>
       <c r="AF47" s="10">
+        <v>341237</v>
+      </c>
+    </row>
+    <row r="48" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+      <c r="A48" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B48" s="10">
         <v>666700</v>
       </c>
-    </row>
-    <row r="48" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A48" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B48" s="10">
-        <v>460000</v>
-      </c>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
+      <c r="C48" s="8">
+        <v>266680</v>
+      </c>
+      <c r="D48" s="8">
+        <v>266680</v>
+      </c>
       <c r="E48" s="8"/>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
@@ -2882,13 +2887,11 @@
       <c r="Q48" s="8"/>
       <c r="R48" s="8"/>
       <c r="S48" s="8"/>
-      <c r="T48" s="8">
-        <v>184000</v>
-      </c>
+      <c r="T48" s="8"/>
       <c r="U48" s="8"/>
       <c r="V48" s="8"/>
       <c r="W48" s="8">
-        <v>184000</v>
+        <v>133340</v>
       </c>
       <c r="X48" s="8"/>
       <c r="Y48" s="8"/>
@@ -2897,19 +2900,17 @@
       <c r="AB48" s="8"/>
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
-      <c r="AE48" s="8">
-        <v>92000</v>
-      </c>
+      <c r="AE48" s="8"/>
       <c r="AF48" s="10">
-        <v>460000</v>
+        <v>666700</v>
       </c>
     </row>
     <row r="49" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B49" s="10">
-        <v>206880</v>
+        <v>460000</v>
       </c>
       <c r="C49" s="8"/>
       <c r="D49" s="8"/>
@@ -2929,13 +2930,13 @@
       <c r="R49" s="8"/>
       <c r="S49" s="8"/>
       <c r="T49" s="8">
-        <v>82752</v>
-      </c>
-      <c r="U49" s="8">
-        <v>124128</v>
-      </c>
+        <v>184000</v>
+      </c>
+      <c r="U49" s="8"/>
       <c r="V49" s="8"/>
-      <c r="W49" s="8"/>
+      <c r="W49" s="8">
+        <v>184000</v>
+      </c>
       <c r="X49" s="8"/>
       <c r="Y49" s="8"/>
       <c r="Z49" s="8"/>
@@ -2943,17 +2944,19 @@
       <c r="AB49" s="8"/>
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
-      <c r="AE49" s="8"/>
+      <c r="AE49" s="8">
+        <v>92000</v>
+      </c>
       <c r="AF49" s="10">
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A50" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B50" s="10">
         <v>206880</v>
-      </c>
-    </row>
-    <row r="50" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A50" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B50" s="10">
-        <v>799875</v>
       </c>
       <c r="C50" s="8"/>
       <c r="D50" s="8"/>
@@ -2972,34 +2975,32 @@
       <c r="Q50" s="8"/>
       <c r="R50" s="8"/>
       <c r="S50" s="8"/>
-      <c r="T50" s="8"/>
+      <c r="T50" s="8">
+        <v>82752</v>
+      </c>
       <c r="U50" s="8">
-        <v>319950</v>
+        <v>124128</v>
       </c>
       <c r="V50" s="8"/>
       <c r="W50" s="8"/>
-      <c r="X50" s="8">
-        <v>319950</v>
-      </c>
+      <c r="X50" s="8"/>
       <c r="Y50" s="8"/>
       <c r="Z50" s="8"/>
       <c r="AA50" s="8"/>
-      <c r="AB50" s="8">
-        <v>159975</v>
-      </c>
+      <c r="AB50" s="8"/>
       <c r="AC50" s="8"/>
       <c r="AD50" s="8"/>
       <c r="AE50" s="8"/>
       <c r="AF50" s="10">
+        <v>206880</v>
+      </c>
+    </row>
+    <row r="51" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A51" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B51" s="10">
         <v>799875</v>
-      </c>
-    </row>
-    <row r="51" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A51" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B51" s="10">
-        <v>90000</v>
       </c>
       <c r="C51" s="8"/>
       <c r="D51" s="8"/>
@@ -3019,166 +3020,256 @@
       <c r="R51" s="8"/>
       <c r="S51" s="8"/>
       <c r="T51" s="8"/>
-      <c r="U51" s="8"/>
+      <c r="U51" s="8">
+        <v>319950</v>
+      </c>
       <c r="V51" s="8"/>
-      <c r="W51" s="8">
-        <v>60000</v>
-      </c>
+      <c r="W51" s="8"/>
       <c r="X51" s="8">
-        <v>30000</v>
+        <v>319950</v>
       </c>
       <c r="Y51" s="8"/>
       <c r="Z51" s="8"/>
       <c r="AA51" s="8"/>
-      <c r="AB51" s="8"/>
+      <c r="AB51" s="8">
+        <v>159975</v>
+      </c>
       <c r="AC51" s="8"/>
       <c r="AD51" s="8"/>
       <c r="AE51" s="8"/>
       <c r="AF51" s="10">
+        <v>799875</v>
+      </c>
+    </row>
+    <row r="52" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A52" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B52" s="10">
+        <v>411073</v>
+      </c>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="8"/>
+      <c r="G52" s="8"/>
+      <c r="H52" s="8"/>
+      <c r="I52" s="8"/>
+      <c r="J52" s="8"/>
+      <c r="K52" s="8"/>
+      <c r="L52" s="8"/>
+      <c r="M52" s="8"/>
+      <c r="N52" s="8"/>
+      <c r="O52" s="8"/>
+      <c r="P52" s="8"/>
+      <c r="Q52" s="8"/>
+      <c r="R52" s="8"/>
+      <c r="S52" s="8"/>
+      <c r="T52" s="8"/>
+      <c r="U52" s="8"/>
+      <c r="V52" s="8">
+        <v>164429</v>
+      </c>
+      <c r="W52" s="8">
+        <v>246644</v>
+      </c>
+      <c r="X52" s="8"/>
+      <c r="Y52" s="8"/>
+      <c r="Z52" s="8"/>
+      <c r="AA52" s="8"/>
+      <c r="AB52" s="8"/>
+      <c r="AC52" s="8"/>
+      <c r="AD52" s="8"/>
+      <c r="AE52" s="8"/>
+      <c r="AF52" s="10">
+        <v>411073</v>
+      </c>
+    </row>
+    <row r="53" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A53" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" s="10">
         <v>90000</v>
       </c>
-    </row>
-    <row r="52" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B52" s="12">
-        <v>11584792</v>
-      </c>
-      <c r="C52" s="12">
+      <c r="C53" s="8"/>
+      <c r="D53" s="8"/>
+      <c r="E53" s="8"/>
+      <c r="F53" s="8"/>
+      <c r="G53" s="8"/>
+      <c r="H53" s="8"/>
+      <c r="I53" s="8"/>
+      <c r="J53" s="8"/>
+      <c r="K53" s="8"/>
+      <c r="L53" s="8"/>
+      <c r="M53" s="8"/>
+      <c r="N53" s="8"/>
+      <c r="O53" s="8"/>
+      <c r="P53" s="8"/>
+      <c r="Q53" s="8"/>
+      <c r="R53" s="8"/>
+      <c r="S53" s="8"/>
+      <c r="T53" s="8"/>
+      <c r="U53" s="8"/>
+      <c r="V53" s="8"/>
+      <c r="W53" s="8">
+        <v>60000</v>
+      </c>
+      <c r="X53" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Y53" s="8"/>
+      <c r="Z53" s="8"/>
+      <c r="AA53" s="8"/>
+      <c r="AB53" s="8"/>
+      <c r="AC53" s="8"/>
+      <c r="AD53" s="8"/>
+      <c r="AE53" s="8"/>
+      <c r="AF53" s="10">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B54" s="12">
+        <v>11995865</v>
+      </c>
+      <c r="C54" s="12">
         <v>403175</v>
       </c>
-      <c r="D52" s="12">
+      <c r="D54" s="12">
         <v>403175</v>
       </c>
-      <c r="E52" s="12">
+      <c r="E54" s="12">
         <v>0</v>
       </c>
-      <c r="F52" s="12">
+      <c r="F54" s="12">
         <v>0</v>
       </c>
-      <c r="G52" s="12">
+      <c r="G54" s="12">
         <v>0</v>
       </c>
-      <c r="H52" s="12">
+      <c r="H54" s="12">
         <v>0</v>
       </c>
-      <c r="I52" s="12">
+      <c r="I54" s="12">
         <v>0</v>
       </c>
-      <c r="J52" s="12">
+      <c r="J54" s="12">
         <v>0</v>
       </c>
-      <c r="K52" s="12">
+      <c r="K54" s="12">
         <v>0</v>
       </c>
-      <c r="L52" s="12">
+      <c r="L54" s="12">
         <v>0</v>
       </c>
-      <c r="M52" s="12">
+      <c r="M54" s="12">
         <v>0</v>
       </c>
-      <c r="N52" s="12">
+      <c r="N54" s="12">
         <v>0</v>
       </c>
-      <c r="O52" s="12">
+      <c r="O54" s="12">
         <v>728301</v>
       </c>
-      <c r="P52" s="12">
+      <c r="P54" s="12">
         <v>521426</v>
       </c>
-      <c r="Q52" s="12">
+      <c r="Q54" s="12">
         <v>180000</v>
       </c>
-      <c r="R52" s="12">
+      <c r="R54" s="12">
         <v>1139167</v>
       </c>
-      <c r="S52" s="12">
+      <c r="S54" s="12">
         <v>1539976</v>
       </c>
-      <c r="T52" s="12">
+      <c r="T54" s="12">
         <v>1943215</v>
       </c>
-      <c r="U52" s="12">
+      <c r="U54" s="12">
         <v>1035340</v>
       </c>
-      <c r="V52" s="12">
-        <v>100926</v>
-      </c>
-      <c r="W52" s="12">
-        <v>1504626</v>
-      </c>
-      <c r="X52" s="12">
+      <c r="V54" s="12">
+        <v>265355</v>
+      </c>
+      <c r="W54" s="12">
+        <v>1751270</v>
+      </c>
+      <c r="X54" s="12">
         <v>349950</v>
       </c>
-      <c r="Y52" s="12">
+      <c r="Y54" s="12">
         <v>821658</v>
       </c>
-      <c r="Z52" s="12">
+      <c r="Z54" s="12">
         <v>477638</v>
       </c>
-      <c r="AA52" s="12">
+      <c r="AA54" s="12">
         <v>184244</v>
       </c>
-      <c r="AB52" s="12">
+      <c r="AB54" s="12">
         <v>159975</v>
       </c>
-      <c r="AC52" s="12">
+      <c r="AC54" s="12">
         <v>0</v>
       </c>
-      <c r="AD52" s="12">
+      <c r="AD54" s="12">
         <v>0</v>
       </c>
-      <c r="AE52" s="12">
+      <c r="AE54" s="12">
         <v>92000</v>
       </c>
-      <c r="AF52" s="12">
-        <v>11584792</v>
-      </c>
-    </row>
-    <row r="54" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A54" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
-      <c r="I54" s="4"/>
-      <c r="J54" s="4"/>
-      <c r="K54" s="4"/>
-      <c r="L54" s="4"/>
-      <c r="M54" s="4"/>
-      <c r="N54" s="4"/>
-      <c r="O54" s="4"/>
-      <c r="P54" s="4"/>
-      <c r="Q54" s="4"/>
-      <c r="R54" s="4"/>
-      <c r="S54" s="4"/>
-      <c r="T54" s="4"/>
-      <c r="U54" s="4"/>
-      <c r="V54" s="4"/>
-      <c r="W54" s="4"/>
-      <c r="X54" s="4"/>
-      <c r="Y54" s="4"/>
-      <c r="Z54" s="4"/>
-      <c r="AA54" s="4"/>
-      <c r="AB54" s="4"/>
-      <c r="AC54" s="4"/>
-      <c r="AD54" s="4"/>
-      <c r="AE54" s="4"/>
-      <c r="AF54" s="4"/>
+      <c r="AF54" s="12">
+        <v>11995865</v>
+      </c>
+    </row>
+    <row r="56" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A56" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+      <c r="D56" s="4"/>
+      <c r="E56" s="4"/>
+      <c r="F56" s="4"/>
+      <c r="G56" s="4"/>
+      <c r="H56" s="4"/>
+      <c r="I56" s="4"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+      <c r="O56" s="4"/>
+      <c r="P56" s="4"/>
+      <c r="Q56" s="4"/>
+      <c r="R56" s="4"/>
+      <c r="S56" s="4"/>
+      <c r="T56" s="4"/>
+      <c r="U56" s="4"/>
+      <c r="V56" s="4"/>
+      <c r="W56" s="4"/>
+      <c r="X56" s="4"/>
+      <c r="Y56" s="4"/>
+      <c r="Z56" s="4"/>
+      <c r="AA56" s="4"/>
+      <c r="AB56" s="4"/>
+      <c r="AC56" s="4"/>
+      <c r="AD56" s="4"/>
+      <c r="AE56" s="4"/>
+      <c r="AF56" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="A2:AF2"/>
-    <mergeCell ref="A54:AF54"/>
+    <mergeCell ref="A56:AF56"/>
     <mergeCell ref="A4:AF4"/>
-    <mergeCell ref="A29:AF29"/>
+    <mergeCell ref="A30:AF30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-09 16:07)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53458D76-64F9-4404-8FAB-CEDFC51536CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFCB84DD-5C02-42A6-AB79-29CB1CC3D2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A77E88AE-6544-4B2B-B48E-925DB25E7F96}"/>
+    <workbookView xWindow="6576" yWindow="0" windowWidth="13572" windowHeight="10368" xr2:uid="{F00F8ECD-36FB-4083-AF76-2D702A2A26FB}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -700,7 +700,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CD617BA-78FA-484D-A319-00766E2BB694}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBFA1E18-B2F5-4CA2-92E8-4A6F7427DF2E}">
   <dimension ref="A1:AF56"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-11 08:46)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFCB84DD-5C02-42A6-AB79-29CB1CC3D2D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D25490A4-1D00-4284-8117-616511255501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6576" yWindow="0" windowWidth="13572" windowHeight="10368" xr2:uid="{F00F8ECD-36FB-4083-AF76-2D702A2A26FB}"/>
+    <workbookView xWindow="6924" yWindow="348" windowWidth="13572" windowHeight="10368" xr2:uid="{1523805D-A87C-4F10-A9DF-3C38D3F24A38}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (22 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-09</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-11</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -700,7 +700,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBFA1E18-B2F5-4CA2-92E8-4A6F7427DF2E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7006E00E-6FAE-4795-BDC2-11094AA796AD}">
   <dimension ref="A1:AF56"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 11:56)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D25490A4-1D00-4284-8117-616511255501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF742029-345F-4299-BC39-DFC41076DE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6924" yWindow="348" windowWidth="13572" windowHeight="10368" xr2:uid="{1523805D-A87C-4F10-A9DF-3C38D3F24A38}"/>
+    <workbookView xWindow="7272" yWindow="696" windowWidth="13572" windowHeight="10368" xr2:uid="{4305E47D-3950-4BDC-B968-2DDF74415905}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,12 +39,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="60">
-  <si>
-    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (22 โครงการ PO)</t>
-  </si>
-  <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-11</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="61">
+  <si>
+    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (23 โครงการ PO)</t>
+  </si>
+  <si>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-14</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -207,6 +207,9 @@
   </si>
   <si>
     <t>CRLEV-26-030  Peter KohLanta Residence</t>
+  </si>
+  <si>
+    <t>MMJ : AP บ้านกลางเมืองคุณมอส</t>
   </si>
   <si>
     <t>K'Ink &amp; K'Cody Residence</t>
@@ -700,8 +703,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7006E00E-6FAE-4795-BDC2-11094AA796AD}">
-  <dimension ref="A1:AF56"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EBA1058-08C8-4174-AD23-659D8FB8F588}">
+  <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -1858,7 +1861,7 @@
         <v>56</v>
       </c>
       <c r="B27" s="10">
-        <v>164242</v>
+        <v>171149</v>
       </c>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
@@ -1880,10 +1883,10 @@
       <c r="T27" s="8"/>
       <c r="U27" s="8"/>
       <c r="V27" s="8">
-        <v>50341</v>
+        <v>52931</v>
       </c>
       <c r="W27" s="8">
-        <v>83901</v>
+        <v>88218</v>
       </c>
       <c r="X27" s="8">
         <v>30000</v>
@@ -1896,293 +1899,293 @@
       <c r="AD27" s="8"/>
       <c r="AE27" s="8"/>
       <c r="AF27" s="10">
+        <v>171149</v>
+      </c>
+    </row>
+    <row r="28" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A28" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="10">
         <v>164242</v>
       </c>
-    </row>
-    <row r="28" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="B28" s="12">
-        <v>4660876</v>
-      </c>
-      <c r="C28" s="12">
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="8"/>
+      <c r="U28" s="8"/>
+      <c r="V28" s="8">
+        <v>50341</v>
+      </c>
+      <c r="W28" s="8">
+        <v>83901</v>
+      </c>
+      <c r="X28" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Y28" s="8"/>
+      <c r="Z28" s="8"/>
+      <c r="AA28" s="8"/>
+      <c r="AB28" s="8"/>
+      <c r="AC28" s="8"/>
+      <c r="AD28" s="8"/>
+      <c r="AE28" s="8"/>
+      <c r="AF28" s="10">
+        <v>164242</v>
+      </c>
+    </row>
+    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B29" s="12">
+        <v>4832025</v>
+      </c>
+      <c r="C29" s="12">
         <v>139012</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D29" s="12">
         <v>231688</v>
       </c>
-      <c r="E28" s="12">
+      <c r="E29" s="12">
         <v>0</v>
       </c>
-      <c r="F28" s="12">
+      <c r="F29" s="12">
         <v>0</v>
       </c>
-      <c r="G28" s="12">
+      <c r="G29" s="12">
         <v>0</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H29" s="12">
         <v>0</v>
       </c>
-      <c r="I28" s="12">
+      <c r="I29" s="12">
         <v>0</v>
       </c>
-      <c r="J28" s="12">
+      <c r="J29" s="12">
         <v>0</v>
       </c>
-      <c r="K28" s="12">
+      <c r="K29" s="12">
         <v>0</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L29" s="12">
         <v>0</v>
       </c>
-      <c r="M28" s="12">
+      <c r="M29" s="12">
         <v>0</v>
       </c>
-      <c r="N28" s="12">
+      <c r="N29" s="12">
         <v>0</v>
       </c>
-      <c r="O28" s="12">
+      <c r="O29" s="12">
         <v>229452</v>
       </c>
-      <c r="P28" s="12">
+      <c r="P29" s="12">
         <v>223986</v>
       </c>
-      <c r="Q28" s="12">
+      <c r="Q29" s="12">
         <v>229402</v>
       </c>
-      <c r="R28" s="12">
+      <c r="R29" s="12">
         <v>272600</v>
       </c>
-      <c r="S28" s="12">
+      <c r="S29" s="12">
         <v>337404</v>
       </c>
-      <c r="T28" s="12">
+      <c r="T29" s="12">
         <v>739676</v>
       </c>
-      <c r="U28" s="12">
+      <c r="U29" s="12">
         <v>327000</v>
       </c>
-      <c r="V28" s="12">
-        <v>406489</v>
-      </c>
-      <c r="W28" s="12">
-        <v>840397</v>
-      </c>
-      <c r="X28" s="12">
-        <v>296922</v>
-      </c>
-      <c r="Y28" s="12">
+      <c r="V29" s="12">
+        <v>459420</v>
+      </c>
+      <c r="W29" s="12">
+        <v>928615</v>
+      </c>
+      <c r="X29" s="12">
+        <v>326922</v>
+      </c>
+      <c r="Y29" s="12">
         <v>155974</v>
       </c>
-      <c r="Z28" s="12">
+      <c r="Z29" s="12">
         <v>187274</v>
       </c>
-      <c r="AA28" s="12">
+      <c r="AA29" s="12">
         <v>0</v>
       </c>
-      <c r="AB28" s="12">
+      <c r="AB29" s="12">
         <v>0</v>
       </c>
-      <c r="AC28" s="12">
+      <c r="AC29" s="12">
         <v>0</v>
       </c>
-      <c r="AD28" s="12">
+      <c r="AD29" s="12">
         <v>43600</v>
       </c>
-      <c r="AE28" s="12">
+      <c r="AE29" s="12">
         <v>0</v>
       </c>
-      <c r="AF28" s="12">
-        <v>4660876</v>
-      </c>
-    </row>
-    <row r="30" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
-      <c r="E30" s="5"/>
-      <c r="F30" s="5"/>
-      <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-      <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
-      <c r="K30" s="5"/>
-      <c r="L30" s="5"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="5"/>
-      <c r="O30" s="5"/>
-      <c r="P30" s="5"/>
-      <c r="Q30" s="5"/>
-      <c r="R30" s="5"/>
-      <c r="S30" s="5"/>
-      <c r="T30" s="5"/>
-      <c r="U30" s="5"/>
-      <c r="V30" s="5"/>
-      <c r="W30" s="5"/>
-      <c r="X30" s="5"/>
-      <c r="Y30" s="5"/>
-      <c r="Z30" s="5"/>
-      <c r="AA30" s="5"/>
-      <c r="AB30" s="5"/>
-      <c r="AC30" s="5"/>
-      <c r="AD30" s="5"/>
-      <c r="AE30" s="5"/>
-      <c r="AF30" s="5"/>
-    </row>
-    <row r="31" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+      <c r="AF29" s="12">
+        <v>4832025</v>
+      </c>
+    </row>
+    <row r="31" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
+      <c r="M31" s="5"/>
+      <c r="N31" s="5"/>
+      <c r="O31" s="5"/>
+      <c r="P31" s="5"/>
+      <c r="Q31" s="5"/>
+      <c r="R31" s="5"/>
+      <c r="S31" s="5"/>
+      <c r="T31" s="5"/>
+      <c r="U31" s="5"/>
+      <c r="V31" s="5"/>
+      <c r="W31" s="5"/>
+      <c r="X31" s="5"/>
+      <c r="Y31" s="5"/>
+      <c r="Z31" s="5"/>
+      <c r="AA31" s="5"/>
+      <c r="AB31" s="5"/>
+      <c r="AC31" s="5"/>
+      <c r="AD31" s="5"/>
+      <c r="AE31" s="5"/>
+      <c r="AF31" s="5"/>
+    </row>
+    <row r="32" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B32" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C32" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D32" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E31" s="7" t="s">
+      <c r="E32" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F32" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G31" s="7" t="s">
+      <c r="G32" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H31" s="7" t="s">
+      <c r="H32" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I31" s="7" t="s">
+      <c r="I32" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J31" s="7" t="s">
+      <c r="J32" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K31" s="7" t="s">
+      <c r="K32" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="L31" s="7" t="s">
+      <c r="L32" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="M31" s="7" t="s">
+      <c r="M32" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N31" s="7" t="s">
+      <c r="N32" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="O31" s="7" t="s">
+      <c r="O32" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="P31" s="7" t="s">
+      <c r="P32" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Q31" s="7" t="s">
+      <c r="Q32" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="R31" s="7" t="s">
+      <c r="R32" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="S31" s="7" t="s">
+      <c r="S32" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="T31" s="7" t="s">
+      <c r="T32" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="U31" s="7" t="s">
+      <c r="U32" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="V31" s="7" t="s">
+      <c r="V32" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="W31" s="7" t="s">
+      <c r="W32" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="X31" s="7" t="s">
+      <c r="X32" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="Y31" s="7" t="s">
+      <c r="Y32" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="Z31" s="7" t="s">
+      <c r="Z32" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="AA31" s="7" t="s">
+      <c r="AA32" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AB31" s="7" t="s">
+      <c r="AB32" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="AC31" s="7" t="s">
+      <c r="AC32" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AD31" s="7" t="s">
+      <c r="AD32" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AE31" s="7" t="s">
+      <c r="AE32" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF31" s="6" t="s">
+      <c r="AF32" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A32" s="9" t="s">
+    <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A33" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B32" s="10">
+      <c r="B33" s="10">
         <v>294109</v>
-      </c>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8"/>
-      <c r="I32" s="8"/>
-      <c r="J32" s="8"/>
-      <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="8"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8">
-        <v>130715</v>
-      </c>
-      <c r="P32" s="8"/>
-      <c r="Q32" s="8"/>
-      <c r="R32" s="8"/>
-      <c r="S32" s="8"/>
-      <c r="T32" s="8">
-        <v>130715</v>
-      </c>
-      <c r="U32" s="8"/>
-      <c r="V32" s="8">
-        <v>32679</v>
-      </c>
-      <c r="W32" s="8"/>
-      <c r="X32" s="8"/>
-      <c r="Y32" s="8"/>
-      <c r="Z32" s="8"/>
-      <c r="AA32" s="8"/>
-      <c r="AB32" s="8"/>
-      <c r="AC32" s="8"/>
-      <c r="AD32" s="8"/>
-      <c r="AE32" s="8"/>
-      <c r="AF32" s="10">
-        <v>294109</v>
-      </c>
-    </row>
-    <row r="33" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B33" s="10">
-        <v>409600</v>
       </c>
       <c r="C33" s="8"/>
       <c r="D33" s="8"/>
@@ -2196,23 +2199,23 @@
       <c r="L33" s="8"/>
       <c r="M33" s="8"/>
       <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="8">
-        <v>163840</v>
-      </c>
+      <c r="O33" s="8">
+        <v>130715</v>
+      </c>
+      <c r="P33" s="8"/>
       <c r="Q33" s="8"/>
       <c r="R33" s="8"/>
       <c r="S33" s="8"/>
-      <c r="T33" s="8"/>
+      <c r="T33" s="8">
+        <v>130715</v>
+      </c>
       <c r="U33" s="8"/>
-      <c r="V33" s="8"/>
-      <c r="W33" s="8">
-        <v>163840</v>
-      </c>
+      <c r="V33" s="8">
+        <v>32679</v>
+      </c>
+      <c r="W33" s="8"/>
       <c r="X33" s="8"/>
-      <c r="Y33" s="8">
-        <v>81920</v>
-      </c>
+      <c r="Y33" s="8"/>
       <c r="Z33" s="8"/>
       <c r="AA33" s="8"/>
       <c r="AB33" s="8"/>
@@ -2220,15 +2223,15 @@
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
       <c r="AF33" s="10">
+        <v>294109</v>
+      </c>
+    </row>
+    <row r="34" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A34" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="10">
         <v>409600</v>
-      </c>
-    </row>
-    <row r="34" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" s="10">
-        <v>576318</v>
       </c>
       <c r="C34" s="8"/>
       <c r="D34" s="8"/>
@@ -2242,23 +2245,23 @@
       <c r="L34" s="8"/>
       <c r="M34" s="8"/>
       <c r="N34" s="8"/>
-      <c r="O34" s="8">
-        <v>230527</v>
-      </c>
+      <c r="O34" s="8"/>
       <c r="P34" s="8">
-        <v>230527</v>
+        <v>163840</v>
       </c>
       <c r="Q34" s="8"/>
       <c r="R34" s="8"/>
       <c r="S34" s="8"/>
-      <c r="T34" s="8">
-        <v>115264</v>
-      </c>
+      <c r="T34" s="8"/>
       <c r="U34" s="8"/>
       <c r="V34" s="8"/>
-      <c r="W34" s="8"/>
+      <c r="W34" s="8">
+        <v>163840</v>
+      </c>
       <c r="X34" s="8"/>
-      <c r="Y34" s="8"/>
+      <c r="Y34" s="8">
+        <v>81920</v>
+      </c>
       <c r="Z34" s="8"/>
       <c r="AA34" s="8"/>
       <c r="AB34" s="8"/>
@@ -2266,15 +2269,15 @@
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
       <c r="AF34" s="10">
+        <v>409600</v>
+      </c>
+    </row>
+    <row r="35" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="10">
         <v>576318</v>
-      </c>
-    </row>
-    <row r="35" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B35" s="10">
-        <v>322960</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -2288,16 +2291,18 @@
       <c r="L35" s="8"/>
       <c r="M35" s="8"/>
       <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
+      <c r="O35" s="8">
+        <v>230527</v>
+      </c>
+      <c r="P35" s="8">
+        <v>230527</v>
+      </c>
       <c r="Q35" s="8"/>
-      <c r="R35" s="8">
-        <v>129184</v>
-      </c>
-      <c r="S35" s="8">
-        <v>193776</v>
-      </c>
-      <c r="T35" s="8"/>
+      <c r="R35" s="8"/>
+      <c r="S35" s="8"/>
+      <c r="T35" s="8">
+        <v>115264</v>
+      </c>
       <c r="U35" s="8"/>
       <c r="V35" s="8"/>
       <c r="W35" s="8"/>
@@ -2310,15 +2315,15 @@
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
       <c r="AF35" s="10">
+        <v>576318</v>
+      </c>
+    </row>
+    <row r="36" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A36" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="10">
         <v>322960</v>
-      </c>
-    </row>
-    <row r="36" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A36" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B36" s="10">
-        <v>252248</v>
       </c>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
@@ -2335,16 +2340,18 @@
       <c r="O36" s="8"/>
       <c r="P36" s="8"/>
       <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
-      <c r="S36" s="8"/>
+      <c r="R36" s="8">
+        <v>129184</v>
+      </c>
+      <c r="S36" s="8">
+        <v>193776</v>
+      </c>
       <c r="T36" s="8"/>
       <c r="U36" s="8"/>
       <c r="V36" s="8"/>
       <c r="W36" s="8"/>
       <c r="X36" s="8"/>
-      <c r="Y36" s="8">
-        <v>252248</v>
-      </c>
+      <c r="Y36" s="8"/>
       <c r="Z36" s="8"/>
       <c r="AA36" s="8"/>
       <c r="AB36" s="8"/>
@@ -2352,15 +2359,15 @@
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
       <c r="AF36" s="10">
-        <v>252248</v>
+        <v>322960</v>
       </c>
     </row>
     <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B37" s="10">
-        <v>338450</v>
+        <v>252248</v>
       </c>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
@@ -2377,20 +2384,16 @@
       <c r="O37" s="8"/>
       <c r="P37" s="8"/>
       <c r="Q37" s="8"/>
-      <c r="R37" s="8">
-        <v>135380</v>
-      </c>
-      <c r="S37" s="8">
-        <v>135380</v>
-      </c>
-      <c r="T37" s="8">
-        <v>67690</v>
-      </c>
+      <c r="R37" s="8"/>
+      <c r="S37" s="8"/>
+      <c r="T37" s="8"/>
       <c r="U37" s="8"/>
       <c r="V37" s="8"/>
       <c r="W37" s="8"/>
       <c r="X37" s="8"/>
-      <c r="Y37" s="8"/>
+      <c r="Y37" s="8">
+        <v>252248</v>
+      </c>
       <c r="Z37" s="8"/>
       <c r="AA37" s="8"/>
       <c r="AB37" s="8"/>
@@ -2398,15 +2401,15 @@
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
       <c r="AF37" s="10">
+        <v>252248</v>
+      </c>
+    </row>
+    <row r="38" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A38" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="10">
         <v>338450</v>
-      </c>
-    </row>
-    <row r="38" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B38" s="10">
-        <v>1156110</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2424,17 +2427,17 @@
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8">
-        <v>462444</v>
-      </c>
-      <c r="S38" s="8"/>
+        <v>135380</v>
+      </c>
+      <c r="S38" s="8">
+        <v>135380</v>
+      </c>
       <c r="T38" s="8">
-        <v>346833</v>
+        <v>67690</v>
       </c>
       <c r="U38" s="8"/>
       <c r="V38" s="8"/>
-      <c r="W38" s="8">
-        <v>346833</v>
-      </c>
+      <c r="W38" s="8"/>
       <c r="X38" s="8"/>
       <c r="Y38" s="8"/>
       <c r="Z38" s="8"/>
@@ -2444,15 +2447,15 @@
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
       <c r="AF38" s="10">
+        <v>338450</v>
+      </c>
+    </row>
+    <row r="39" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="10">
         <v>1156110</v>
-      </c>
-    </row>
-    <row r="39" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A39" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="10">
-        <v>594115</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -2469,36 +2472,36 @@
       <c r="O39" s="8"/>
       <c r="P39" s="8"/>
       <c r="Q39" s="8"/>
-      <c r="R39" s="8"/>
+      <c r="R39" s="8">
+        <v>462444</v>
+      </c>
       <c r="S39" s="8"/>
-      <c r="T39" s="8"/>
+      <c r="T39" s="8">
+        <v>346833</v>
+      </c>
       <c r="U39" s="8"/>
       <c r="V39" s="8"/>
-      <c r="W39" s="8"/>
+      <c r="W39" s="8">
+        <v>346833</v>
+      </c>
       <c r="X39" s="8"/>
-      <c r="Y39" s="8">
-        <v>237646</v>
-      </c>
-      <c r="Z39" s="8">
-        <v>237646</v>
-      </c>
-      <c r="AA39" s="8">
-        <v>118823</v>
-      </c>
+      <c r="Y39" s="8"/>
+      <c r="Z39" s="8"/>
+      <c r="AA39" s="8"/>
       <c r="AB39" s="8"/>
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
       <c r="AF39" s="10">
+        <v>1156110</v>
+      </c>
+    </row>
+    <row r="40" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="10">
         <v>594115</v>
-      </c>
-    </row>
-    <row r="40" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A40" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" s="10">
-        <v>338679</v>
       </c>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
@@ -2515,36 +2518,36 @@
       <c r="O40" s="8"/>
       <c r="P40" s="8"/>
       <c r="Q40" s="8"/>
-      <c r="R40" s="8">
-        <v>136629</v>
-      </c>
+      <c r="R40" s="8"/>
       <c r="S40" s="8"/>
       <c r="T40" s="8"/>
       <c r="U40" s="8"/>
       <c r="V40" s="8"/>
-      <c r="W40" s="8">
-        <v>136629</v>
-      </c>
+      <c r="W40" s="8"/>
       <c r="X40" s="8"/>
-      <c r="Y40" s="8"/>
-      <c r="Z40" s="8"/>
+      <c r="Y40" s="8">
+        <v>237646</v>
+      </c>
+      <c r="Z40" s="8">
+        <v>237646</v>
+      </c>
       <c r="AA40" s="8">
-        <v>65421</v>
+        <v>118823</v>
       </c>
       <c r="AB40" s="8"/>
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
       <c r="AF40" s="10">
+        <v>594115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A41" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="10">
         <v>338679</v>
-      </c>
-    </row>
-    <row r="41" spans="1:32" ht="69" x14ac:dyDescent="0.25">
-      <c r="A41" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="B41" s="10">
-        <v>1707090</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
@@ -2561,36 +2564,36 @@
       <c r="O41" s="8"/>
       <c r="P41" s="8"/>
       <c r="Q41" s="8"/>
-      <c r="R41" s="8"/>
-      <c r="S41" s="8">
-        <v>682836</v>
-      </c>
-      <c r="T41" s="8">
-        <v>682836</v>
-      </c>
-      <c r="U41" s="8">
-        <v>341418</v>
-      </c>
+      <c r="R41" s="8">
+        <v>136629</v>
+      </c>
+      <c r="S41" s="8"/>
+      <c r="T41" s="8"/>
+      <c r="U41" s="8"/>
       <c r="V41" s="8"/>
-      <c r="W41" s="8"/>
+      <c r="W41" s="8">
+        <v>136629</v>
+      </c>
       <c r="X41" s="8"/>
       <c r="Y41" s="8"/>
       <c r="Z41" s="8"/>
-      <c r="AA41" s="8"/>
+      <c r="AA41" s="8">
+        <v>65421</v>
+      </c>
       <c r="AB41" s="8"/>
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
       <c r="AF41" s="10">
-        <v>1707090</v>
+        <v>338679</v>
       </c>
     </row>
     <row r="42" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B42" s="10">
-        <v>80000</v>
+        <v>1707090</v>
       </c>
       <c r="C42" s="8"/>
       <c r="D42" s="8"/>
@@ -2607,14 +2610,16 @@
       <c r="O42" s="8"/>
       <c r="P42" s="8"/>
       <c r="Q42" s="8"/>
-      <c r="R42" s="8">
-        <v>32000</v>
-      </c>
+      <c r="R42" s="8"/>
       <c r="S42" s="8">
-        <v>48000</v>
-      </c>
-      <c r="T42" s="8"/>
-      <c r="U42" s="8"/>
+        <v>682836</v>
+      </c>
+      <c r="T42" s="8">
+        <v>682836</v>
+      </c>
+      <c r="U42" s="8">
+        <v>341418</v>
+      </c>
       <c r="V42" s="8"/>
       <c r="W42" s="8"/>
       <c r="X42" s="8"/>
@@ -2626,15 +2631,15 @@
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
       <c r="AF42" s="10">
-        <v>80000</v>
+        <v>1707090</v>
       </c>
     </row>
     <row r="43" spans="1:32" ht="69" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B43" s="10">
-        <v>1199960</v>
+        <v>80000</v>
       </c>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
@@ -2651,36 +2656,34 @@
       <c r="O43" s="8"/>
       <c r="P43" s="8"/>
       <c r="Q43" s="8"/>
-      <c r="R43" s="8"/>
+      <c r="R43" s="8">
+        <v>32000</v>
+      </c>
       <c r="S43" s="8">
-        <v>479984</v>
+        <v>48000</v>
       </c>
       <c r="T43" s="8"/>
       <c r="U43" s="8"/>
       <c r="V43" s="8"/>
-      <c r="W43" s="8">
-        <v>479984</v>
-      </c>
+      <c r="W43" s="8"/>
       <c r="X43" s="8"/>
       <c r="Y43" s="8"/>
-      <c r="Z43" s="8">
-        <v>239992</v>
-      </c>
+      <c r="Z43" s="8"/>
       <c r="AA43" s="8"/>
       <c r="AB43" s="8"/>
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
       <c r="AF43" s="10">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="10">
         <v>1199960</v>
-      </c>
-    </row>
-    <row r="44" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A44" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B44" s="10">
-        <v>600000</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -2694,39 +2697,39 @@
       <c r="L44" s="8"/>
       <c r="M44" s="8"/>
       <c r="N44" s="8"/>
-      <c r="O44" s="8">
-        <v>240000</v>
-      </c>
+      <c r="O44" s="8"/>
       <c r="P44" s="8"/>
-      <c r="Q44" s="8">
-        <v>180000</v>
-      </c>
-      <c r="R44" s="8">
-        <v>180000</v>
-      </c>
-      <c r="S44" s="8"/>
+      <c r="Q44" s="8"/>
+      <c r="R44" s="8"/>
+      <c r="S44" s="8">
+        <v>479984</v>
+      </c>
       <c r="T44" s="8"/>
       <c r="U44" s="8"/>
       <c r="V44" s="8"/>
-      <c r="W44" s="8"/>
+      <c r="W44" s="8">
+        <v>479984</v>
+      </c>
       <c r="X44" s="8"/>
       <c r="Y44" s="8"/>
-      <c r="Z44" s="8"/>
+      <c r="Z44" s="8">
+        <v>239992</v>
+      </c>
       <c r="AA44" s="8"/>
       <c r="AB44" s="8"/>
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
       <c r="AF44" s="10">
+        <v>1199960</v>
+      </c>
+    </row>
+    <row r="45" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="10">
         <v>600000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A45" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B45" s="10">
-        <v>317648</v>
       </c>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
@@ -2741,14 +2744,14 @@
       <c r="M45" s="8"/>
       <c r="N45" s="8"/>
       <c r="O45" s="8">
-        <v>127059</v>
-      </c>
-      <c r="P45" s="8">
-        <v>127059</v>
-      </c>
-      <c r="Q45" s="8"/>
+        <v>240000</v>
+      </c>
+      <c r="P45" s="8"/>
+      <c r="Q45" s="8">
+        <v>180000</v>
+      </c>
       <c r="R45" s="8">
-        <v>63530</v>
+        <v>180000</v>
       </c>
       <c r="S45" s="8"/>
       <c r="T45" s="8"/>
@@ -2764,15 +2767,15 @@
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
       <c r="AF45" s="10">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="10">
         <v>317648</v>
-      </c>
-    </row>
-    <row r="46" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A46" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B46" s="10">
-        <v>832813</v>
       </c>
       <c r="C46" s="8"/>
       <c r="D46" s="8"/>
@@ -2786,23 +2789,23 @@
       <c r="L46" s="8"/>
       <c r="M46" s="8"/>
       <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
-      <c r="P46" s="8"/>
+      <c r="O46" s="8">
+        <v>127059</v>
+      </c>
+      <c r="P46" s="8">
+        <v>127059</v>
+      </c>
       <c r="Q46" s="8"/>
-      <c r="R46" s="8"/>
+      <c r="R46" s="8">
+        <v>63530</v>
+      </c>
       <c r="S46" s="8"/>
-      <c r="T46" s="8">
-        <v>333125</v>
-      </c>
-      <c r="U46" s="8">
-        <v>249844</v>
-      </c>
+      <c r="T46" s="8"/>
+      <c r="U46" s="8"/>
       <c r="V46" s="8"/>
       <c r="W46" s="8"/>
       <c r="X46" s="8"/>
-      <c r="Y46" s="8">
-        <v>249844</v>
-      </c>
+      <c r="Y46" s="8"/>
       <c r="Z46" s="8"/>
       <c r="AA46" s="8"/>
       <c r="AB46" s="8"/>
@@ -2810,22 +2813,18 @@
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
       <c r="AF46" s="10">
+        <v>317648</v>
+      </c>
+    </row>
+    <row r="47" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="10">
         <v>832813</v>
       </c>
-    </row>
-    <row r="47" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A47" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B47" s="10">
-        <v>341237</v>
-      </c>
-      <c r="C47" s="8">
-        <v>136495</v>
-      </c>
-      <c r="D47" s="8">
-        <v>136495</v>
-      </c>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
       <c r="E47" s="8"/>
       <c r="F47" s="8"/>
       <c r="G47" s="8"/>
@@ -2841,14 +2840,18 @@
       <c r="Q47" s="8"/>
       <c r="R47" s="8"/>
       <c r="S47" s="8"/>
-      <c r="T47" s="8"/>
-      <c r="U47" s="8"/>
-      <c r="V47" s="8">
-        <v>68247</v>
-      </c>
+      <c r="T47" s="8">
+        <v>333125</v>
+      </c>
+      <c r="U47" s="8">
+        <v>249844</v>
+      </c>
+      <c r="V47" s="8"/>
       <c r="W47" s="8"/>
       <c r="X47" s="8"/>
-      <c r="Y47" s="8"/>
+      <c r="Y47" s="8">
+        <v>249844</v>
+      </c>
       <c r="Z47" s="8"/>
       <c r="AA47" s="8"/>
       <c r="AB47" s="8"/>
@@ -2856,21 +2859,21 @@
       <c r="AD47" s="8"/>
       <c r="AE47" s="8"/>
       <c r="AF47" s="10">
+        <v>832813</v>
+      </c>
+    </row>
+    <row r="48" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A48" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="10">
         <v>341237</v>
       </c>
-    </row>
-    <row r="48" spans="1:32" ht="69" x14ac:dyDescent="0.25">
-      <c r="A48" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="B48" s="10">
-        <v>666700</v>
-      </c>
       <c r="C48" s="8">
-        <v>266680</v>
+        <v>136495</v>
       </c>
       <c r="D48" s="8">
-        <v>266680</v>
+        <v>136495</v>
       </c>
       <c r="E48" s="8"/>
       <c r="F48" s="8"/>
@@ -2889,10 +2892,10 @@
       <c r="S48" s="8"/>
       <c r="T48" s="8"/>
       <c r="U48" s="8"/>
-      <c r="V48" s="8"/>
-      <c r="W48" s="8">
-        <v>133340</v>
-      </c>
+      <c r="V48" s="8">
+        <v>68247</v>
+      </c>
+      <c r="W48" s="8"/>
       <c r="X48" s="8"/>
       <c r="Y48" s="8"/>
       <c r="Z48" s="8"/>
@@ -2902,18 +2905,22 @@
       <c r="AD48" s="8"/>
       <c r="AE48" s="8"/>
       <c r="AF48" s="10">
+        <v>341237</v>
+      </c>
+    </row>
+    <row r="49" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+      <c r="A49" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="10">
         <v>666700</v>
       </c>
-    </row>
-    <row r="49" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A49" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="B49" s="10">
-        <v>460000</v>
-      </c>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
+      <c r="C49" s="8">
+        <v>266680</v>
+      </c>
+      <c r="D49" s="8">
+        <v>266680</v>
+      </c>
       <c r="E49" s="8"/>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
@@ -2929,13 +2936,11 @@
       <c r="Q49" s="8"/>
       <c r="R49" s="8"/>
       <c r="S49" s="8"/>
-      <c r="T49" s="8">
-        <v>184000</v>
-      </c>
+      <c r="T49" s="8"/>
       <c r="U49" s="8"/>
       <c r="V49" s="8"/>
       <c r="W49" s="8">
-        <v>184000</v>
+        <v>133340</v>
       </c>
       <c r="X49" s="8"/>
       <c r="Y49" s="8"/>
@@ -2944,19 +2949,17 @@
       <c r="AB49" s="8"/>
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
-      <c r="AE49" s="8">
-        <v>92000</v>
-      </c>
+      <c r="AE49" s="8"/>
       <c r="AF49" s="10">
-        <v>460000</v>
+        <v>666700</v>
       </c>
     </row>
     <row r="50" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B50" s="10">
-        <v>206880</v>
+        <v>460000</v>
       </c>
       <c r="C50" s="8"/>
       <c r="D50" s="8"/>
@@ -2976,13 +2979,13 @@
       <c r="R50" s="8"/>
       <c r="S50" s="8"/>
       <c r="T50" s="8">
-        <v>82752</v>
-      </c>
-      <c r="U50" s="8">
-        <v>124128</v>
-      </c>
+        <v>184000</v>
+      </c>
+      <c r="U50" s="8"/>
       <c r="V50" s="8"/>
-      <c r="W50" s="8"/>
+      <c r="W50" s="8">
+        <v>184000</v>
+      </c>
       <c r="X50" s="8"/>
       <c r="Y50" s="8"/>
       <c r="Z50" s="8"/>
@@ -2990,17 +2993,19 @@
       <c r="AB50" s="8"/>
       <c r="AC50" s="8"/>
       <c r="AD50" s="8"/>
-      <c r="AE50" s="8"/>
+      <c r="AE50" s="8">
+        <v>92000</v>
+      </c>
       <c r="AF50" s="10">
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+      <c r="A51" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="10">
         <v>206880</v>
-      </c>
-    </row>
-    <row r="51" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A51" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B51" s="10">
-        <v>799875</v>
       </c>
       <c r="C51" s="8"/>
       <c r="D51" s="8"/>
@@ -3019,34 +3024,32 @@
       <c r="Q51" s="8"/>
       <c r="R51" s="8"/>
       <c r="S51" s="8"/>
-      <c r="T51" s="8"/>
+      <c r="T51" s="8">
+        <v>82752</v>
+      </c>
       <c r="U51" s="8">
-        <v>319950</v>
+        <v>124128</v>
       </c>
       <c r="V51" s="8"/>
       <c r="W51" s="8"/>
-      <c r="X51" s="8">
-        <v>319950</v>
-      </c>
+      <c r="X51" s="8"/>
       <c r="Y51" s="8"/>
       <c r="Z51" s="8"/>
       <c r="AA51" s="8"/>
-      <c r="AB51" s="8">
-        <v>159975</v>
-      </c>
+      <c r="AB51" s="8"/>
       <c r="AC51" s="8"/>
       <c r="AD51" s="8"/>
       <c r="AE51" s="8"/>
       <c r="AF51" s="10">
-        <v>799875</v>
+        <v>206880</v>
       </c>
     </row>
     <row r="52" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B52" s="10">
-        <v>411073</v>
+        <v>799875</v>
       </c>
       <c r="C52" s="8"/>
       <c r="D52" s="8"/>
@@ -3066,31 +3069,33 @@
       <c r="R52" s="8"/>
       <c r="S52" s="8"/>
       <c r="T52" s="8"/>
-      <c r="U52" s="8"/>
-      <c r="V52" s="8">
-        <v>164429</v>
-      </c>
-      <c r="W52" s="8">
-        <v>246644</v>
-      </c>
-      <c r="X52" s="8"/>
+      <c r="U52" s="8">
+        <v>319950</v>
+      </c>
+      <c r="V52" s="8"/>
+      <c r="W52" s="8"/>
+      <c r="X52" s="8">
+        <v>319950</v>
+      </c>
       <c r="Y52" s="8"/>
       <c r="Z52" s="8"/>
       <c r="AA52" s="8"/>
-      <c r="AB52" s="8"/>
+      <c r="AB52" s="8">
+        <v>159975</v>
+      </c>
       <c r="AC52" s="8"/>
       <c r="AD52" s="8"/>
       <c r="AE52" s="8"/>
       <c r="AF52" s="10">
+        <v>799875</v>
+      </c>
+    </row>
+    <row r="53" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A53" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="10">
         <v>411073</v>
-      </c>
-    </row>
-    <row r="53" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
-      <c r="A53" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B53" s="10">
-        <v>90000</v>
       </c>
       <c r="C53" s="8"/>
       <c r="D53" s="8"/>
@@ -3111,13 +3116,13 @@
       <c r="S53" s="8"/>
       <c r="T53" s="8"/>
       <c r="U53" s="8"/>
-      <c r="V53" s="8"/>
+      <c r="V53" s="8">
+        <v>164429</v>
+      </c>
       <c r="W53" s="8">
-        <v>60000</v>
-      </c>
-      <c r="X53" s="8">
-        <v>30000</v>
-      </c>
+        <v>246644</v>
+      </c>
+      <c r="X53" s="8"/>
       <c r="Y53" s="8"/>
       <c r="Z53" s="8"/>
       <c r="AA53" s="8"/>
@@ -3126,150 +3131,238 @@
       <c r="AD53" s="8"/>
       <c r="AE53" s="8"/>
       <c r="AF53" s="10">
+        <v>411073</v>
+      </c>
+    </row>
+    <row r="54" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A54" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="10">
         <v>90000</v>
       </c>
-    </row>
-    <row r="54" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="11" t="s">
+      <c r="C54" s="8"/>
+      <c r="D54" s="8"/>
+      <c r="E54" s="8"/>
+      <c r="F54" s="8"/>
+      <c r="G54" s="8"/>
+      <c r="H54" s="8"/>
+      <c r="I54" s="8"/>
+      <c r="J54" s="8"/>
+      <c r="K54" s="8"/>
+      <c r="L54" s="8"/>
+      <c r="M54" s="8"/>
+      <c r="N54" s="8"/>
+      <c r="O54" s="8"/>
+      <c r="P54" s="8"/>
+      <c r="Q54" s="8"/>
+      <c r="R54" s="8"/>
+      <c r="S54" s="8"/>
+      <c r="T54" s="8"/>
+      <c r="U54" s="8"/>
+      <c r="V54" s="8"/>
+      <c r="W54" s="8">
+        <v>60000</v>
+      </c>
+      <c r="X54" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Y54" s="8"/>
+      <c r="Z54" s="8"/>
+      <c r="AA54" s="8"/>
+      <c r="AB54" s="8"/>
+      <c r="AC54" s="8"/>
+      <c r="AD54" s="8"/>
+      <c r="AE54" s="8"/>
+      <c r="AF54" s="10">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="55" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A55" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="12">
-        <v>11995865</v>
-      </c>
-      <c r="C54" s="12">
+      <c r="B55" s="10">
+        <v>90000</v>
+      </c>
+      <c r="C55" s="8"/>
+      <c r="D55" s="8"/>
+      <c r="E55" s="8"/>
+      <c r="F55" s="8"/>
+      <c r="G55" s="8"/>
+      <c r="H55" s="8"/>
+      <c r="I55" s="8"/>
+      <c r="J55" s="8"/>
+      <c r="K55" s="8"/>
+      <c r="L55" s="8"/>
+      <c r="M55" s="8"/>
+      <c r="N55" s="8"/>
+      <c r="O55" s="8"/>
+      <c r="P55" s="8"/>
+      <c r="Q55" s="8"/>
+      <c r="R55" s="8"/>
+      <c r="S55" s="8"/>
+      <c r="T55" s="8"/>
+      <c r="U55" s="8"/>
+      <c r="V55" s="8"/>
+      <c r="W55" s="8">
+        <v>60000</v>
+      </c>
+      <c r="X55" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Y55" s="8"/>
+      <c r="Z55" s="8"/>
+      <c r="AA55" s="8"/>
+      <c r="AB55" s="8"/>
+      <c r="AC55" s="8"/>
+      <c r="AD55" s="8"/>
+      <c r="AE55" s="8"/>
+      <c r="AF55" s="10">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="56" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="12">
+        <v>12085865</v>
+      </c>
+      <c r="C56" s="12">
         <v>403175</v>
       </c>
-      <c r="D54" s="12">
+      <c r="D56" s="12">
         <v>403175</v>
       </c>
-      <c r="E54" s="12">
+      <c r="E56" s="12">
         <v>0</v>
       </c>
-      <c r="F54" s="12">
+      <c r="F56" s="12">
         <v>0</v>
       </c>
-      <c r="G54" s="12">
+      <c r="G56" s="12">
         <v>0</v>
       </c>
-      <c r="H54" s="12">
+      <c r="H56" s="12">
         <v>0</v>
       </c>
-      <c r="I54" s="12">
+      <c r="I56" s="12">
         <v>0</v>
       </c>
-      <c r="J54" s="12">
+      <c r="J56" s="12">
         <v>0</v>
       </c>
-      <c r="K54" s="12">
+      <c r="K56" s="12">
         <v>0</v>
       </c>
-      <c r="L54" s="12">
+      <c r="L56" s="12">
         <v>0</v>
       </c>
-      <c r="M54" s="12">
+      <c r="M56" s="12">
         <v>0</v>
       </c>
-      <c r="N54" s="12">
+      <c r="N56" s="12">
         <v>0</v>
       </c>
-      <c r="O54" s="12">
+      <c r="O56" s="12">
         <v>728301</v>
       </c>
-      <c r="P54" s="12">
+      <c r="P56" s="12">
         <v>521426</v>
       </c>
-      <c r="Q54" s="12">
+      <c r="Q56" s="12">
         <v>180000</v>
       </c>
-      <c r="R54" s="12">
+      <c r="R56" s="12">
         <v>1139167</v>
       </c>
-      <c r="S54" s="12">
+      <c r="S56" s="12">
         <v>1539976</v>
       </c>
-      <c r="T54" s="12">
+      <c r="T56" s="12">
         <v>1943215</v>
       </c>
-      <c r="U54" s="12">
+      <c r="U56" s="12">
         <v>1035340</v>
       </c>
-      <c r="V54" s="12">
+      <c r="V56" s="12">
         <v>265355</v>
       </c>
-      <c r="W54" s="12">
-        <v>1751270</v>
-      </c>
-      <c r="X54" s="12">
-        <v>349950</v>
-      </c>
-      <c r="Y54" s="12">
+      <c r="W56" s="12">
+        <v>1811270</v>
+      </c>
+      <c r="X56" s="12">
+        <v>379950</v>
+      </c>
+      <c r="Y56" s="12">
         <v>821658</v>
       </c>
-      <c r="Z54" s="12">
+      <c r="Z56" s="12">
         <v>477638</v>
       </c>
-      <c r="AA54" s="12">
+      <c r="AA56" s="12">
         <v>184244</v>
       </c>
-      <c r="AB54" s="12">
+      <c r="AB56" s="12">
         <v>159975</v>
       </c>
-      <c r="AC54" s="12">
+      <c r="AC56" s="12">
         <v>0</v>
       </c>
-      <c r="AD54" s="12">
+      <c r="AD56" s="12">
         <v>0</v>
       </c>
-      <c r="AE54" s="12">
+      <c r="AE56" s="12">
         <v>92000</v>
       </c>
-      <c r="AF54" s="12">
-        <v>11995865</v>
-      </c>
-    </row>
-    <row r="56" spans="1:32" x14ac:dyDescent="0.2">
-      <c r="A56" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B56" s="4"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
-      <c r="I56" s="4"/>
-      <c r="J56" s="4"/>
-      <c r="K56" s="4"/>
-      <c r="L56" s="4"/>
-      <c r="M56" s="4"/>
-      <c r="N56" s="4"/>
-      <c r="O56" s="4"/>
-      <c r="P56" s="4"/>
-      <c r="Q56" s="4"/>
-      <c r="R56" s="4"/>
-      <c r="S56" s="4"/>
-      <c r="T56" s="4"/>
-      <c r="U56" s="4"/>
-      <c r="V56" s="4"/>
-      <c r="W56" s="4"/>
-      <c r="X56" s="4"/>
-      <c r="Y56" s="4"/>
-      <c r="Z56" s="4"/>
-      <c r="AA56" s="4"/>
-      <c r="AB56" s="4"/>
-      <c r="AC56" s="4"/>
-      <c r="AD56" s="4"/>
-      <c r="AE56" s="4"/>
-      <c r="AF56" s="4"/>
+      <c r="AF56" s="12">
+        <v>12085865</v>
+      </c>
+    </row>
+    <row r="58" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="A58" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+      <c r="F58" s="4"/>
+      <c r="G58" s="4"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
+      <c r="O58" s="4"/>
+      <c r="P58" s="4"/>
+      <c r="Q58" s="4"/>
+      <c r="R58" s="4"/>
+      <c r="S58" s="4"/>
+      <c r="T58" s="4"/>
+      <c r="U58" s="4"/>
+      <c r="V58" s="4"/>
+      <c r="W58" s="4"/>
+      <c r="X58" s="4"/>
+      <c r="Y58" s="4"/>
+      <c r="Z58" s="4"/>
+      <c r="AA58" s="4"/>
+      <c r="AB58" s="4"/>
+      <c r="AC58" s="4"/>
+      <c r="AD58" s="4"/>
+      <c r="AE58" s="4"/>
+      <c r="AF58" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="A2:AF2"/>
-    <mergeCell ref="A56:AF56"/>
+    <mergeCell ref="A58:AF58"/>
     <mergeCell ref="A4:AF4"/>
-    <mergeCell ref="A30:AF30"/>
+    <mergeCell ref="A31:AF31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 13:55)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF742029-345F-4299-BC39-DFC41076DE62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B3ACCBB-F293-4DAE-B497-748E77D41442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7272" yWindow="696" windowWidth="13572" windowHeight="10368" xr2:uid="{4305E47D-3950-4BDC-B968-2DDF74415905}"/>
+    <workbookView xWindow="7272" yWindow="696" windowWidth="13572" windowHeight="10368" xr2:uid="{BC829408-18FD-40FC-9571-733223359C7C}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EBA1058-08C8-4174-AD23-659D8FB8F588}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91BFB2B0-1D1E-42AC-A794-CD79205E15D5}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 16:32)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0B3ACCBB-F293-4DAE-B497-748E77D41442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B6A10BC-ED9B-451F-836F-A92585822C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7272" yWindow="696" windowWidth="13572" windowHeight="10368" xr2:uid="{BC829408-18FD-40FC-9571-733223359C7C}"/>
+    <workbookView xWindow="7272" yWindow="696" windowWidth="13572" windowHeight="10368" xr2:uid="{738EDDE8-E90A-43B1-ADD7-0F8517380CB5}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91BFB2B0-1D1E-42AC-A794-CD79205E15D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{261FAD62-26ED-4E17-AFFC-09BECB5A3197}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 16:38)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B6A10BC-ED9B-451F-836F-A92585822C1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{949B6775-3830-41E6-B46C-4980D3DB8318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7272" yWindow="696" windowWidth="13572" windowHeight="10368" xr2:uid="{738EDDE8-E90A-43B1-ADD7-0F8517380CB5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2E754B2D-6C9D-439E-986C-58D8FC007F13}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{261FAD62-26ED-4E17-AFFC-09BECB5A3197}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B041C4-1C9A-4B04-89B2-18AF300E7556}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 16:40)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{949B6775-3830-41E6-B46C-4980D3DB8318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{04E3AC31-8ABF-46E2-9E66-524F096981FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2E754B2D-6C9D-439E-986C-58D8FC007F13}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{832C3F62-903A-4851-ADE7-C9D9BFE808F0}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B041C4-1C9A-4B04-89B2-18AF300E7556}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B082FC-14C8-45A6-87B7-43D177A76C8F}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 16:52)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04E3AC31-8ABF-46E2-9E66-524F096981FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D78F5FB9-39B3-4725-90E3-138B8D0B5DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{832C3F62-903A-4851-ADE7-C9D9BFE808F0}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{187F46F4-04D3-40BF-A117-DC06D819461D}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50B082FC-14C8-45A6-87B7-43D177A76C8F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63BCD2C9-7B31-4DAF-9369-BD4D42FEB561}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 17:35)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D78F5FB9-39B3-4725-90E3-138B8D0B5DC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C01FA834-E75A-4A39-901E-96C5A7DF9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{187F46F4-04D3-40BF-A117-DC06D819461D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D9228B90-8ACF-4135-9E32-D5CB12BE0014}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63BCD2C9-7B31-4DAF-9369-BD4D42FEB561}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB2FA042-65DA-415F-9DE8-ACE38D7A56F7}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-14 17:41)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C01FA834-E75A-4A39-901E-96C5A7DF9580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BB4A49D-8F73-4B87-B6E1-55F00B611587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D9228B90-8ACF-4135-9E32-D5CB12BE0014}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D078D6B2-8AA1-4BD7-83D7-0B60219C5757}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB2FA042-65DA-415F-9DE8-ACE38D7A56F7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6B763A-8927-4689-A722-719ABCC26871}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-15 09:37)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6BB4A49D-8F73-4B87-B6E1-55F00B611587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{53841B5D-97C2-424A-97D3-F7518703D667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D078D6B2-8AA1-4BD7-83D7-0B60219C5757}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{380C0B49-9853-4CCD-ACCC-3778BBB5FE19}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (23 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-14</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-15</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6B763A-8927-4689-A722-719ABCC26871}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9978274E-595B-4A00-9F61-EE028B6CBA04}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-15 15:58)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53841B5D-97C2-424A-97D3-F7518703D667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EECE9FF-D23B-4570-BE3C-5B9B459D85DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{380C0B49-9853-4CCD-ACCC-3778BBB5FE19}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D16B0D97-A246-475F-9FE3-A6CDDF5B5A83}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9978274E-595B-4A00-9F61-EE028B6CBA04}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5F50D57-9272-4D8D-B29C-EDBC2CD21C69}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-17 16:02)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EECE9FF-D23B-4570-BE3C-5B9B459D85DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1EDC067-C983-4D1D-9FA2-36E0613C0A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D16B0D97-A246-475F-9FE3-A6CDDF5B5A83}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9727E46D-0CA8-41F7-8BCF-52D4A5D525E6}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (23 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-15</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-17</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5F50D57-9272-4D8D-B29C-EDBC2CD21C69}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F808D685-2184-437C-A288-0B5134603F75}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-22 11:34)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1EDC067-C983-4D1D-9FA2-36E0613C0A5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{309BEEA1-7877-4F2D-AF5B-E71DF9AD1BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9727E46D-0CA8-41F7-8BCF-52D4A5D525E6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FE24A543-CB5B-4C15-8000-CCA0C8CC6A28}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (23 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-17</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-22</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -703,7 +703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F808D685-2184-437C-A288-0B5134603F75}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96BC8503-E70F-459A-BC09-49468BBB623E}">
   <dimension ref="A1:AF58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1907,7 +1907,7 @@
         <v>57</v>
       </c>
       <c r="B28" s="10">
-        <v>164242</v>
+        <v>158800</v>
       </c>
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
@@ -1929,10 +1929,10 @@
       <c r="T28" s="8"/>
       <c r="U28" s="8"/>
       <c r="V28" s="8">
-        <v>50341</v>
+        <v>48300</v>
       </c>
       <c r="W28" s="8">
-        <v>83901</v>
+        <v>80500</v>
       </c>
       <c r="X28" s="8">
         <v>30000</v>
@@ -1945,7 +1945,7 @@
       <c r="AD28" s="8"/>
       <c r="AE28" s="8"/>
       <c r="AF28" s="10">
-        <v>164242</v>
+        <v>158800</v>
       </c>
     </row>
     <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -1953,7 +1953,7 @@
         <v>58</v>
       </c>
       <c r="B29" s="12">
-        <v>4832025</v>
+        <v>4826583</v>
       </c>
       <c r="C29" s="12">
         <v>139012</v>
@@ -2013,10 +2013,10 @@
         <v>327000</v>
       </c>
       <c r="V29" s="12">
-        <v>459420</v>
+        <v>457379</v>
       </c>
       <c r="W29" s="12">
-        <v>928615</v>
+        <v>925214</v>
       </c>
       <c r="X29" s="12">
         <v>326922</v>
@@ -2043,7 +2043,7 @@
         <v>0</v>
       </c>
       <c r="AF29" s="12">
-        <v>4832025</v>
+        <v>4826583</v>
       </c>
     </row>
     <row r="31" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-22 13:51)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{309BEEA1-7877-4F2D-AF5B-E71DF9AD1BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{476E8975-DB6D-4506-9C3F-08F6BD2934B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FE24A543-CB5B-4C15-8000-CCA0C8CC6A28}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E776A27-F0C1-47BA-9ABF-E64A2435029D}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="66">
   <si>
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (23 โครงการ PO)</t>
   </si>
@@ -141,6 +141,21 @@
   </si>
   <si>
     <t>Jun-27</t>
+  </si>
+  <si>
+    <t>Jul-27</t>
+  </si>
+  <si>
+    <t>Aug-27</t>
+  </si>
+  <si>
+    <t>Sep-27</t>
+  </si>
+  <si>
+    <t>Oct-27</t>
+  </si>
+  <si>
+    <t>Nov-27</t>
   </si>
   <si>
     <t>รวม (฿)</t>
@@ -703,18 +718,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96BC8503-E70F-459A-BC09-49468BBB623E}">
-  <dimension ref="A1:AF58"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94B8C11F-44F2-4F2C-8642-5BB90466B6E4}">
+  <dimension ref="A1:AK58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
     <col min="2" max="2" width="15" style="1" customWidth="1"/>
-    <col min="3" max="31" width="11" style="1" customWidth="1"/>
-    <col min="32" max="32" width="15" style="1" customWidth="1"/>
-    <col min="33" max="16384" width="8.88671875" style="1"/>
+    <col min="3" max="36" width="11" style="1" customWidth="1"/>
+    <col min="37" max="37" width="15" style="1" customWidth="1"/>
+    <col min="38" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:37" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -749,8 +764,13 @@
       <c r="AD1" s="2"/>
       <c r="AE1" s="2"/>
       <c r="AF1" s="2"/>
-    </row>
-    <row r="2" spans="1:32" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AG1" s="2"/>
+      <c r="AH1" s="2"/>
+      <c r="AI1" s="2"/>
+      <c r="AJ1" s="2"/>
+      <c r="AK1" s="2"/>
+    </row>
+    <row r="2" spans="1:37" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -785,8 +805,13 @@
       <c r="AD2" s="3"/>
       <c r="AE2" s="3"/>
       <c r="AF2" s="3"/>
-    </row>
-    <row r="4" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AG2" s="3"/>
+      <c r="AH2" s="3"/>
+      <c r="AI2" s="3"/>
+      <c r="AJ2" s="3"/>
+      <c r="AK2" s="3"/>
+    </row>
+    <row r="4" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
@@ -821,8 +846,13 @@
       <c r="AD4" s="5"/>
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
-    </row>
-    <row r="5" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AG4" s="5"/>
+      <c r="AH4" s="5"/>
+      <c r="AI4" s="5"/>
+      <c r="AJ4" s="5"/>
+      <c r="AK4" s="5"/>
+    </row>
+    <row r="5" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
@@ -916,13 +946,28 @@
       <c r="AE5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF5" s="6" t="s">
+      <c r="AF5" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AG5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AH5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AI5" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ5" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK5" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B6" s="10">
         <v>130000</v>
@@ -962,13 +1007,18 @@
       <c r="AC6" s="8"/>
       <c r="AD6" s="8"/>
       <c r="AE6" s="8"/>
-      <c r="AF6" s="10">
+      <c r="AF6" s="8"/>
+      <c r="AG6" s="8"/>
+      <c r="AH6" s="8"/>
+      <c r="AI6" s="8"/>
+      <c r="AJ6" s="8"/>
+      <c r="AK6" s="10">
         <v>130000</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B7" s="10">
         <v>139446</v>
@@ -1008,13 +1058,18 @@
       <c r="AC7" s="8"/>
       <c r="AD7" s="8"/>
       <c r="AE7" s="8"/>
-      <c r="AF7" s="10">
+      <c r="AF7" s="8"/>
+      <c r="AG7" s="8"/>
+      <c r="AH7" s="8"/>
+      <c r="AI7" s="8"/>
+      <c r="AJ7" s="8"/>
+      <c r="AK7" s="10">
         <v>139446</v>
       </c>
     </row>
-    <row r="8" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B8" s="10">
         <v>280000</v>
@@ -1054,13 +1109,18 @@
       <c r="AC8" s="8"/>
       <c r="AD8" s="8"/>
       <c r="AE8" s="8"/>
-      <c r="AF8" s="10">
+      <c r="AF8" s="8"/>
+      <c r="AG8" s="8"/>
+      <c r="AH8" s="8"/>
+      <c r="AI8" s="8"/>
+      <c r="AJ8" s="8"/>
+      <c r="AK8" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="9" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B9" s="10">
         <v>89000</v>
@@ -1098,13 +1158,18 @@
       <c r="AC9" s="8"/>
       <c r="AD9" s="8"/>
       <c r="AE9" s="8"/>
-      <c r="AF9" s="10">
+      <c r="AF9" s="8"/>
+      <c r="AG9" s="8"/>
+      <c r="AH9" s="8"/>
+      <c r="AI9" s="8"/>
+      <c r="AJ9" s="8"/>
+      <c r="AK9" s="10">
         <v>89000</v>
       </c>
     </row>
-    <row r="10" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B10" s="10">
         <v>0</v>
@@ -1138,13 +1203,18 @@
       <c r="AC10" s="8"/>
       <c r="AD10" s="8"/>
       <c r="AE10" s="8"/>
-      <c r="AF10" s="10">
+      <c r="AF10" s="8"/>
+      <c r="AG10" s="8"/>
+      <c r="AH10" s="8"/>
+      <c r="AI10" s="8"/>
+      <c r="AJ10" s="8"/>
+      <c r="AK10" s="10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B11" s="10">
         <v>138000</v>
@@ -1182,13 +1252,18 @@
       <c r="AC11" s="8"/>
       <c r="AD11" s="8"/>
       <c r="AE11" s="8"/>
-      <c r="AF11" s="10">
+      <c r="AF11" s="8"/>
+      <c r="AG11" s="8"/>
+      <c r="AH11" s="8"/>
+      <c r="AI11" s="8"/>
+      <c r="AJ11" s="8"/>
+      <c r="AK11" s="10">
         <v>138000</v>
       </c>
     </row>
-    <row r="12" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B12" s="10">
         <v>280000</v>
@@ -1228,13 +1303,18 @@
       <c r="AC12" s="8"/>
       <c r="AD12" s="8"/>
       <c r="AE12" s="8"/>
-      <c r="AF12" s="10">
+      <c r="AF12" s="8"/>
+      <c r="AG12" s="8"/>
+      <c r="AH12" s="8"/>
+      <c r="AI12" s="8"/>
+      <c r="AJ12" s="8"/>
+      <c r="AK12" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="13" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B13" s="10">
         <v>233248</v>
@@ -1272,13 +1352,18 @@
       <c r="AC13" s="8"/>
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
-      <c r="AF13" s="10">
+      <c r="AF13" s="8"/>
+      <c r="AG13" s="8"/>
+      <c r="AH13" s="8"/>
+      <c r="AI13" s="8"/>
+      <c r="AJ13" s="8"/>
+      <c r="AK13" s="10">
         <v>233248</v>
       </c>
     </row>
-    <row r="14" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B14" s="10">
         <v>120000</v>
@@ -1318,13 +1403,18 @@
       <c r="AC14" s="8"/>
       <c r="AD14" s="8"/>
       <c r="AE14" s="8"/>
-      <c r="AF14" s="10">
+      <c r="AF14" s="8"/>
+      <c r="AG14" s="8"/>
+      <c r="AH14" s="8"/>
+      <c r="AI14" s="8"/>
+      <c r="AJ14" s="8"/>
+      <c r="AK14" s="10">
         <v>120000</v>
       </c>
     </row>
-    <row r="15" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B15" s="10">
         <v>656680</v>
@@ -1362,13 +1452,18 @@
       <c r="AC15" s="8"/>
       <c r="AD15" s="8"/>
       <c r="AE15" s="8"/>
-      <c r="AF15" s="10">
+      <c r="AF15" s="8"/>
+      <c r="AG15" s="8"/>
+      <c r="AH15" s="8"/>
+      <c r="AI15" s="8"/>
+      <c r="AJ15" s="8"/>
+      <c r="AK15" s="10">
         <v>656680</v>
       </c>
     </row>
-    <row r="16" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B16" s="10">
         <v>40000</v>
@@ -1404,13 +1499,18 @@
       <c r="AC16" s="8"/>
       <c r="AD16" s="8"/>
       <c r="AE16" s="8"/>
-      <c r="AF16" s="10">
+      <c r="AF16" s="8"/>
+      <c r="AG16" s="8"/>
+      <c r="AH16" s="8"/>
+      <c r="AI16" s="8"/>
+      <c r="AJ16" s="8"/>
+      <c r="AK16" s="10">
         <v>40000</v>
       </c>
     </row>
-    <row r="17" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B17" s="10">
         <v>430000</v>
@@ -1450,13 +1550,18 @@
       <c r="AC17" s="8"/>
       <c r="AD17" s="8"/>
       <c r="AE17" s="8"/>
-      <c r="AF17" s="10">
+      <c r="AF17" s="8"/>
+      <c r="AG17" s="8"/>
+      <c r="AH17" s="8"/>
+      <c r="AI17" s="8"/>
+      <c r="AJ17" s="8"/>
+      <c r="AK17" s="10">
         <v>430000</v>
       </c>
     </row>
-    <row r="18" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B18" s="10">
         <v>234860</v>
@@ -1494,13 +1599,18 @@
       <c r="AC18" s="8"/>
       <c r="AD18" s="8"/>
       <c r="AE18" s="8"/>
-      <c r="AF18" s="10">
+      <c r="AF18" s="8"/>
+      <c r="AG18" s="8"/>
+      <c r="AH18" s="8"/>
+      <c r="AI18" s="8"/>
+      <c r="AJ18" s="8"/>
+      <c r="AK18" s="10">
         <v>234860</v>
       </c>
     </row>
-    <row r="19" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B19" s="10">
         <v>119980</v>
@@ -1538,13 +1648,18 @@
       <c r="AC19" s="8"/>
       <c r="AD19" s="8"/>
       <c r="AE19" s="8"/>
-      <c r="AF19" s="10">
+      <c r="AF19" s="8"/>
+      <c r="AG19" s="8"/>
+      <c r="AH19" s="8"/>
+      <c r="AI19" s="8"/>
+      <c r="AJ19" s="8"/>
+      <c r="AK19" s="10">
         <v>119980</v>
       </c>
     </row>
-    <row r="20" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B20" s="10">
         <v>280000</v>
@@ -1584,13 +1699,18 @@
       <c r="AC20" s="8"/>
       <c r="AD20" s="8"/>
       <c r="AE20" s="8"/>
-      <c r="AF20" s="10">
+      <c r="AF20" s="8"/>
+      <c r="AG20" s="8"/>
+      <c r="AH20" s="8"/>
+      <c r="AI20" s="8"/>
+      <c r="AJ20" s="8"/>
+      <c r="AK20" s="10">
         <v>280000</v>
       </c>
     </row>
-    <row r="21" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B21" s="10">
         <v>284858</v>
@@ -1630,13 +1750,18 @@
       <c r="AC21" s="8"/>
       <c r="AD21" s="8"/>
       <c r="AE21" s="8"/>
-      <c r="AF21" s="10">
+      <c r="AF21" s="8"/>
+      <c r="AG21" s="8"/>
+      <c r="AH21" s="8"/>
+      <c r="AI21" s="8"/>
+      <c r="AJ21" s="8"/>
+      <c r="AK21" s="10">
         <v>284858</v>
       </c>
     </row>
-    <row r="22" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B22" s="10">
         <v>246650</v>
@@ -1676,13 +1801,18 @@
       <c r="AC22" s="8"/>
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
-      <c r="AF22" s="10">
+      <c r="AF22" s="8"/>
+      <c r="AG22" s="8"/>
+      <c r="AH22" s="8"/>
+      <c r="AI22" s="8"/>
+      <c r="AJ22" s="8"/>
+      <c r="AK22" s="10">
         <v>246650</v>
       </c>
     </row>
-    <row r="23" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B23" s="10">
         <v>218000</v>
@@ -1722,13 +1852,18 @@
         <v>43600</v>
       </c>
       <c r="AE23" s="8"/>
-      <c r="AF23" s="10">
+      <c r="AF23" s="8"/>
+      <c r="AG23" s="8"/>
+      <c r="AH23" s="8"/>
+      <c r="AI23" s="8"/>
+      <c r="AJ23" s="8"/>
+      <c r="AK23" s="10">
         <v>218000</v>
       </c>
     </row>
-    <row r="24" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B24" s="10">
         <v>58000</v>
@@ -1764,13 +1899,18 @@
       <c r="AC24" s="8"/>
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
-      <c r="AF24" s="10">
+      <c r="AF24" s="8"/>
+      <c r="AG24" s="8"/>
+      <c r="AH24" s="8"/>
+      <c r="AI24" s="8"/>
+      <c r="AJ24" s="8"/>
+      <c r="AK24" s="10">
         <v>58000</v>
       </c>
     </row>
-    <row r="25" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B25" s="10">
         <v>341476</v>
@@ -1808,13 +1948,18 @@
       <c r="AC25" s="8"/>
       <c r="AD25" s="8"/>
       <c r="AE25" s="8"/>
-      <c r="AF25" s="10">
+      <c r="AF25" s="8"/>
+      <c r="AG25" s="8"/>
+      <c r="AH25" s="8"/>
+      <c r="AI25" s="8"/>
+      <c r="AJ25" s="8"/>
+      <c r="AK25" s="10">
         <v>341476</v>
       </c>
     </row>
-    <row r="26" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B26" s="10">
         <v>176436</v>
@@ -1852,13 +1997,18 @@
       <c r="AC26" s="8"/>
       <c r="AD26" s="8"/>
       <c r="AE26" s="8"/>
-      <c r="AF26" s="10">
+      <c r="AF26" s="8"/>
+      <c r="AG26" s="8"/>
+      <c r="AH26" s="8"/>
+      <c r="AI26" s="8"/>
+      <c r="AJ26" s="8"/>
+      <c r="AK26" s="10">
         <v>176436</v>
       </c>
     </row>
-    <row r="27" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B27" s="10">
         <v>171149</v>
@@ -1888,9 +2038,7 @@
       <c r="W27" s="8">
         <v>88218</v>
       </c>
-      <c r="X27" s="8">
-        <v>30000</v>
-      </c>
+      <c r="X27" s="8"/>
       <c r="Y27" s="8"/>
       <c r="Z27" s="8"/>
       <c r="AA27" s="8"/>
@@ -1898,13 +2046,20 @@
       <c r="AC27" s="8"/>
       <c r="AD27" s="8"/>
       <c r="AE27" s="8"/>
-      <c r="AF27" s="10">
+      <c r="AF27" s="8"/>
+      <c r="AG27" s="8"/>
+      <c r="AH27" s="8"/>
+      <c r="AI27" s="8"/>
+      <c r="AJ27" s="8">
+        <v>30000</v>
+      </c>
+      <c r="AK27" s="10">
         <v>171149</v>
       </c>
     </row>
-    <row r="28" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B28" s="10">
         <v>158800</v>
@@ -1944,13 +2099,18 @@
       <c r="AC28" s="8"/>
       <c r="AD28" s="8"/>
       <c r="AE28" s="8"/>
-      <c r="AF28" s="10">
+      <c r="AF28" s="8"/>
+      <c r="AG28" s="8"/>
+      <c r="AH28" s="8"/>
+      <c r="AI28" s="8"/>
+      <c r="AJ28" s="8"/>
+      <c r="AK28" s="10">
         <v>158800</v>
       </c>
     </row>
-    <row r="29" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B29" s="12">
         <v>4826583</v>
@@ -2019,7 +2179,7 @@
         <v>925214</v>
       </c>
       <c r="X29" s="12">
-        <v>326922</v>
+        <v>296922</v>
       </c>
       <c r="Y29" s="12">
         <v>155974</v>
@@ -2043,12 +2203,27 @@
         <v>0</v>
       </c>
       <c r="AF29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AI29" s="12">
+        <v>0</v>
+      </c>
+      <c r="AJ29" s="12">
+        <v>30000</v>
+      </c>
+      <c r="AK29" s="12">
         <v>4826583</v>
       </c>
     </row>
-    <row r="31" spans="1:32" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -2081,8 +2256,13 @@
       <c r="AD31" s="5"/>
       <c r="AE31" s="5"/>
       <c r="AF31" s="5"/>
-    </row>
-    <row r="32" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AG31" s="5"/>
+      <c r="AH31" s="5"/>
+      <c r="AI31" s="5"/>
+      <c r="AJ31" s="5"/>
+      <c r="AK31" s="5"/>
+    </row>
+    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>3</v>
       </c>
@@ -2176,13 +2356,28 @@
       <c r="AE32" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF32" s="6" t="s">
+      <c r="AF32" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="33" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="AG32" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="AH32" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AI32" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AJ32" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AK32" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B33" s="10">
         <v>294109</v>
@@ -2222,13 +2417,18 @@
       <c r="AC33" s="8"/>
       <c r="AD33" s="8"/>
       <c r="AE33" s="8"/>
-      <c r="AF33" s="10">
+      <c r="AF33" s="8"/>
+      <c r="AG33" s="8"/>
+      <c r="AH33" s="8"/>
+      <c r="AI33" s="8"/>
+      <c r="AJ33" s="8"/>
+      <c r="AK33" s="10">
         <v>294109</v>
       </c>
     </row>
-    <row r="34" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B34" s="10">
         <v>409600</v>
@@ -2268,13 +2468,18 @@
       <c r="AC34" s="8"/>
       <c r="AD34" s="8"/>
       <c r="AE34" s="8"/>
-      <c r="AF34" s="10">
+      <c r="AF34" s="8"/>
+      <c r="AG34" s="8"/>
+      <c r="AH34" s="8"/>
+      <c r="AI34" s="8"/>
+      <c r="AJ34" s="8"/>
+      <c r="AK34" s="10">
         <v>409600</v>
       </c>
     </row>
-    <row r="35" spans="1:32" ht="80.400000000000006" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="B35" s="10">
         <v>576318</v>
@@ -2314,13 +2519,18 @@
       <c r="AC35" s="8"/>
       <c r="AD35" s="8"/>
       <c r="AE35" s="8"/>
-      <c r="AF35" s="10">
+      <c r="AF35" s="8"/>
+      <c r="AG35" s="8"/>
+      <c r="AH35" s="8"/>
+      <c r="AI35" s="8"/>
+      <c r="AJ35" s="8"/>
+      <c r="AK35" s="10">
         <v>576318</v>
       </c>
     </row>
-    <row r="36" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="B36" s="10">
         <v>322960</v>
@@ -2358,13 +2568,18 @@
       <c r="AC36" s="8"/>
       <c r="AD36" s="8"/>
       <c r="AE36" s="8"/>
-      <c r="AF36" s="10">
+      <c r="AF36" s="8"/>
+      <c r="AG36" s="8"/>
+      <c r="AH36" s="8"/>
+      <c r="AI36" s="8"/>
+      <c r="AJ36" s="8"/>
+      <c r="AK36" s="10">
         <v>322960</v>
       </c>
     </row>
-    <row r="37" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B37" s="10">
         <v>252248</v>
@@ -2400,13 +2615,18 @@
       <c r="AC37" s="8"/>
       <c r="AD37" s="8"/>
       <c r="AE37" s="8"/>
-      <c r="AF37" s="10">
+      <c r="AF37" s="8"/>
+      <c r="AG37" s="8"/>
+      <c r="AH37" s="8"/>
+      <c r="AI37" s="8"/>
+      <c r="AJ37" s="8"/>
+      <c r="AK37" s="10">
         <v>252248</v>
       </c>
     </row>
-    <row r="38" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="B38" s="10">
         <v>338450</v>
@@ -2446,13 +2666,18 @@
       <c r="AC38" s="8"/>
       <c r="AD38" s="8"/>
       <c r="AE38" s="8"/>
-      <c r="AF38" s="10">
+      <c r="AF38" s="8"/>
+      <c r="AG38" s="8"/>
+      <c r="AH38" s="8"/>
+      <c r="AI38" s="8"/>
+      <c r="AJ38" s="8"/>
+      <c r="AK38" s="10">
         <v>338450</v>
       </c>
     </row>
-    <row r="39" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B39" s="10">
         <v>1156110</v>
@@ -2492,13 +2717,18 @@
       <c r="AC39" s="8"/>
       <c r="AD39" s="8"/>
       <c r="AE39" s="8"/>
-      <c r="AF39" s="10">
+      <c r="AF39" s="8"/>
+      <c r="AG39" s="8"/>
+      <c r="AH39" s="8"/>
+      <c r="AI39" s="8"/>
+      <c r="AJ39" s="8"/>
+      <c r="AK39" s="10">
         <v>1156110</v>
       </c>
     </row>
-    <row r="40" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B40" s="10">
         <v>594115</v>
@@ -2538,13 +2768,18 @@
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
       <c r="AE40" s="8"/>
-      <c r="AF40" s="10">
+      <c r="AF40" s="8"/>
+      <c r="AG40" s="8"/>
+      <c r="AH40" s="8"/>
+      <c r="AI40" s="8"/>
+      <c r="AJ40" s="8"/>
+      <c r="AK40" s="10">
         <v>594115</v>
       </c>
     </row>
-    <row r="41" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B41" s="10">
         <v>338679</v>
@@ -2584,13 +2819,18 @@
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
       <c r="AE41" s="8"/>
-      <c r="AF41" s="10">
+      <c r="AF41" s="8"/>
+      <c r="AG41" s="8"/>
+      <c r="AH41" s="8"/>
+      <c r="AI41" s="8"/>
+      <c r="AJ41" s="8"/>
+      <c r="AK41" s="10">
         <v>338679</v>
       </c>
     </row>
-    <row r="42" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B42" s="10">
         <v>1707090</v>
@@ -2630,13 +2870,18 @@
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
       <c r="AE42" s="8"/>
-      <c r="AF42" s="10">
+      <c r="AF42" s="8"/>
+      <c r="AG42" s="8"/>
+      <c r="AH42" s="8"/>
+      <c r="AI42" s="8"/>
+      <c r="AJ42" s="8"/>
+      <c r="AK42" s="10">
         <v>1707090</v>
       </c>
     </row>
-    <row r="43" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B43" s="10">
         <v>80000</v>
@@ -2674,13 +2919,18 @@
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
       <c r="AE43" s="8"/>
-      <c r="AF43" s="10">
+      <c r="AF43" s="8"/>
+      <c r="AG43" s="8"/>
+      <c r="AH43" s="8"/>
+      <c r="AI43" s="8"/>
+      <c r="AJ43" s="8"/>
+      <c r="AK43" s="10">
         <v>80000</v>
       </c>
     </row>
-    <row r="44" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B44" s="10">
         <v>1199960</v>
@@ -2720,13 +2970,18 @@
       <c r="AC44" s="8"/>
       <c r="AD44" s="8"/>
       <c r="AE44" s="8"/>
-      <c r="AF44" s="10">
+      <c r="AF44" s="8"/>
+      <c r="AG44" s="8"/>
+      <c r="AH44" s="8"/>
+      <c r="AI44" s="8"/>
+      <c r="AJ44" s="8"/>
+      <c r="AK44" s="10">
         <v>1199960</v>
       </c>
     </row>
-    <row r="45" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B45" s="10">
         <v>600000</v>
@@ -2766,13 +3021,18 @@
       <c r="AC45" s="8"/>
       <c r="AD45" s="8"/>
       <c r="AE45" s="8"/>
-      <c r="AF45" s="10">
+      <c r="AF45" s="8"/>
+      <c r="AG45" s="8"/>
+      <c r="AH45" s="8"/>
+      <c r="AI45" s="8"/>
+      <c r="AJ45" s="8"/>
+      <c r="AK45" s="10">
         <v>600000</v>
       </c>
     </row>
-    <row r="46" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B46" s="10">
         <v>317648</v>
@@ -2812,13 +3072,18 @@
       <c r="AC46" s="8"/>
       <c r="AD46" s="8"/>
       <c r="AE46" s="8"/>
-      <c r="AF46" s="10">
+      <c r="AF46" s="8"/>
+      <c r="AG46" s="8"/>
+      <c r="AH46" s="8"/>
+      <c r="AI46" s="8"/>
+      <c r="AJ46" s="8"/>
+      <c r="AK46" s="10">
         <v>317648</v>
       </c>
     </row>
-    <row r="47" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B47" s="10">
         <v>832813</v>
@@ -2858,13 +3123,18 @@
       <c r="AC47" s="8"/>
       <c r="AD47" s="8"/>
       <c r="AE47" s="8"/>
-      <c r="AF47" s="10">
+      <c r="AF47" s="8"/>
+      <c r="AG47" s="8"/>
+      <c r="AH47" s="8"/>
+      <c r="AI47" s="8"/>
+      <c r="AJ47" s="8"/>
+      <c r="AK47" s="10">
         <v>832813</v>
       </c>
     </row>
-    <row r="48" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B48" s="10">
         <v>341237</v>
@@ -2904,13 +3174,18 @@
       <c r="AC48" s="8"/>
       <c r="AD48" s="8"/>
       <c r="AE48" s="8"/>
-      <c r="AF48" s="10">
+      <c r="AF48" s="8"/>
+      <c r="AG48" s="8"/>
+      <c r="AH48" s="8"/>
+      <c r="AI48" s="8"/>
+      <c r="AJ48" s="8"/>
+      <c r="AK48" s="10">
         <v>341237</v>
       </c>
     </row>
-    <row r="49" spans="1:32" ht="69" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B49" s="10">
         <v>666700</v>
@@ -2950,13 +3225,18 @@
       <c r="AC49" s="8"/>
       <c r="AD49" s="8"/>
       <c r="AE49" s="8"/>
-      <c r="AF49" s="10">
+      <c r="AF49" s="8"/>
+      <c r="AG49" s="8"/>
+      <c r="AH49" s="8"/>
+      <c r="AI49" s="8"/>
+      <c r="AJ49" s="8"/>
+      <c r="AK49" s="10">
         <v>666700</v>
       </c>
     </row>
-    <row r="50" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B50" s="10">
         <v>460000</v>
@@ -2996,13 +3276,18 @@
       <c r="AE50" s="8">
         <v>92000</v>
       </c>
-      <c r="AF50" s="10">
+      <c r="AF50" s="8"/>
+      <c r="AG50" s="8"/>
+      <c r="AH50" s="8"/>
+      <c r="AI50" s="8"/>
+      <c r="AJ50" s="8"/>
+      <c r="AK50" s="10">
         <v>460000</v>
       </c>
     </row>
-    <row r="51" spans="1:32" ht="46.2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B51" s="10">
         <v>206880</v>
@@ -3040,13 +3325,18 @@
       <c r="AC51" s="8"/>
       <c r="AD51" s="8"/>
       <c r="AE51" s="8"/>
-      <c r="AF51" s="10">
+      <c r="AF51" s="8"/>
+      <c r="AG51" s="8"/>
+      <c r="AH51" s="8"/>
+      <c r="AI51" s="8"/>
+      <c r="AJ51" s="8"/>
+      <c r="AK51" s="10">
         <v>206880</v>
       </c>
     </row>
-    <row r="52" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B52" s="10">
         <v>799875</v>
@@ -3086,13 +3376,18 @@
       <c r="AC52" s="8"/>
       <c r="AD52" s="8"/>
       <c r="AE52" s="8"/>
-      <c r="AF52" s="10">
+      <c r="AF52" s="8"/>
+      <c r="AG52" s="8"/>
+      <c r="AH52" s="8"/>
+      <c r="AI52" s="8"/>
+      <c r="AJ52" s="8"/>
+      <c r="AK52" s="10">
         <v>799875</v>
       </c>
     </row>
-    <row r="53" spans="1:32" ht="57.6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B53" s="10">
         <v>411073</v>
@@ -3130,13 +3425,18 @@
       <c r="AC53" s="8"/>
       <c r="AD53" s="8"/>
       <c r="AE53" s="8"/>
-      <c r="AF53" s="10">
+      <c r="AF53" s="8"/>
+      <c r="AG53" s="8"/>
+      <c r="AH53" s="8"/>
+      <c r="AI53" s="8"/>
+      <c r="AJ53" s="8"/>
+      <c r="AK53" s="10">
         <v>411073</v>
       </c>
     </row>
-    <row r="54" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B54" s="10">
         <v>90000</v>
@@ -3164,9 +3464,7 @@
       <c r="W54" s="8">
         <v>60000</v>
       </c>
-      <c r="X54" s="8">
-        <v>30000</v>
-      </c>
+      <c r="X54" s="8"/>
       <c r="Y54" s="8"/>
       <c r="Z54" s="8"/>
       <c r="AA54" s="8"/>
@@ -3174,13 +3472,20 @@
       <c r="AC54" s="8"/>
       <c r="AD54" s="8"/>
       <c r="AE54" s="8"/>
-      <c r="AF54" s="10">
+      <c r="AF54" s="8"/>
+      <c r="AG54" s="8"/>
+      <c r="AH54" s="8"/>
+      <c r="AI54" s="8"/>
+      <c r="AJ54" s="8">
+        <v>30000</v>
+      </c>
+      <c r="AK54" s="10">
         <v>90000</v>
       </c>
     </row>
-    <row r="55" spans="1:32" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B55" s="10">
         <v>90000</v>
@@ -3218,13 +3523,18 @@
       <c r="AC55" s="8"/>
       <c r="AD55" s="8"/>
       <c r="AE55" s="8"/>
-      <c r="AF55" s="10">
+      <c r="AF55" s="8"/>
+      <c r="AG55" s="8"/>
+      <c r="AH55" s="8"/>
+      <c r="AI55" s="8"/>
+      <c r="AJ55" s="8"/>
+      <c r="AK55" s="10">
         <v>90000</v>
       </c>
     </row>
-    <row r="56" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="11" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B56" s="12">
         <v>12085865</v>
@@ -3293,7 +3603,7 @@
         <v>1811270</v>
       </c>
       <c r="X56" s="12">
-        <v>379950</v>
+        <v>349950</v>
       </c>
       <c r="Y56" s="12">
         <v>821658</v>
@@ -3317,12 +3627,27 @@
         <v>92000</v>
       </c>
       <c r="AF56" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG56" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH56" s="12">
+        <v>0</v>
+      </c>
+      <c r="AI56" s="12">
+        <v>0</v>
+      </c>
+      <c r="AJ56" s="12">
+        <v>30000</v>
+      </c>
+      <c r="AK56" s="12">
         <v>12085865</v>
       </c>
     </row>
-    <row r="58" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:37" x14ac:dyDescent="0.2">
       <c r="A58" s="4" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -3355,14 +3680,19 @@
       <c r="AD58" s="4"/>
       <c r="AE58" s="4"/>
       <c r="AF58" s="4"/>
+      <c r="AG58" s="4"/>
+      <c r="AH58" s="4"/>
+      <c r="AI58" s="4"/>
+      <c r="AJ58" s="4"/>
+      <c r="AK58" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="A2:AF2"/>
-    <mergeCell ref="A58:AF58"/>
-    <mergeCell ref="A4:AF4"/>
-    <mergeCell ref="A31:AF31"/>
+    <mergeCell ref="A1:AK1"/>
+    <mergeCell ref="A2:AK2"/>
+    <mergeCell ref="A58:AK58"/>
+    <mergeCell ref="A4:AK4"/>
+    <mergeCell ref="A31:AK31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-22 14:01)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{476E8975-DB6D-4506-9C3F-08F6BD2934B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BAED90B-6719-4EA0-9316-93FC05D404ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4E776A27-F0C1-47BA-9ABF-E64A2435029D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{10EA8200-63E7-4A93-AF1B-3C8B6F8D129D}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -718,7 +718,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94B8C11F-44F2-4F2C-8642-5BB90466B6E4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E0EF4B1-D70D-466D-9FBF-DE97DCAF4E5F}">
   <dimension ref="A1:AK58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-22 16:16)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2BAED90B-6719-4EA0-9316-93FC05D404ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE4C6B58-D972-4CC0-9540-0BB32BD86133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{10EA8200-63E7-4A93-AF1B-3C8B6F8D129D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05044D08-4A21-4975-B773-1960599A5386}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -718,7 +718,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E0EF4B1-D70D-466D-9FBF-DE97DCAF4E5F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74E766A6-1120-4D54-885A-974277E9BA7C}">
   <dimension ref="A1:AK58"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-09-25 09:16)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE4C6B58-D972-4CC0-9540-0BB32BD86133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE3BD12D-062C-4472-97D0-BAAFCDD5C2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05044D08-4A21-4975-B773-1960599A5386}"/>
+    <workbookView xWindow="2172" yWindow="1776" windowWidth="13572" windowHeight="10368" xr2:uid="{9C1A0B4E-EAE1-4787-B7FF-251A4FD0E53F}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -39,12 +39,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="66">
-  <si>
-    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (23 โครงการ PO)</t>
-  </si>
-  <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-22</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="68">
+  <si>
+    <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
+  </si>
+  <si>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-25</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -225,6 +225,12 @@
   </si>
   <si>
     <t>MMJ : AP บ้านกลางเมืองคุณมอส</t>
+  </si>
+  <si>
+    <t>SKP Residence</t>
+  </si>
+  <si>
+    <t>บ้านคุณหญิงต้น</t>
   </si>
   <si>
     <t>K'Ink &amp; K'Cody Residence</t>
@@ -718,8 +724,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74E766A6-1120-4D54-885A-974277E9BA7C}">
-  <dimension ref="A1:AK58"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD477BE-9F95-4BD4-86B1-85C5381668FA}">
+  <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
@@ -2057,12 +2063,12 @@
         <v>171149</v>
       </c>
     </row>
-    <row r="28" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:37" ht="23.4" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>62</v>
       </c>
       <c r="B28" s="10">
-        <v>158800</v>
+        <v>0</v>
       </c>
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
@@ -2083,15 +2089,9 @@
       <c r="S28" s="8"/>
       <c r="T28" s="8"/>
       <c r="U28" s="8"/>
-      <c r="V28" s="8">
-        <v>48300</v>
-      </c>
-      <c r="W28" s="8">
-        <v>80500</v>
-      </c>
-      <c r="X28" s="8">
-        <v>30000</v>
-      </c>
+      <c r="V28" s="8"/>
+      <c r="W28" s="8"/>
+      <c r="X28" s="8"/>
       <c r="Y28" s="8"/>
       <c r="Z28" s="8"/>
       <c r="AA28" s="8"/>
@@ -2105,384 +2105,378 @@
       <c r="AI28" s="8"/>
       <c r="AJ28" s="8"/>
       <c r="AK28" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:37" ht="23.4" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="10">
+        <v>0</v>
+      </c>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="8"/>
+      <c r="T29" s="8"/>
+      <c r="U29" s="8"/>
+      <c r="V29" s="8"/>
+      <c r="W29" s="8"/>
+      <c r="X29" s="8"/>
+      <c r="Y29" s="8"/>
+      <c r="Z29" s="8"/>
+      <c r="AA29" s="8"/>
+      <c r="AB29" s="8"/>
+      <c r="AC29" s="8"/>
+      <c r="AD29" s="8"/>
+      <c r="AE29" s="8"/>
+      <c r="AF29" s="8"/>
+      <c r="AG29" s="8"/>
+      <c r="AH29" s="8"/>
+      <c r="AI29" s="8"/>
+      <c r="AJ29" s="8"/>
+      <c r="AK29" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="10">
         <v>158800</v>
       </c>
-    </row>
-    <row r="29" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="12">
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8"/>
+      <c r="N30" s="8"/>
+      <c r="O30" s="8"/>
+      <c r="P30" s="8"/>
+      <c r="Q30" s="8"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="8"/>
+      <c r="T30" s="8"/>
+      <c r="U30" s="8"/>
+      <c r="V30" s="8">
+        <v>48300</v>
+      </c>
+      <c r="W30" s="8">
+        <v>80500</v>
+      </c>
+      <c r="X30" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Y30" s="8"/>
+      <c r="Z30" s="8"/>
+      <c r="AA30" s="8"/>
+      <c r="AB30" s="8"/>
+      <c r="AC30" s="8"/>
+      <c r="AD30" s="8"/>
+      <c r="AE30" s="8"/>
+      <c r="AF30" s="8"/>
+      <c r="AG30" s="8"/>
+      <c r="AH30" s="8"/>
+      <c r="AI30" s="8"/>
+      <c r="AJ30" s="8"/>
+      <c r="AK30" s="10">
+        <v>158800</v>
+      </c>
+    </row>
+    <row r="31" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" s="12">
         <v>4826583</v>
       </c>
-      <c r="C29" s="12">
+      <c r="C31" s="12">
         <v>139012</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D31" s="12">
         <v>231688</v>
       </c>
-      <c r="E29" s="12">
-        <v>0</v>
-      </c>
-      <c r="F29" s="12">
-        <v>0</v>
-      </c>
-      <c r="G29" s="12">
-        <v>0</v>
-      </c>
-      <c r="H29" s="12">
-        <v>0</v>
-      </c>
-      <c r="I29" s="12">
-        <v>0</v>
-      </c>
-      <c r="J29" s="12">
-        <v>0</v>
-      </c>
-      <c r="K29" s="12">
-        <v>0</v>
-      </c>
-      <c r="L29" s="12">
-        <v>0</v>
-      </c>
-      <c r="M29" s="12">
-        <v>0</v>
-      </c>
-      <c r="N29" s="12">
-        <v>0</v>
-      </c>
-      <c r="O29" s="12">
+      <c r="E31" s="12">
+        <v>0</v>
+      </c>
+      <c r="F31" s="12">
+        <v>0</v>
+      </c>
+      <c r="G31" s="12">
+        <v>0</v>
+      </c>
+      <c r="H31" s="12">
+        <v>0</v>
+      </c>
+      <c r="I31" s="12">
+        <v>0</v>
+      </c>
+      <c r="J31" s="12">
+        <v>0</v>
+      </c>
+      <c r="K31" s="12">
+        <v>0</v>
+      </c>
+      <c r="L31" s="12">
+        <v>0</v>
+      </c>
+      <c r="M31" s="12">
+        <v>0</v>
+      </c>
+      <c r="N31" s="12">
+        <v>0</v>
+      </c>
+      <c r="O31" s="12">
         <v>229452</v>
       </c>
-      <c r="P29" s="12">
+      <c r="P31" s="12">
         <v>223986</v>
       </c>
-      <c r="Q29" s="12">
+      <c r="Q31" s="12">
         <v>229402</v>
       </c>
-      <c r="R29" s="12">
+      <c r="R31" s="12">
         <v>272600</v>
       </c>
-      <c r="S29" s="12">
+      <c r="S31" s="12">
         <v>337404</v>
       </c>
-      <c r="T29" s="12">
+      <c r="T31" s="12">
         <v>739676</v>
       </c>
-      <c r="U29" s="12">
+      <c r="U31" s="12">
         <v>327000</v>
       </c>
-      <c r="V29" s="12">
+      <c r="V31" s="12">
         <v>457379</v>
       </c>
-      <c r="W29" s="12">
+      <c r="W31" s="12">
         <v>925214</v>
       </c>
-      <c r="X29" s="12">
+      <c r="X31" s="12">
         <v>296922</v>
       </c>
-      <c r="Y29" s="12">
+      <c r="Y31" s="12">
         <v>155974</v>
       </c>
-      <c r="Z29" s="12">
+      <c r="Z31" s="12">
         <v>187274</v>
       </c>
-      <c r="AA29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AB29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AC29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AD29" s="12">
+      <c r="AA31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AB31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AC31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="12">
         <v>43600</v>
       </c>
-      <c r="AE29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AF29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AG29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AH29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AI29" s="12">
-        <v>0</v>
-      </c>
-      <c r="AJ29" s="12">
+      <c r="AE31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AF31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AI31" s="12">
+        <v>0</v>
+      </c>
+      <c r="AJ31" s="12">
         <v>30000</v>
       </c>
-      <c r="AK29" s="12">
+      <c r="AK31" s="12">
         <v>4826583</v>
       </c>
     </row>
-    <row r="31" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5"/>
-      <c r="P31" s="5"/>
-      <c r="Q31" s="5"/>
-      <c r="R31" s="5"/>
-      <c r="S31" s="5"/>
-      <c r="T31" s="5"/>
-      <c r="U31" s="5"/>
-      <c r="V31" s="5"/>
-      <c r="W31" s="5"/>
-      <c r="X31" s="5"/>
-      <c r="Y31" s="5"/>
-      <c r="Z31" s="5"/>
-      <c r="AA31" s="5"/>
-      <c r="AB31" s="5"/>
-      <c r="AC31" s="5"/>
-      <c r="AD31" s="5"/>
-      <c r="AE31" s="5"/>
-      <c r="AF31" s="5"/>
-      <c r="AG31" s="5"/>
-      <c r="AH31" s="5"/>
-      <c r="AI31" s="5"/>
-      <c r="AJ31" s="5"/>
-      <c r="AK31" s="5"/>
-    </row>
-    <row r="32" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+    <row r="33" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
+      <c r="U33" s="5"/>
+      <c r="V33" s="5"/>
+      <c r="W33" s="5"/>
+      <c r="X33" s="5"/>
+      <c r="Y33" s="5"/>
+      <c r="Z33" s="5"/>
+      <c r="AA33" s="5"/>
+      <c r="AB33" s="5"/>
+      <c r="AC33" s="5"/>
+      <c r="AD33" s="5"/>
+      <c r="AE33" s="5"/>
+      <c r="AF33" s="5"/>
+      <c r="AG33" s="5"/>
+      <c r="AH33" s="5"/>
+      <c r="AI33" s="5"/>
+      <c r="AJ33" s="5"/>
+      <c r="AK33" s="5"/>
+    </row>
+    <row r="34" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B34" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C34" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D34" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="E34" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F34" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="G34" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H32" s="7" t="s">
+      <c r="H34" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I32" s="7" t="s">
+      <c r="I34" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="J32" s="7" t="s">
+      <c r="J34" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="K32" s="7" t="s">
+      <c r="K34" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="L32" s="7" t="s">
+      <c r="L34" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="M32" s="7" t="s">
+      <c r="M34" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N32" s="7" t="s">
+      <c r="N34" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="O32" s="7" t="s">
+      <c r="O34" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="P32" s="7" t="s">
+      <c r="P34" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Q32" s="7" t="s">
+      <c r="Q34" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="R32" s="7" t="s">
+      <c r="R34" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="S32" s="7" t="s">
+      <c r="S34" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="T32" s="7" t="s">
+      <c r="T34" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="U32" s="7" t="s">
+      <c r="U34" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="V32" s="7" t="s">
+      <c r="V34" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="W32" s="7" t="s">
+      <c r="W34" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="X32" s="7" t="s">
+      <c r="X34" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="Y32" s="7" t="s">
+      <c r="Y34" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="Z32" s="7" t="s">
+      <c r="Z34" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="AA32" s="7" t="s">
+      <c r="AA34" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="AB32" s="7" t="s">
+      <c r="AB34" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="AC32" s="7" t="s">
+      <c r="AC34" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AD32" s="7" t="s">
+      <c r="AD34" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="AE32" s="7" t="s">
+      <c r="AE34" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="AF32" s="7" t="s">
+      <c r="AF34" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="AG32" s="7" t="s">
+      <c r="AG34" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="AH32" s="7" t="s">
+      <c r="AH34" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="AI32" s="7" t="s">
+      <c r="AI34" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="AJ32" s="7" t="s">
+      <c r="AJ34" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="AK32" s="6" t="s">
+      <c r="AK34" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="33" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
+    <row r="35" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B33" s="10">
+      <c r="B35" s="10">
         <v>294109</v>
-      </c>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8"/>
-      <c r="I33" s="8"/>
-      <c r="J33" s="8"/>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8">
-        <v>130715</v>
-      </c>
-      <c r="P33" s="8"/>
-      <c r="Q33" s="8"/>
-      <c r="R33" s="8"/>
-      <c r="S33" s="8"/>
-      <c r="T33" s="8">
-        <v>130715</v>
-      </c>
-      <c r="U33" s="8"/>
-      <c r="V33" s="8">
-        <v>32679</v>
-      </c>
-      <c r="W33" s="8"/>
-      <c r="X33" s="8"/>
-      <c r="Y33" s="8"/>
-      <c r="Z33" s="8"/>
-      <c r="AA33" s="8"/>
-      <c r="AB33" s="8"/>
-      <c r="AC33" s="8"/>
-      <c r="AD33" s="8"/>
-      <c r="AE33" s="8"/>
-      <c r="AF33" s="8"/>
-      <c r="AG33" s="8"/>
-      <c r="AH33" s="8"/>
-      <c r="AI33" s="8"/>
-      <c r="AJ33" s="8"/>
-      <c r="AK33" s="10">
-        <v>294109</v>
-      </c>
-    </row>
-    <row r="34" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
-      <c r="A34" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B34" s="10">
-        <v>409600</v>
-      </c>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8"/>
-      <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8">
-        <v>163840</v>
-      </c>
-      <c r="Q34" s="8"/>
-      <c r="R34" s="8"/>
-      <c r="S34" s="8"/>
-      <c r="T34" s="8"/>
-      <c r="U34" s="8"/>
-      <c r="V34" s="8"/>
-      <c r="W34" s="8">
-        <v>163840</v>
-      </c>
-      <c r="X34" s="8"/>
-      <c r="Y34" s="8">
-        <v>81920</v>
-      </c>
-      <c r="Z34" s="8"/>
-      <c r="AA34" s="8"/>
-      <c r="AB34" s="8"/>
-      <c r="AC34" s="8"/>
-      <c r="AD34" s="8"/>
-      <c r="AE34" s="8"/>
-      <c r="AF34" s="8"/>
-      <c r="AG34" s="8"/>
-      <c r="AH34" s="8"/>
-      <c r="AI34" s="8"/>
-      <c r="AJ34" s="8"/>
-      <c r="AK34" s="10">
-        <v>409600</v>
-      </c>
-    </row>
-    <row r="35" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
-      <c r="A35" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B35" s="10">
-        <v>576318</v>
       </c>
       <c r="C35" s="8"/>
       <c r="D35" s="8"/>
@@ -2497,19 +2491,19 @@
       <c r="M35" s="8"/>
       <c r="N35" s="8"/>
       <c r="O35" s="8">
-        <v>230527</v>
-      </c>
-      <c r="P35" s="8">
-        <v>230527</v>
-      </c>
+        <v>130715</v>
+      </c>
+      <c r="P35" s="8"/>
       <c r="Q35" s="8"/>
       <c r="R35" s="8"/>
       <c r="S35" s="8"/>
       <c r="T35" s="8">
-        <v>115264</v>
+        <v>130715</v>
       </c>
       <c r="U35" s="8"/>
-      <c r="V35" s="8"/>
+      <c r="V35" s="8">
+        <v>32679</v>
+      </c>
       <c r="W35" s="8"/>
       <c r="X35" s="8"/>
       <c r="Y35" s="8"/>
@@ -2525,15 +2519,15 @@
       <c r="AI35" s="8"/>
       <c r="AJ35" s="8"/>
       <c r="AK35" s="10">
-        <v>576318</v>
-      </c>
-    </row>
-    <row r="36" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+        <v>294109</v>
+      </c>
+    </row>
+    <row r="36" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B36" s="10">
-        <v>322960</v>
+        <v>409600</v>
       </c>
       <c r="C36" s="8"/>
       <c r="D36" s="8"/>
@@ -2548,20 +2542,22 @@
       <c r="M36" s="8"/>
       <c r="N36" s="8"/>
       <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
+      <c r="P36" s="8">
+        <v>163840</v>
+      </c>
       <c r="Q36" s="8"/>
-      <c r="R36" s="8">
-        <v>129184</v>
-      </c>
-      <c r="S36" s="8">
-        <v>193776</v>
-      </c>
+      <c r="R36" s="8"/>
+      <c r="S36" s="8"/>
       <c r="T36" s="8"/>
       <c r="U36" s="8"/>
       <c r="V36" s="8"/>
-      <c r="W36" s="8"/>
+      <c r="W36" s="8">
+        <v>163840</v>
+      </c>
       <c r="X36" s="8"/>
-      <c r="Y36" s="8"/>
+      <c r="Y36" s="8">
+        <v>81920</v>
+      </c>
       <c r="Z36" s="8"/>
       <c r="AA36" s="8"/>
       <c r="AB36" s="8"/>
@@ -2574,15 +2570,15 @@
       <c r="AI36" s="8"/>
       <c r="AJ36" s="8"/>
       <c r="AK36" s="10">
-        <v>322960</v>
-      </c>
-    </row>
-    <row r="37" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+        <v>409600</v>
+      </c>
+    </row>
+    <row r="37" spans="1:37" ht="80.400000000000006" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B37" s="10">
-        <v>252248</v>
+        <v>576318</v>
       </c>
       <c r="C37" s="8"/>
       <c r="D37" s="8"/>
@@ -2596,19 +2592,23 @@
       <c r="L37" s="8"/>
       <c r="M37" s="8"/>
       <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
-      <c r="P37" s="8"/>
+      <c r="O37" s="8">
+        <v>230527</v>
+      </c>
+      <c r="P37" s="8">
+        <v>230527</v>
+      </c>
       <c r="Q37" s="8"/>
       <c r="R37" s="8"/>
       <c r="S37" s="8"/>
-      <c r="T37" s="8"/>
+      <c r="T37" s="8">
+        <v>115264</v>
+      </c>
       <c r="U37" s="8"/>
       <c r="V37" s="8"/>
       <c r="W37" s="8"/>
       <c r="X37" s="8"/>
-      <c r="Y37" s="8">
-        <v>252248</v>
-      </c>
+      <c r="Y37" s="8"/>
       <c r="Z37" s="8"/>
       <c r="AA37" s="8"/>
       <c r="AB37" s="8"/>
@@ -2621,15 +2621,15 @@
       <c r="AI37" s="8"/>
       <c r="AJ37" s="8"/>
       <c r="AK37" s="10">
-        <v>252248</v>
-      </c>
-    </row>
-    <row r="38" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+        <v>576318</v>
+      </c>
+    </row>
+    <row r="38" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B38" s="10">
-        <v>338450</v>
+        <v>322960</v>
       </c>
       <c r="C38" s="8"/>
       <c r="D38" s="8"/>
@@ -2647,14 +2647,12 @@
       <c r="P38" s="8"/>
       <c r="Q38" s="8"/>
       <c r="R38" s="8">
-        <v>135380</v>
+        <v>129184</v>
       </c>
       <c r="S38" s="8">
-        <v>135380</v>
-      </c>
-      <c r="T38" s="8">
-        <v>67690</v>
-      </c>
+        <v>193776</v>
+      </c>
+      <c r="T38" s="8"/>
       <c r="U38" s="8"/>
       <c r="V38" s="8"/>
       <c r="W38" s="8"/>
@@ -2672,15 +2670,15 @@
       <c r="AI38" s="8"/>
       <c r="AJ38" s="8"/>
       <c r="AK38" s="10">
-        <v>338450</v>
-      </c>
-    </row>
-    <row r="39" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+        <v>322960</v>
+      </c>
+    </row>
+    <row r="39" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B39" s="10">
-        <v>1156110</v>
+        <v>252248</v>
       </c>
       <c r="C39" s="8"/>
       <c r="D39" s="8"/>
@@ -2697,20 +2695,16 @@
       <c r="O39" s="8"/>
       <c r="P39" s="8"/>
       <c r="Q39" s="8"/>
-      <c r="R39" s="8">
-        <v>462444</v>
-      </c>
+      <c r="R39" s="8"/>
       <c r="S39" s="8"/>
-      <c r="T39" s="8">
-        <v>346833</v>
-      </c>
+      <c r="T39" s="8"/>
       <c r="U39" s="8"/>
       <c r="V39" s="8"/>
-      <c r="W39" s="8">
-        <v>346833</v>
-      </c>
+      <c r="W39" s="8"/>
       <c r="X39" s="8"/>
-      <c r="Y39" s="8"/>
+      <c r="Y39" s="8">
+        <v>252248</v>
+      </c>
       <c r="Z39" s="8"/>
       <c r="AA39" s="8"/>
       <c r="AB39" s="8"/>
@@ -2723,15 +2717,15 @@
       <c r="AI39" s="8"/>
       <c r="AJ39" s="8"/>
       <c r="AK39" s="10">
-        <v>1156110</v>
+        <v>252248</v>
       </c>
     </row>
     <row r="40" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B40" s="10">
-        <v>594115</v>
+        <v>338450</v>
       </c>
       <c r="C40" s="8"/>
       <c r="D40" s="8"/>
@@ -2748,22 +2742,22 @@
       <c r="O40" s="8"/>
       <c r="P40" s="8"/>
       <c r="Q40" s="8"/>
-      <c r="R40" s="8"/>
-      <c r="S40" s="8"/>
-      <c r="T40" s="8"/>
+      <c r="R40" s="8">
+        <v>135380</v>
+      </c>
+      <c r="S40" s="8">
+        <v>135380</v>
+      </c>
+      <c r="T40" s="8">
+        <v>67690</v>
+      </c>
       <c r="U40" s="8"/>
       <c r="V40" s="8"/>
       <c r="W40" s="8"/>
       <c r="X40" s="8"/>
-      <c r="Y40" s="8">
-        <v>237646</v>
-      </c>
-      <c r="Z40" s="8">
-        <v>237646</v>
-      </c>
-      <c r="AA40" s="8">
-        <v>118823</v>
-      </c>
+      <c r="Y40" s="8"/>
+      <c r="Z40" s="8"/>
+      <c r="AA40" s="8"/>
       <c r="AB40" s="8"/>
       <c r="AC40" s="8"/>
       <c r="AD40" s="8"/>
@@ -2774,15 +2768,15 @@
       <c r="AI40" s="8"/>
       <c r="AJ40" s="8"/>
       <c r="AK40" s="10">
-        <v>594115</v>
+        <v>338450</v>
       </c>
     </row>
     <row r="41" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B41" s="10">
-        <v>338679</v>
+        <v>1156110</v>
       </c>
       <c r="C41" s="8"/>
       <c r="D41" s="8"/>
@@ -2800,21 +2794,21 @@
       <c r="P41" s="8"/>
       <c r="Q41" s="8"/>
       <c r="R41" s="8">
-        <v>136629</v>
+        <v>462444</v>
       </c>
       <c r="S41" s="8"/>
-      <c r="T41" s="8"/>
+      <c r="T41" s="8">
+        <v>346833</v>
+      </c>
       <c r="U41" s="8"/>
       <c r="V41" s="8"/>
       <c r="W41" s="8">
-        <v>136629</v>
+        <v>346833</v>
       </c>
       <c r="X41" s="8"/>
       <c r="Y41" s="8"/>
       <c r="Z41" s="8"/>
-      <c r="AA41" s="8">
-        <v>65421</v>
-      </c>
+      <c r="AA41" s="8"/>
       <c r="AB41" s="8"/>
       <c r="AC41" s="8"/>
       <c r="AD41" s="8"/>
@@ -2825,15 +2819,15 @@
       <c r="AI41" s="8"/>
       <c r="AJ41" s="8"/>
       <c r="AK41" s="10">
-        <v>338679</v>
-      </c>
-    </row>
-    <row r="42" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+        <v>1156110</v>
+      </c>
+    </row>
+    <row r="42" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B42" s="10">
-        <v>1707090</v>
+        <v>594115</v>
       </c>
       <c r="C42" s="8"/>
       <c r="D42" s="8"/>
@@ -2851,21 +2845,21 @@
       <c r="P42" s="8"/>
       <c r="Q42" s="8"/>
       <c r="R42" s="8"/>
-      <c r="S42" s="8">
-        <v>682836</v>
-      </c>
-      <c r="T42" s="8">
-        <v>682836</v>
-      </c>
-      <c r="U42" s="8">
-        <v>341418</v>
-      </c>
+      <c r="S42" s="8"/>
+      <c r="T42" s="8"/>
+      <c r="U42" s="8"/>
       <c r="V42" s="8"/>
       <c r="W42" s="8"/>
       <c r="X42" s="8"/>
-      <c r="Y42" s="8"/>
-      <c r="Z42" s="8"/>
-      <c r="AA42" s="8"/>
+      <c r="Y42" s="8">
+        <v>237646</v>
+      </c>
+      <c r="Z42" s="8">
+        <v>237646</v>
+      </c>
+      <c r="AA42" s="8">
+        <v>118823</v>
+      </c>
       <c r="AB42" s="8"/>
       <c r="AC42" s="8"/>
       <c r="AD42" s="8"/>
@@ -2876,15 +2870,15 @@
       <c r="AI42" s="8"/>
       <c r="AJ42" s="8"/>
       <c r="AK42" s="10">
-        <v>1707090</v>
-      </c>
-    </row>
-    <row r="43" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+        <v>594115</v>
+      </c>
+    </row>
+    <row r="43" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B43" s="10">
-        <v>80000</v>
+        <v>338679</v>
       </c>
       <c r="C43" s="8"/>
       <c r="D43" s="8"/>
@@ -2902,19 +2896,21 @@
       <c r="P43" s="8"/>
       <c r="Q43" s="8"/>
       <c r="R43" s="8">
-        <v>32000</v>
-      </c>
-      <c r="S43" s="8">
-        <v>48000</v>
-      </c>
+        <v>136629</v>
+      </c>
+      <c r="S43" s="8"/>
       <c r="T43" s="8"/>
       <c r="U43" s="8"/>
       <c r="V43" s="8"/>
-      <c r="W43" s="8"/>
+      <c r="W43" s="8">
+        <v>136629</v>
+      </c>
       <c r="X43" s="8"/>
       <c r="Y43" s="8"/>
       <c r="Z43" s="8"/>
-      <c r="AA43" s="8"/>
+      <c r="AA43" s="8">
+        <v>65421</v>
+      </c>
       <c r="AB43" s="8"/>
       <c r="AC43" s="8"/>
       <c r="AD43" s="8"/>
@@ -2925,15 +2921,15 @@
       <c r="AI43" s="8"/>
       <c r="AJ43" s="8"/>
       <c r="AK43" s="10">
-        <v>80000</v>
+        <v>338679</v>
       </c>
     </row>
     <row r="44" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B44" s="10">
-        <v>1199960</v>
+        <v>1707090</v>
       </c>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -2952,19 +2948,19 @@
       <c r="Q44" s="8"/>
       <c r="R44" s="8"/>
       <c r="S44" s="8">
-        <v>479984</v>
-      </c>
-      <c r="T44" s="8"/>
-      <c r="U44" s="8"/>
+        <v>682836</v>
+      </c>
+      <c r="T44" s="8">
+        <v>682836</v>
+      </c>
+      <c r="U44" s="8">
+        <v>341418</v>
+      </c>
       <c r="V44" s="8"/>
-      <c r="W44" s="8">
-        <v>479984</v>
-      </c>
+      <c r="W44" s="8"/>
       <c r="X44" s="8"/>
       <c r="Y44" s="8"/>
-      <c r="Z44" s="8">
-        <v>239992</v>
-      </c>
+      <c r="Z44" s="8"/>
       <c r="AA44" s="8"/>
       <c r="AB44" s="8"/>
       <c r="AC44" s="8"/>
@@ -2976,15 +2972,15 @@
       <c r="AI44" s="8"/>
       <c r="AJ44" s="8"/>
       <c r="AK44" s="10">
-        <v>1199960</v>
-      </c>
-    </row>
-    <row r="45" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+        <v>1707090</v>
+      </c>
+    </row>
+    <row r="45" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B45" s="10">
-        <v>600000</v>
+        <v>80000</v>
       </c>
       <c r="C45" s="8"/>
       <c r="D45" s="8"/>
@@ -2998,17 +2994,15 @@
       <c r="L45" s="8"/>
       <c r="M45" s="8"/>
       <c r="N45" s="8"/>
-      <c r="O45" s="8">
-        <v>240000</v>
-      </c>
+      <c r="O45" s="8"/>
       <c r="P45" s="8"/>
-      <c r="Q45" s="8">
-        <v>180000</v>
-      </c>
+      <c r="Q45" s="8"/>
       <c r="R45" s="8">
-        <v>180000</v>
-      </c>
-      <c r="S45" s="8"/>
+        <v>32000</v>
+      </c>
+      <c r="S45" s="8">
+        <v>48000</v>
+      </c>
       <c r="T45" s="8"/>
       <c r="U45" s="8"/>
       <c r="V45" s="8"/>
@@ -3027,15 +3021,15 @@
       <c r="AI45" s="8"/>
       <c r="AJ45" s="8"/>
       <c r="AK45" s="10">
-        <v>600000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B46" s="10">
-        <v>317648</v>
+        <v>1199960</v>
       </c>
       <c r="C46" s="8"/>
       <c r="D46" s="8"/>
@@ -3049,24 +3043,24 @@
       <c r="L46" s="8"/>
       <c r="M46" s="8"/>
       <c r="N46" s="8"/>
-      <c r="O46" s="8">
-        <v>127059</v>
-      </c>
-      <c r="P46" s="8">
-        <v>127059</v>
-      </c>
+      <c r="O46" s="8"/>
+      <c r="P46" s="8"/>
       <c r="Q46" s="8"/>
-      <c r="R46" s="8">
-        <v>63530</v>
-      </c>
-      <c r="S46" s="8"/>
+      <c r="R46" s="8"/>
+      <c r="S46" s="8">
+        <v>479984</v>
+      </c>
       <c r="T46" s="8"/>
       <c r="U46" s="8"/>
       <c r="V46" s="8"/>
-      <c r="W46" s="8"/>
+      <c r="W46" s="8">
+        <v>479984</v>
+      </c>
       <c r="X46" s="8"/>
       <c r="Y46" s="8"/>
-      <c r="Z46" s="8"/>
+      <c r="Z46" s="8">
+        <v>239992</v>
+      </c>
       <c r="AA46" s="8"/>
       <c r="AB46" s="8"/>
       <c r="AC46" s="8"/>
@@ -3078,15 +3072,15 @@
       <c r="AI46" s="8"/>
       <c r="AJ46" s="8"/>
       <c r="AK46" s="10">
-        <v>317648</v>
-      </c>
-    </row>
-    <row r="47" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+        <v>1199960</v>
+      </c>
+    </row>
+    <row r="47" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B47" s="10">
-        <v>832813</v>
+        <v>600000</v>
       </c>
       <c r="C47" s="8"/>
       <c r="D47" s="8"/>
@@ -3100,23 +3094,23 @@
       <c r="L47" s="8"/>
       <c r="M47" s="8"/>
       <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
+      <c r="O47" s="8">
+        <v>240000</v>
+      </c>
       <c r="P47" s="8"/>
-      <c r="Q47" s="8"/>
-      <c r="R47" s="8"/>
+      <c r="Q47" s="8">
+        <v>180000</v>
+      </c>
+      <c r="R47" s="8">
+        <v>180000</v>
+      </c>
       <c r="S47" s="8"/>
-      <c r="T47" s="8">
-        <v>333125</v>
-      </c>
-      <c r="U47" s="8">
-        <v>249844</v>
-      </c>
+      <c r="T47" s="8"/>
+      <c r="U47" s="8"/>
       <c r="V47" s="8"/>
       <c r="W47" s="8"/>
       <c r="X47" s="8"/>
-      <c r="Y47" s="8">
-        <v>249844</v>
-      </c>
+      <c r="Y47" s="8"/>
       <c r="Z47" s="8"/>
       <c r="AA47" s="8"/>
       <c r="AB47" s="8"/>
@@ -3129,22 +3123,18 @@
       <c r="AI47" s="8"/>
       <c r="AJ47" s="8"/>
       <c r="AK47" s="10">
-        <v>832813</v>
+        <v>600000</v>
       </c>
     </row>
     <row r="48" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B48" s="10">
-        <v>341237</v>
-      </c>
-      <c r="C48" s="8">
-        <v>136495</v>
-      </c>
-      <c r="D48" s="8">
-        <v>136495</v>
-      </c>
+        <v>317648</v>
+      </c>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
       <c r="E48" s="8"/>
       <c r="F48" s="8"/>
       <c r="G48" s="8"/>
@@ -3155,16 +3145,20 @@
       <c r="L48" s="8"/>
       <c r="M48" s="8"/>
       <c r="N48" s="8"/>
-      <c r="O48" s="8"/>
-      <c r="P48" s="8"/>
+      <c r="O48" s="8">
+        <v>127059</v>
+      </c>
+      <c r="P48" s="8">
+        <v>127059</v>
+      </c>
       <c r="Q48" s="8"/>
-      <c r="R48" s="8"/>
+      <c r="R48" s="8">
+        <v>63530</v>
+      </c>
       <c r="S48" s="8"/>
       <c r="T48" s="8"/>
       <c r="U48" s="8"/>
-      <c r="V48" s="8">
-        <v>68247</v>
-      </c>
+      <c r="V48" s="8"/>
       <c r="W48" s="8"/>
       <c r="X48" s="8"/>
       <c r="Y48" s="8"/>
@@ -3180,22 +3174,18 @@
       <c r="AI48" s="8"/>
       <c r="AJ48" s="8"/>
       <c r="AK48" s="10">
-        <v>341237</v>
-      </c>
-    </row>
-    <row r="49" spans="1:37" ht="69" x14ac:dyDescent="0.25">
+        <v>317648</v>
+      </c>
+    </row>
+    <row r="49" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B49" s="10">
-        <v>666700</v>
-      </c>
-      <c r="C49" s="8">
-        <v>266680</v>
-      </c>
-      <c r="D49" s="8">
-        <v>266680</v>
-      </c>
+        <v>832813</v>
+      </c>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
       <c r="E49" s="8"/>
       <c r="F49" s="8"/>
       <c r="G49" s="8"/>
@@ -3211,14 +3201,18 @@
       <c r="Q49" s="8"/>
       <c r="R49" s="8"/>
       <c r="S49" s="8"/>
-      <c r="T49" s="8"/>
-      <c r="U49" s="8"/>
+      <c r="T49" s="8">
+        <v>333125</v>
+      </c>
+      <c r="U49" s="8">
+        <v>249844</v>
+      </c>
       <c r="V49" s="8"/>
-      <c r="W49" s="8">
-        <v>133340</v>
-      </c>
+      <c r="W49" s="8"/>
       <c r="X49" s="8"/>
-      <c r="Y49" s="8"/>
+      <c r="Y49" s="8">
+        <v>249844</v>
+      </c>
       <c r="Z49" s="8"/>
       <c r="AA49" s="8"/>
       <c r="AB49" s="8"/>
@@ -3231,18 +3225,22 @@
       <c r="AI49" s="8"/>
       <c r="AJ49" s="8"/>
       <c r="AK49" s="10">
-        <v>666700</v>
-      </c>
-    </row>
-    <row r="50" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+        <v>832813</v>
+      </c>
+    </row>
+    <row r="50" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B50" s="10">
-        <v>460000</v>
-      </c>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
+        <v>341237</v>
+      </c>
+      <c r="C50" s="8">
+        <v>136495</v>
+      </c>
+      <c r="D50" s="8">
+        <v>136495</v>
+      </c>
       <c r="E50" s="8"/>
       <c r="F50" s="8"/>
       <c r="G50" s="8"/>
@@ -3258,14 +3256,12 @@
       <c r="Q50" s="8"/>
       <c r="R50" s="8"/>
       <c r="S50" s="8"/>
-      <c r="T50" s="8">
-        <v>184000</v>
-      </c>
+      <c r="T50" s="8"/>
       <c r="U50" s="8"/>
-      <c r="V50" s="8"/>
-      <c r="W50" s="8">
-        <v>184000</v>
-      </c>
+      <c r="V50" s="8">
+        <v>68247</v>
+      </c>
+      <c r="W50" s="8"/>
       <c r="X50" s="8"/>
       <c r="Y50" s="8"/>
       <c r="Z50" s="8"/>
@@ -3273,27 +3269,29 @@
       <c r="AB50" s="8"/>
       <c r="AC50" s="8"/>
       <c r="AD50" s="8"/>
-      <c r="AE50" s="8">
-        <v>92000</v>
-      </c>
+      <c r="AE50" s="8"/>
       <c r="AF50" s="8"/>
       <c r="AG50" s="8"/>
       <c r="AH50" s="8"/>
       <c r="AI50" s="8"/>
       <c r="AJ50" s="8"/>
       <c r="AK50" s="10">
-        <v>460000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
+        <v>341237</v>
+      </c>
+    </row>
+    <row r="51" spans="1:37" ht="69" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B51" s="10">
-        <v>206880</v>
-      </c>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
+        <v>666700</v>
+      </c>
+      <c r="C51" s="8">
+        <v>266680</v>
+      </c>
+      <c r="D51" s="8">
+        <v>266680</v>
+      </c>
       <c r="E51" s="8"/>
       <c r="F51" s="8"/>
       <c r="G51" s="8"/>
@@ -3309,14 +3307,12 @@
       <c r="Q51" s="8"/>
       <c r="R51" s="8"/>
       <c r="S51" s="8"/>
-      <c r="T51" s="8">
-        <v>82752</v>
-      </c>
-      <c r="U51" s="8">
-        <v>124128</v>
-      </c>
+      <c r="T51" s="8"/>
+      <c r="U51" s="8"/>
       <c r="V51" s="8"/>
-      <c r="W51" s="8"/>
+      <c r="W51" s="8">
+        <v>133340</v>
+      </c>
       <c r="X51" s="8"/>
       <c r="Y51" s="8"/>
       <c r="Z51" s="8"/>
@@ -3331,15 +3327,15 @@
       <c r="AI51" s="8"/>
       <c r="AJ51" s="8"/>
       <c r="AK51" s="10">
-        <v>206880</v>
-      </c>
-    </row>
-    <row r="52" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+        <v>666700</v>
+      </c>
+    </row>
+    <row r="52" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B52" s="10">
-        <v>799875</v>
+        <v>460000</v>
       </c>
       <c r="C52" s="8"/>
       <c r="D52" s="8"/>
@@ -3358,39 +3354,39 @@
       <c r="Q52" s="8"/>
       <c r="R52" s="8"/>
       <c r="S52" s="8"/>
-      <c r="T52" s="8"/>
-      <c r="U52" s="8">
-        <v>319950</v>
-      </c>
+      <c r="T52" s="8">
+        <v>184000</v>
+      </c>
+      <c r="U52" s="8"/>
       <c r="V52" s="8"/>
-      <c r="W52" s="8"/>
-      <c r="X52" s="8">
-        <v>319950</v>
-      </c>
+      <c r="W52" s="8">
+        <v>184000</v>
+      </c>
+      <c r="X52" s="8"/>
       <c r="Y52" s="8"/>
       <c r="Z52" s="8"/>
       <c r="AA52" s="8"/>
-      <c r="AB52" s="8">
-        <v>159975</v>
-      </c>
+      <c r="AB52" s="8"/>
       <c r="AC52" s="8"/>
       <c r="AD52" s="8"/>
-      <c r="AE52" s="8"/>
+      <c r="AE52" s="8">
+        <v>92000</v>
+      </c>
       <c r="AF52" s="8"/>
       <c r="AG52" s="8"/>
       <c r="AH52" s="8"/>
       <c r="AI52" s="8"/>
       <c r="AJ52" s="8"/>
       <c r="AK52" s="10">
-        <v>799875</v>
-      </c>
-    </row>
-    <row r="53" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
+        <v>460000</v>
+      </c>
+    </row>
+    <row r="53" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B53" s="10">
-        <v>411073</v>
+        <v>206880</v>
       </c>
       <c r="C53" s="8"/>
       <c r="D53" s="8"/>
@@ -3409,14 +3405,14 @@
       <c r="Q53" s="8"/>
       <c r="R53" s="8"/>
       <c r="S53" s="8"/>
-      <c r="T53" s="8"/>
-      <c r="U53" s="8"/>
-      <c r="V53" s="8">
-        <v>164429</v>
-      </c>
-      <c r="W53" s="8">
-        <v>246644</v>
-      </c>
+      <c r="T53" s="8">
+        <v>82752</v>
+      </c>
+      <c r="U53" s="8">
+        <v>124128</v>
+      </c>
+      <c r="V53" s="8"/>
+      <c r="W53" s="8"/>
       <c r="X53" s="8"/>
       <c r="Y53" s="8"/>
       <c r="Z53" s="8"/>
@@ -3431,15 +3427,15 @@
       <c r="AI53" s="8"/>
       <c r="AJ53" s="8"/>
       <c r="AK53" s="10">
-        <v>411073</v>
-      </c>
-    </row>
-    <row r="54" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+        <v>206880</v>
+      </c>
+    </row>
+    <row r="54" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B54" s="10">
-        <v>90000</v>
+        <v>799875</v>
       </c>
       <c r="C54" s="8"/>
       <c r="D54" s="8"/>
@@ -3459,16 +3455,20 @@
       <c r="R54" s="8"/>
       <c r="S54" s="8"/>
       <c r="T54" s="8"/>
-      <c r="U54" s="8"/>
+      <c r="U54" s="8">
+        <v>319950</v>
+      </c>
       <c r="V54" s="8"/>
-      <c r="W54" s="8">
-        <v>60000</v>
-      </c>
-      <c r="X54" s="8"/>
+      <c r="W54" s="8"/>
+      <c r="X54" s="8">
+        <v>319950</v>
+      </c>
       <c r="Y54" s="8"/>
       <c r="Z54" s="8"/>
       <c r="AA54" s="8"/>
-      <c r="AB54" s="8"/>
+      <c r="AB54" s="8">
+        <v>159975</v>
+      </c>
       <c r="AC54" s="8"/>
       <c r="AD54" s="8"/>
       <c r="AE54" s="8"/>
@@ -3476,19 +3476,17 @@
       <c r="AG54" s="8"/>
       <c r="AH54" s="8"/>
       <c r="AI54" s="8"/>
-      <c r="AJ54" s="8">
-        <v>30000</v>
-      </c>
+      <c r="AJ54" s="8"/>
       <c r="AK54" s="10">
-        <v>90000</v>
-      </c>
-    </row>
-    <row r="55" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+        <v>799875</v>
+      </c>
+    </row>
+    <row r="55" spans="1:37" ht="57.6" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B55" s="10">
-        <v>90000</v>
+        <v>411073</v>
       </c>
       <c r="C55" s="8"/>
       <c r="D55" s="8"/>
@@ -3509,13 +3507,13 @@
       <c r="S55" s="8"/>
       <c r="T55" s="8"/>
       <c r="U55" s="8"/>
-      <c r="V55" s="8"/>
+      <c r="V55" s="8">
+        <v>164429</v>
+      </c>
       <c r="W55" s="8">
-        <v>60000</v>
-      </c>
-      <c r="X55" s="8">
-        <v>30000</v>
-      </c>
+        <v>246644</v>
+      </c>
+      <c r="X55" s="8"/>
       <c r="Y55" s="8"/>
       <c r="Z55" s="8"/>
       <c r="AA55" s="8"/>
@@ -3529,170 +3527,358 @@
       <c r="AI55" s="8"/>
       <c r="AJ55" s="8"/>
       <c r="AK55" s="10">
+        <v>411073</v>
+      </c>
+    </row>
+    <row r="56" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A56" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56" s="10">
         <v>90000</v>
       </c>
-    </row>
-    <row r="56" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="11" t="s">
+      <c r="C56" s="8"/>
+      <c r="D56" s="8"/>
+      <c r="E56" s="8"/>
+      <c r="F56" s="8"/>
+      <c r="G56" s="8"/>
+      <c r="H56" s="8"/>
+      <c r="I56" s="8"/>
+      <c r="J56" s="8"/>
+      <c r="K56" s="8"/>
+      <c r="L56" s="8"/>
+      <c r="M56" s="8"/>
+      <c r="N56" s="8"/>
+      <c r="O56" s="8"/>
+      <c r="P56" s="8"/>
+      <c r="Q56" s="8"/>
+      <c r="R56" s="8"/>
+      <c r="S56" s="8"/>
+      <c r="T56" s="8"/>
+      <c r="U56" s="8"/>
+      <c r="V56" s="8"/>
+      <c r="W56" s="8">
+        <v>60000</v>
+      </c>
+      <c r="X56" s="8"/>
+      <c r="Y56" s="8"/>
+      <c r="Z56" s="8"/>
+      <c r="AA56" s="8"/>
+      <c r="AB56" s="8"/>
+      <c r="AC56" s="8"/>
+      <c r="AD56" s="8"/>
+      <c r="AE56" s="8"/>
+      <c r="AF56" s="8"/>
+      <c r="AG56" s="8"/>
+      <c r="AH56" s="8"/>
+      <c r="AI56" s="8"/>
+      <c r="AJ56" s="8">
+        <v>30000</v>
+      </c>
+      <c r="AK56" s="10">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="57" spans="1:37" ht="23.4" x14ac:dyDescent="0.25">
+      <c r="A57" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B57" s="10">
+        <v>0</v>
+      </c>
+      <c r="C57" s="8"/>
+      <c r="D57" s="8"/>
+      <c r="E57" s="8"/>
+      <c r="F57" s="8"/>
+      <c r="G57" s="8"/>
+      <c r="H57" s="8"/>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8"/>
+      <c r="K57" s="8"/>
+      <c r="L57" s="8"/>
+      <c r="M57" s="8"/>
+      <c r="N57" s="8"/>
+      <c r="O57" s="8"/>
+      <c r="P57" s="8"/>
+      <c r="Q57" s="8"/>
+      <c r="R57" s="8"/>
+      <c r="S57" s="8"/>
+      <c r="T57" s="8"/>
+      <c r="U57" s="8"/>
+      <c r="V57" s="8"/>
+      <c r="W57" s="8"/>
+      <c r="X57" s="8"/>
+      <c r="Y57" s="8"/>
+      <c r="Z57" s="8"/>
+      <c r="AA57" s="8"/>
+      <c r="AB57" s="8"/>
+      <c r="AC57" s="8"/>
+      <c r="AD57" s="8"/>
+      <c r="AE57" s="8"/>
+      <c r="AF57" s="8"/>
+      <c r="AG57" s="8"/>
+      <c r="AH57" s="8"/>
+      <c r="AI57" s="8"/>
+      <c r="AJ57" s="8"/>
+      <c r="AK57" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:37" ht="23.4" x14ac:dyDescent="0.25">
+      <c r="A58" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B56" s="12">
+      <c r="B58" s="10">
+        <v>0</v>
+      </c>
+      <c r="C58" s="8"/>
+      <c r="D58" s="8"/>
+      <c r="E58" s="8"/>
+      <c r="F58" s="8"/>
+      <c r="G58" s="8"/>
+      <c r="H58" s="8"/>
+      <c r="I58" s="8"/>
+      <c r="J58" s="8"/>
+      <c r="K58" s="8"/>
+      <c r="L58" s="8"/>
+      <c r="M58" s="8"/>
+      <c r="N58" s="8"/>
+      <c r="O58" s="8"/>
+      <c r="P58" s="8"/>
+      <c r="Q58" s="8"/>
+      <c r="R58" s="8"/>
+      <c r="S58" s="8"/>
+      <c r="T58" s="8"/>
+      <c r="U58" s="8"/>
+      <c r="V58" s="8"/>
+      <c r="W58" s="8"/>
+      <c r="X58" s="8"/>
+      <c r="Y58" s="8"/>
+      <c r="Z58" s="8"/>
+      <c r="AA58" s="8"/>
+      <c r="AB58" s="8"/>
+      <c r="AC58" s="8"/>
+      <c r="AD58" s="8"/>
+      <c r="AE58" s="8"/>
+      <c r="AF58" s="8"/>
+      <c r="AG58" s="8"/>
+      <c r="AH58" s="8"/>
+      <c r="AI58" s="8"/>
+      <c r="AJ58" s="8"/>
+      <c r="AK58" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:37" ht="34.799999999999997" x14ac:dyDescent="0.25">
+      <c r="A59" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B59" s="10">
+        <v>90000</v>
+      </c>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+      <c r="F59" s="8"/>
+      <c r="G59" s="8"/>
+      <c r="H59" s="8"/>
+      <c r="I59" s="8"/>
+      <c r="J59" s="8"/>
+      <c r="K59" s="8"/>
+      <c r="L59" s="8"/>
+      <c r="M59" s="8"/>
+      <c r="N59" s="8"/>
+      <c r="O59" s="8"/>
+      <c r="P59" s="8"/>
+      <c r="Q59" s="8"/>
+      <c r="R59" s="8"/>
+      <c r="S59" s="8"/>
+      <c r="T59" s="8"/>
+      <c r="U59" s="8"/>
+      <c r="V59" s="8"/>
+      <c r="W59" s="8">
+        <v>60000</v>
+      </c>
+      <c r="X59" s="8">
+        <v>30000</v>
+      </c>
+      <c r="Y59" s="8"/>
+      <c r="Z59" s="8"/>
+      <c r="AA59" s="8"/>
+      <c r="AB59" s="8"/>
+      <c r="AC59" s="8"/>
+      <c r="AD59" s="8"/>
+      <c r="AE59" s="8"/>
+      <c r="AF59" s="8"/>
+      <c r="AG59" s="8"/>
+      <c r="AH59" s="8"/>
+      <c r="AI59" s="8"/>
+      <c r="AJ59" s="8"/>
+      <c r="AK59" s="10">
+        <v>90000</v>
+      </c>
+    </row>
+    <row r="60" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B60" s="12">
         <v>12085865</v>
       </c>
-      <c r="C56" s="12">
+      <c r="C60" s="12">
         <v>403175</v>
       </c>
-      <c r="D56" s="12">
+      <c r="D60" s="12">
         <v>403175</v>
       </c>
-      <c r="E56" s="12">
-        <v>0</v>
-      </c>
-      <c r="F56" s="12">
-        <v>0</v>
-      </c>
-      <c r="G56" s="12">
-        <v>0</v>
-      </c>
-      <c r="H56" s="12">
-        <v>0</v>
-      </c>
-      <c r="I56" s="12">
-        <v>0</v>
-      </c>
-      <c r="J56" s="12">
-        <v>0</v>
-      </c>
-      <c r="K56" s="12">
-        <v>0</v>
-      </c>
-      <c r="L56" s="12">
-        <v>0</v>
-      </c>
-      <c r="M56" s="12">
-        <v>0</v>
-      </c>
-      <c r="N56" s="12">
-        <v>0</v>
-      </c>
-      <c r="O56" s="12">
+      <c r="E60" s="12">
+        <v>0</v>
+      </c>
+      <c r="F60" s="12">
+        <v>0</v>
+      </c>
+      <c r="G60" s="12">
+        <v>0</v>
+      </c>
+      <c r="H60" s="12">
+        <v>0</v>
+      </c>
+      <c r="I60" s="12">
+        <v>0</v>
+      </c>
+      <c r="J60" s="12">
+        <v>0</v>
+      </c>
+      <c r="K60" s="12">
+        <v>0</v>
+      </c>
+      <c r="L60" s="12">
+        <v>0</v>
+      </c>
+      <c r="M60" s="12">
+        <v>0</v>
+      </c>
+      <c r="N60" s="12">
+        <v>0</v>
+      </c>
+      <c r="O60" s="12">
         <v>728301</v>
       </c>
-      <c r="P56" s="12">
+      <c r="P60" s="12">
         <v>521426</v>
       </c>
-      <c r="Q56" s="12">
+      <c r="Q60" s="12">
         <v>180000</v>
       </c>
-      <c r="R56" s="12">
+      <c r="R60" s="12">
         <v>1139167</v>
       </c>
-      <c r="S56" s="12">
+      <c r="S60" s="12">
         <v>1539976</v>
       </c>
-      <c r="T56" s="12">
+      <c r="T60" s="12">
         <v>1943215</v>
       </c>
-      <c r="U56" s="12">
+      <c r="U60" s="12">
         <v>1035340</v>
       </c>
-      <c r="V56" s="12">
+      <c r="V60" s="12">
         <v>265355</v>
       </c>
-      <c r="W56" s="12">
+      <c r="W60" s="12">
         <v>1811270</v>
       </c>
-      <c r="X56" s="12">
+      <c r="X60" s="12">
         <v>349950</v>
       </c>
-      <c r="Y56" s="12">
+      <c r="Y60" s="12">
         <v>821658</v>
       </c>
-      <c r="Z56" s="12">
+      <c r="Z60" s="12">
         <v>477638</v>
       </c>
-      <c r="AA56" s="12">
+      <c r="AA60" s="12">
         <v>184244</v>
       </c>
-      <c r="AB56" s="12">
+      <c r="AB60" s="12">
         <v>159975</v>
       </c>
-      <c r="AC56" s="12">
-        <v>0</v>
-      </c>
-      <c r="AD56" s="12">
-        <v>0</v>
-      </c>
-      <c r="AE56" s="12">
+      <c r="AC60" s="12">
+        <v>0</v>
+      </c>
+      <c r="AD60" s="12">
+        <v>0</v>
+      </c>
+      <c r="AE60" s="12">
         <v>92000</v>
       </c>
-      <c r="AF56" s="12">
-        <v>0</v>
-      </c>
-      <c r="AG56" s="12">
-        <v>0</v>
-      </c>
-      <c r="AH56" s="12">
-        <v>0</v>
-      </c>
-      <c r="AI56" s="12">
-        <v>0</v>
-      </c>
-      <c r="AJ56" s="12">
+      <c r="AF60" s="12">
+        <v>0</v>
+      </c>
+      <c r="AG60" s="12">
+        <v>0</v>
+      </c>
+      <c r="AH60" s="12">
+        <v>0</v>
+      </c>
+      <c r="AI60" s="12">
+        <v>0</v>
+      </c>
+      <c r="AJ60" s="12">
         <v>30000</v>
       </c>
-      <c r="AK56" s="12">
+      <c r="AK60" s="12">
         <v>12085865</v>
       </c>
     </row>
-    <row r="58" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="A58" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B58" s="4"/>
-      <c r="C58" s="4"/>
-      <c r="D58" s="4"/>
-      <c r="E58" s="4"/>
-      <c r="F58" s="4"/>
-      <c r="G58" s="4"/>
-      <c r="H58" s="4"/>
-      <c r="I58" s="4"/>
-      <c r="J58" s="4"/>
-      <c r="K58" s="4"/>
-      <c r="L58" s="4"/>
-      <c r="M58" s="4"/>
-      <c r="N58" s="4"/>
-      <c r="O58" s="4"/>
-      <c r="P58" s="4"/>
-      <c r="Q58" s="4"/>
-      <c r="R58" s="4"/>
-      <c r="S58" s="4"/>
-      <c r="T58" s="4"/>
-      <c r="U58" s="4"/>
-      <c r="V58" s="4"/>
-      <c r="W58" s="4"/>
-      <c r="X58" s="4"/>
-      <c r="Y58" s="4"/>
-      <c r="Z58" s="4"/>
-      <c r="AA58" s="4"/>
-      <c r="AB58" s="4"/>
-      <c r="AC58" s="4"/>
-      <c r="AD58" s="4"/>
-      <c r="AE58" s="4"/>
-      <c r="AF58" s="4"/>
-      <c r="AG58" s="4"/>
-      <c r="AH58" s="4"/>
-      <c r="AI58" s="4"/>
-      <c r="AJ58" s="4"/>
-      <c r="AK58" s="4"/>
+    <row r="62" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="A62" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+      <c r="D62" s="4"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
+      <c r="J62" s="4"/>
+      <c r="K62" s="4"/>
+      <c r="L62" s="4"/>
+      <c r="M62" s="4"/>
+      <c r="N62" s="4"/>
+      <c r="O62" s="4"/>
+      <c r="P62" s="4"/>
+      <c r="Q62" s="4"/>
+      <c r="R62" s="4"/>
+      <c r="S62" s="4"/>
+      <c r="T62" s="4"/>
+      <c r="U62" s="4"/>
+      <c r="V62" s="4"/>
+      <c r="W62" s="4"/>
+      <c r="X62" s="4"/>
+      <c r="Y62" s="4"/>
+      <c r="Z62" s="4"/>
+      <c r="AA62" s="4"/>
+      <c r="AB62" s="4"/>
+      <c r="AC62" s="4"/>
+      <c r="AD62" s="4"/>
+      <c r="AE62" s="4"/>
+      <c r="AF62" s="4"/>
+      <c r="AG62" s="4"/>
+      <c r="AH62" s="4"/>
+      <c r="AI62" s="4"/>
+      <c r="AJ62" s="4"/>
+      <c r="AK62" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A1:AK1"/>
     <mergeCell ref="A2:AK2"/>
-    <mergeCell ref="A58:AK58"/>
+    <mergeCell ref="A62:AK62"/>
     <mergeCell ref="A4:AK4"/>
-    <mergeCell ref="A31:AK31"/>
+    <mergeCell ref="A33:AK33"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-01 08:31)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE3BD12D-062C-4472-97D0-BAAFCDD5C2E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9049F1E-CC30-4EF2-A8D7-3786165BEC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2172" yWindow="1776" windowWidth="13572" windowHeight="10368" xr2:uid="{9C1A0B4E-EAE1-4787-B7FF-251A4FD0E53F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{78348FD6-6710-4C6F-B1E7-DC06D2295917}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-09-25</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-01</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FD477BE-9F95-4BD4-86B1-85C5381668FA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F83889D-3E79-4ADD-B845-630E3543C40D}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1048,17 +1048,17 @@
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
-      <c r="V7" s="8">
+      <c r="V7" s="8"/>
+      <c r="W7" s="8">
         <v>41834</v>
       </c>
-      <c r="W7" s="8">
+      <c r="X7" s="8">
         <v>69723</v>
       </c>
-      <c r="X7" s="8">
+      <c r="Y7" s="8"/>
+      <c r="Z7" s="8">
         <v>27889</v>
       </c>
-      <c r="Y7" s="8"/>
-      <c r="Z7" s="8"/>
       <c r="AA7" s="8"/>
       <c r="AB7" s="8"/>
       <c r="AC7" s="8"/>
@@ -1298,11 +1298,11 @@
       </c>
       <c r="U12" s="8"/>
       <c r="V12" s="8"/>
-      <c r="W12" s="8">
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8">
         <v>56000</v>
       </c>
-      <c r="X12" s="8"/>
-      <c r="Y12" s="8"/>
       <c r="Z12" s="8"/>
       <c r="AA12" s="8"/>
       <c r="AB12" s="8"/>
@@ -1539,18 +1539,18 @@
       <c r="R17" s="8"/>
       <c r="S17" s="8"/>
       <c r="T17" s="8"/>
-      <c r="U17" s="8">
+      <c r="U17" s="8"/>
+      <c r="V17" s="8">
         <v>129000</v>
       </c>
-      <c r="V17" s="8"/>
-      <c r="W17" s="8">
+      <c r="W17" s="8"/>
+      <c r="X17" s="8">
         <v>215000</v>
       </c>
-      <c r="X17" s="8"/>
-      <c r="Y17" s="8">
+      <c r="Y17" s="8"/>
+      <c r="Z17" s="8">
         <v>86000</v>
       </c>
-      <c r="Z17" s="8"/>
       <c r="AA17" s="8"/>
       <c r="AB17" s="8"/>
       <c r="AC17" s="8"/>
@@ -1694,10 +1694,10 @@
         <v>140000</v>
       </c>
       <c r="V20" s="8"/>
-      <c r="W20" s="8">
+      <c r="W20" s="8"/>
+      <c r="X20" s="8">
         <v>56000</v>
       </c>
-      <c r="X20" s="8"/>
       <c r="Y20" s="8"/>
       <c r="Z20" s="8"/>
       <c r="AA20" s="8"/>
@@ -1745,10 +1745,12 @@
       <c r="T21" s="8"/>
       <c r="U21" s="8"/>
       <c r="V21" s="8">
-        <v>93540</v>
+        <v>45710</v>
       </c>
       <c r="W21" s="8"/>
-      <c r="X21" s="8"/>
+      <c r="X21" s="8">
+        <v>47830</v>
+      </c>
       <c r="Y21" s="8"/>
       <c r="Z21" s="8"/>
       <c r="AA21" s="8"/>
@@ -1797,9 +1799,11 @@
       <c r="U22" s="8"/>
       <c r="V22" s="8"/>
       <c r="W22" s="8">
-        <v>67268</v>
-      </c>
-      <c r="X22" s="8"/>
+        <v>22423</v>
+      </c>
+      <c r="X22" s="8">
+        <v>44845</v>
+      </c>
       <c r="Y22" s="8"/>
       <c r="Z22" s="8"/>
       <c r="AA22" s="8"/>
@@ -1842,15 +1846,15 @@
       <c r="S23" s="8"/>
       <c r="T23" s="8"/>
       <c r="U23" s="8"/>
-      <c r="V23" s="8">
+      <c r="V23" s="8"/>
+      <c r="W23" s="8"/>
+      <c r="X23" s="8"/>
+      <c r="Y23" s="8">
         <v>65400</v>
       </c>
-      <c r="W23" s="8">
+      <c r="Z23" s="8">
         <v>109000</v>
       </c>
-      <c r="X23" s="8"/>
-      <c r="Y23" s="8"/>
-      <c r="Z23" s="8"/>
       <c r="AA23" s="8"/>
       <c r="AB23" s="8"/>
       <c r="AC23" s="8"/>
@@ -1992,10 +1996,10 @@
       <c r="V26" s="8">
         <v>52931</v>
       </c>
-      <c r="W26" s="8">
+      <c r="W26" s="8"/>
+      <c r="X26" s="8">
         <v>123505</v>
       </c>
-      <c r="X26" s="8"/>
       <c r="Y26" s="8"/>
       <c r="Z26" s="8"/>
       <c r="AA26" s="8"/>
@@ -2266,22 +2270,22 @@
         <v>739676</v>
       </c>
       <c r="U31" s="12">
-        <v>327000</v>
+        <v>198000</v>
       </c>
       <c r="V31" s="12">
-        <v>457379</v>
+        <v>431315</v>
       </c>
       <c r="W31" s="12">
-        <v>925214</v>
+        <v>292975</v>
       </c>
       <c r="X31" s="12">
-        <v>296922</v>
+        <v>825936</v>
       </c>
       <c r="Y31" s="12">
-        <v>155974</v>
+        <v>191374</v>
       </c>
       <c r="Z31" s="12">
-        <v>187274</v>
+        <v>410163</v>
       </c>
       <c r="AA31" s="12">
         <v>0</v>
@@ -2551,14 +2555,14 @@
       <c r="T36" s="8"/>
       <c r="U36" s="8"/>
       <c r="V36" s="8"/>
-      <c r="W36" s="8">
+      <c r="W36" s="8"/>
+      <c r="X36" s="8">
         <v>163840</v>
       </c>
-      <c r="X36" s="8"/>
-      <c r="Y36" s="8">
+      <c r="Y36" s="8"/>
+      <c r="Z36" s="8">
         <v>81920</v>
       </c>
-      <c r="Z36" s="8"/>
       <c r="AA36" s="8"/>
       <c r="AB36" s="8"/>
       <c r="AC36" s="8"/>
@@ -2802,12 +2806,12 @@
       </c>
       <c r="U41" s="8"/>
       <c r="V41" s="8"/>
-      <c r="W41" s="8">
-        <v>346833</v>
-      </c>
+      <c r="W41" s="8"/>
       <c r="X41" s="8"/>
       <c r="Y41" s="8"/>
-      <c r="Z41" s="8"/>
+      <c r="Z41" s="8">
+        <v>346833</v>
+      </c>
       <c r="AA41" s="8"/>
       <c r="AB41" s="8"/>
       <c r="AC41" s="8"/>
@@ -2901,10 +2905,10 @@
       <c r="S43" s="8"/>
       <c r="T43" s="8"/>
       <c r="U43" s="8"/>
-      <c r="V43" s="8"/>
-      <c r="W43" s="8">
+      <c r="V43" s="8">
         <v>136629</v>
       </c>
+      <c r="W43" s="8"/>
       <c r="X43" s="8"/>
       <c r="Y43" s="8"/>
       <c r="Z43" s="8"/>
@@ -3053,10 +3057,10 @@
       <c r="T46" s="8"/>
       <c r="U46" s="8"/>
       <c r="V46" s="8"/>
-      <c r="W46" s="8">
+      <c r="W46" s="8"/>
+      <c r="X46" s="8">
         <v>479984</v>
       </c>
-      <c r="X46" s="8"/>
       <c r="Y46" s="8"/>
       <c r="Z46" s="8">
         <v>239992</v>
@@ -3210,10 +3214,10 @@
       <c r="V49" s="8"/>
       <c r="W49" s="8"/>
       <c r="X49" s="8"/>
-      <c r="Y49" s="8">
+      <c r="Y49" s="8"/>
+      <c r="Z49" s="8">
         <v>249844</v>
       </c>
-      <c r="Z49" s="8"/>
       <c r="AA49" s="8"/>
       <c r="AB49" s="8"/>
       <c r="AC49" s="8"/>
@@ -3310,10 +3314,10 @@
       <c r="T51" s="8"/>
       <c r="U51" s="8"/>
       <c r="V51" s="8"/>
-      <c r="W51" s="8">
+      <c r="W51" s="8"/>
+      <c r="X51" s="8">
         <v>133340</v>
       </c>
-      <c r="X51" s="8"/>
       <c r="Y51" s="8"/>
       <c r="Z51" s="8"/>
       <c r="AA51" s="8"/>
@@ -3359,12 +3363,12 @@
       </c>
       <c r="U52" s="8"/>
       <c r="V52" s="8"/>
-      <c r="W52" s="8">
-        <v>184000</v>
-      </c>
+      <c r="W52" s="8"/>
       <c r="X52" s="8"/>
       <c r="Y52" s="8"/>
-      <c r="Z52" s="8"/>
+      <c r="Z52" s="8">
+        <v>184000</v>
+      </c>
       <c r="AA52" s="8"/>
       <c r="AB52" s="8"/>
       <c r="AC52" s="8"/>
@@ -3510,10 +3514,10 @@
       <c r="V55" s="8">
         <v>164429</v>
       </c>
-      <c r="W55" s="8">
+      <c r="W55" s="8"/>
+      <c r="X55" s="8">
         <v>246644</v>
       </c>
-      <c r="X55" s="8"/>
       <c r="Y55" s="8"/>
       <c r="Z55" s="8"/>
       <c r="AA55" s="8"/>
@@ -3783,19 +3787,19 @@
         <v>1035340</v>
       </c>
       <c r="V60" s="12">
-        <v>265355</v>
+        <v>401984</v>
       </c>
       <c r="W60" s="12">
-        <v>1811270</v>
+        <v>120000</v>
       </c>
       <c r="X60" s="12">
-        <v>349950</v>
+        <v>1373758</v>
       </c>
       <c r="Y60" s="12">
-        <v>821658</v>
+        <v>489894</v>
       </c>
       <c r="Z60" s="12">
-        <v>477638</v>
+        <v>1340235</v>
       </c>
       <c r="AA60" s="12">
         <v>184244</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-01 08:46)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9049F1E-CC30-4EF2-A8D7-3786165BEC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F1B4215-3E4F-4B42-BB99-5DFFD6AEBCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{78348FD6-6710-4C6F-B1E7-DC06D2295917}"/>
+    <workbookView xWindow="2232" yWindow="1836" windowWidth="17280" windowHeight="8880" xr2:uid="{865F4A2B-85FF-420E-BAFD-E618D952D33E}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F83889D-3E79-4ADD-B845-630E3543C40D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82E8B01B-F6AC-4DCB-84D0-B4E3919A0C34}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1747,10 +1747,10 @@
       <c r="V21" s="8">
         <v>45710</v>
       </c>
-      <c r="W21" s="8"/>
-      <c r="X21" s="8">
+      <c r="W21" s="8">
         <v>47830</v>
       </c>
+      <c r="X21" s="8"/>
       <c r="Y21" s="8"/>
       <c r="Z21" s="8"/>
       <c r="AA21" s="8"/>
@@ -2276,10 +2276,10 @@
         <v>431315</v>
       </c>
       <c r="W31" s="12">
-        <v>292975</v>
+        <v>340805</v>
       </c>
       <c r="X31" s="12">
-        <v>825936</v>
+        <v>778106</v>
       </c>
       <c r="Y31" s="12">
         <v>191374</v>
@@ -3514,9 +3514,11 @@
       <c r="V55" s="8">
         <v>164429</v>
       </c>
-      <c r="W55" s="8"/>
+      <c r="W55" s="8">
+        <v>164429</v>
+      </c>
       <c r="X55" s="8">
-        <v>246644</v>
+        <v>82215</v>
       </c>
       <c r="Y55" s="8"/>
       <c r="Z55" s="8"/>
@@ -3790,10 +3792,10 @@
         <v>401984</v>
       </c>
       <c r="W60" s="12">
-        <v>120000</v>
+        <v>284429</v>
       </c>
       <c r="X60" s="12">
-        <v>1373758</v>
+        <v>1209329</v>
       </c>
       <c r="Y60" s="12">
         <v>489894</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-01 09:29)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1F1B4215-3E4F-4B42-BB99-5DFFD6AEBCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{088F58FE-C93C-4234-8097-57C41487FEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="1836" windowWidth="17280" windowHeight="8880" xr2:uid="{865F4A2B-85FF-420E-BAFD-E618D952D33E}"/>
+    <workbookView xWindow="2232" yWindow="1836" windowWidth="17280" windowHeight="8880" xr2:uid="{8658B5FA-3323-43CB-822C-7F207F3458E2}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82E8B01B-F6AC-4DCB-84D0-B4E3919A0C34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B838E5E0-6E29-41A1-8EC1-5D7669C6C7AE}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1372,7 +1372,7 @@
         <v>48</v>
       </c>
       <c r="B14" s="10">
-        <v>120000</v>
+        <v>130000</v>
       </c>
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
@@ -1395,10 +1395,10 @@
       <c r="S14" s="8"/>
       <c r="T14" s="8"/>
       <c r="U14" s="8"/>
-      <c r="V14" s="8"/>
-      <c r="W14" s="8">
-        <v>60000</v>
-      </c>
+      <c r="V14" s="8">
+        <v>70000</v>
+      </c>
+      <c r="W14" s="8"/>
       <c r="X14" s="8"/>
       <c r="Y14" s="8"/>
       <c r="Z14" s="8">
@@ -1415,7 +1415,7 @@
       <c r="AI14" s="8"/>
       <c r="AJ14" s="8"/>
       <c r="AK14" s="10">
-        <v>120000</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="15" spans="1:37" ht="69" x14ac:dyDescent="0.25">
@@ -2072,7 +2072,7 @@
         <v>62</v>
       </c>
       <c r="B28" s="10">
-        <v>0</v>
+        <v>90000</v>
       </c>
       <c r="C28" s="8"/>
       <c r="D28" s="8"/>
@@ -2094,9 +2094,15 @@
       <c r="T28" s="8"/>
       <c r="U28" s="8"/>
       <c r="V28" s="8"/>
-      <c r="W28" s="8"/>
-      <c r="X28" s="8"/>
-      <c r="Y28" s="8"/>
+      <c r="W28" s="8">
+        <v>27000</v>
+      </c>
+      <c r="X28" s="8">
+        <v>45000</v>
+      </c>
+      <c r="Y28" s="8">
+        <v>18000</v>
+      </c>
       <c r="Z28" s="8"/>
       <c r="AA28" s="8"/>
       <c r="AB28" s="8"/>
@@ -2109,7 +2115,7 @@
       <c r="AI28" s="8"/>
       <c r="AJ28" s="8"/>
       <c r="AK28" s="10">
-        <v>0</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="29" spans="1:37" ht="23.4" x14ac:dyDescent="0.25">
@@ -2213,7 +2219,7 @@
         <v>65</v>
       </c>
       <c r="B31" s="12">
-        <v>4826583</v>
+        <v>4926583</v>
       </c>
       <c r="C31" s="12">
         <v>139012</v>
@@ -2273,16 +2279,16 @@
         <v>198000</v>
       </c>
       <c r="V31" s="12">
-        <v>431315</v>
+        <v>501315</v>
       </c>
       <c r="W31" s="12">
-        <v>340805</v>
+        <v>307805</v>
       </c>
       <c r="X31" s="12">
-        <v>778106</v>
+        <v>823106</v>
       </c>
       <c r="Y31" s="12">
-        <v>191374</v>
+        <v>209374</v>
       </c>
       <c r="Z31" s="12">
         <v>410163</v>
@@ -2318,7 +2324,7 @@
         <v>30000</v>
       </c>
       <c r="AK31" s="12">
-        <v>4826583</v>
+        <v>4926583</v>
       </c>
     </row>
     <row r="33" spans="1:37" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2505,10 +2511,10 @@
         <v>130715</v>
       </c>
       <c r="U35" s="8"/>
-      <c r="V35" s="8">
+      <c r="V35" s="8"/>
+      <c r="W35" s="8">
         <v>32679</v>
       </c>
-      <c r="W35" s="8"/>
       <c r="X35" s="8"/>
       <c r="Y35" s="8"/>
       <c r="Z35" s="8"/>
@@ -3237,7 +3243,7 @@
         <v>55</v>
       </c>
       <c r="B50" s="10">
-        <v>341237</v>
+        <v>307114</v>
       </c>
       <c r="C50" s="8">
         <v>136495</v>
@@ -3262,10 +3268,10 @@
       <c r="S50" s="8"/>
       <c r="T50" s="8"/>
       <c r="U50" s="8"/>
-      <c r="V50" s="8">
-        <v>68247</v>
-      </c>
-      <c r="W50" s="8"/>
+      <c r="V50" s="8"/>
+      <c r="W50" s="8">
+        <v>34124</v>
+      </c>
       <c r="X50" s="8"/>
       <c r="Y50" s="8"/>
       <c r="Z50" s="8"/>
@@ -3280,7 +3286,7 @@
       <c r="AI50" s="8"/>
       <c r="AJ50" s="8"/>
       <c r="AK50" s="10">
-        <v>341237</v>
+        <v>307114</v>
       </c>
     </row>
     <row r="51" spans="1:37" ht="69" x14ac:dyDescent="0.25">
@@ -3288,7 +3294,7 @@
         <v>56</v>
       </c>
       <c r="B51" s="10">
-        <v>666700</v>
+        <v>700035</v>
       </c>
       <c r="C51" s="8">
         <v>266680</v>
@@ -3314,10 +3320,10 @@
       <c r="T51" s="8"/>
       <c r="U51" s="8"/>
       <c r="V51" s="8"/>
-      <c r="W51" s="8"/>
-      <c r="X51" s="8">
-        <v>133340</v>
-      </c>
+      <c r="W51" s="8">
+        <v>166675</v>
+      </c>
+      <c r="X51" s="8"/>
       <c r="Y51" s="8"/>
       <c r="Z51" s="8"/>
       <c r="AA51" s="8"/>
@@ -3331,7 +3337,7 @@
       <c r="AI51" s="8"/>
       <c r="AJ51" s="8"/>
       <c r="AK51" s="10">
-        <v>666700</v>
+        <v>700035</v>
       </c>
     </row>
     <row r="52" spans="1:37" ht="46.2" x14ac:dyDescent="0.25">
@@ -3566,7 +3572,9 @@
       <c r="W56" s="8">
         <v>60000</v>
       </c>
-      <c r="X56" s="8"/>
+      <c r="X56" s="8">
+        <v>30000</v>
+      </c>
       <c r="Y56" s="8"/>
       <c r="Z56" s="8"/>
       <c r="AA56" s="8"/>
@@ -3578,9 +3586,7 @@
       <c r="AG56" s="8"/>
       <c r="AH56" s="8"/>
       <c r="AI56" s="8"/>
-      <c r="AJ56" s="8">
-        <v>30000</v>
-      </c>
+      <c r="AJ56" s="8"/>
       <c r="AK56" s="10">
         <v>90000</v>
       </c>
@@ -3590,7 +3596,7 @@
         <v>62</v>
       </c>
       <c r="B57" s="10">
-        <v>0</v>
+        <v>133176</v>
       </c>
       <c r="C57" s="8"/>
       <c r="D57" s="8"/>
@@ -3613,7 +3619,9 @@
       <c r="U57" s="8"/>
       <c r="V57" s="8"/>
       <c r="W57" s="8"/>
-      <c r="X57" s="8"/>
+      <c r="X57" s="8">
+        <v>133176</v>
+      </c>
       <c r="Y57" s="8"/>
       <c r="Z57" s="8"/>
       <c r="AA57" s="8"/>
@@ -3627,7 +3635,7 @@
       <c r="AI57" s="8"/>
       <c r="AJ57" s="8"/>
       <c r="AK57" s="10">
-        <v>0</v>
+        <v>133176</v>
       </c>
     </row>
     <row r="58" spans="1:37" ht="23.4" x14ac:dyDescent="0.25">
@@ -3729,7 +3737,7 @@
         <v>65</v>
       </c>
       <c r="B60" s="12">
-        <v>12085865</v>
+        <v>12218253</v>
       </c>
       <c r="C60" s="12">
         <v>403175</v>
@@ -3789,13 +3797,13 @@
         <v>1035340</v>
       </c>
       <c r="V60" s="12">
-        <v>401984</v>
+        <v>301058</v>
       </c>
       <c r="W60" s="12">
-        <v>284429</v>
+        <v>517907</v>
       </c>
       <c r="X60" s="12">
-        <v>1209329</v>
+        <v>1239165</v>
       </c>
       <c r="Y60" s="12">
         <v>489894</v>
@@ -3831,10 +3839,10 @@
         <v>0</v>
       </c>
       <c r="AJ60" s="12">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="AK60" s="12">
-        <v>12085865</v>
+        <v>12218253</v>
       </c>
     </row>
     <row r="62" spans="1:37" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-01 09:32)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{088F58FE-C93C-4234-8097-57C41487FEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E015A9AF-1B12-4A95-BF31-467175FA3DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="1836" windowWidth="17280" windowHeight="8880" xr2:uid="{8658B5FA-3323-43CB-822C-7F207F3458E2}"/>
+    <workbookView xWindow="2232" yWindow="1836" windowWidth="17280" windowHeight="8880" xr2:uid="{37308FD8-B585-4D9A-A4A9-8ADBFE24A999}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B838E5E0-6E29-41A1-8EC1-5D7669C6C7AE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54E40F7B-F6CB-480B-B2C7-D4740E89F8A6}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1042,16 +1042,16 @@
       <c r="M7" s="8"/>
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
+      <c r="P7" s="8">
+        <v>41834</v>
+      </c>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
       <c r="U7" s="8"/>
       <c r="V7" s="8"/>
-      <c r="W7" s="8">
-        <v>41834</v>
-      </c>
+      <c r="W7" s="8"/>
       <c r="X7" s="8">
         <v>69723</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>229452</v>
       </c>
       <c r="P31" s="12">
-        <v>223986</v>
+        <v>265820</v>
       </c>
       <c r="Q31" s="12">
         <v>229402</v>
@@ -2282,7 +2282,7 @@
         <v>501315</v>
       </c>
       <c r="W31" s="12">
-        <v>307805</v>
+        <v>265971</v>
       </c>
       <c r="X31" s="12">
         <v>823106</v>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-07 17:04)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E015A9AF-1B12-4A95-BF31-467175FA3DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BE4C512-E11E-457E-8862-6A6C7604155C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="1836" windowWidth="17280" windowHeight="8880" xr2:uid="{37308FD8-B585-4D9A-A4A9-8ADBFE24A999}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5ABCF8B-B706-416F-9FC7-B57CAB85D9E9}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-01</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-07</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54E40F7B-F6CB-480B-B2C7-D4740E89F8A6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B808F180-E04C-402F-AFE5-9546E9FAE3F5}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-14 15:55)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BE4C512-E11E-457E-8862-6A6C7604155C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FD959E2-C141-4152-82BB-5E8596DD12C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5ABCF8B-B706-416F-9FC7-B57CAB85D9E9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1998D62-86DC-4F47-A426-DD2F0340941D}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-07</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-14</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B808F180-E04C-402F-AFE5-9546E9FAE3F5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9720CD60-6F6E-442D-B436-01EDE58FE47E}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-14 16:05)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0FD959E2-C141-4152-82BB-5E8596DD12C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C92A6D71-E89B-4753-B310-F8F8C44CE506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E1998D62-86DC-4F47-A426-DD2F0340941D}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{98B3F1B2-5442-4033-968B-C9D2071C03E9}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9720CD60-6F6E-442D-B436-01EDE58FE47E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E8BD907-AA88-49CB-9B58-3785272DB38D}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-19 10:02)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C92A6D71-E89B-4753-B310-F8F8C44CE506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB9DFC3A-9A02-4691-AB33-2F1D43D29AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{98B3F1B2-5442-4033-968B-C9D2071C03E9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7E0622DE-04D6-4B34-B65F-B681125011A6}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-14</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-19</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E8BD907-AA88-49CB-9B58-3785272DB38D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15F11255-0606-4C68-81C7-6F5BE8BFCC50}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-21 15:34)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB9DFC3A-9A02-4691-AB33-2F1D43D29AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF4DCCC5-196D-4F7D-8B36-02BD6FFA9BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7E0622DE-04D6-4B34-B65F-B681125011A6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF55DDD8-B163-4EAA-A63B-0738EA6EF11E}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-19</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-21</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15F11255-0606-4C68-81C7-6F5BE8BFCC50}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69C5EC7A-5B31-4BA1-B30D-FB03A66703DE}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-23 20:33)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BF4DCCC5-196D-4F7D-8B36-02BD6FFA9BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3547C6E-FBEA-42C7-97C6-A4764173962A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CF55DDD8-B163-4EAA-A63B-0738EA6EF11E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9E8AEC0C-5B28-42DC-9057-8A60DB7A37C2}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-21</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-23</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69C5EC7A-5B31-4BA1-B30D-FB03A66703DE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11FF7660-AE66-43A1-AD8E-823D1C1B5304}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-26 12:44)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3547C6E-FBEA-42C7-97C6-A4764173962A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DE699EE-F11F-4E20-B187-3CFD73B5F382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9E8AEC0C-5B28-42DC-9057-8A60DB7A37C2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F7BBA262-4CCC-48B9-AC19-167C4217744C}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-23</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-26</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11FF7660-AE66-43A1-AD8E-823D1C1B5304}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{434CEC48-D7C7-4DE5-B7EB-2042421ED20D}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>

<commit_message>
Sync monthly workload dashboard (2026-10-28 16:12)
</commit_message>
<xml_diff>
--- a/Financial_Forecast.xlsx
+++ b/Financial_Forecast.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HPVICTUS\AppData\Local\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DE699EE-F11F-4E20-B187-3CFD73B5F382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{72CCCEEA-7A11-4521-8AAA-08C845D6FF27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F7BBA262-4CCC-48B9-AC19-167C4217744C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F596AAD3-6999-4669-83BF-B6B1B3904E41}"/>
   </bookViews>
   <sheets>
     <sheet name="IAQ Construction" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <t>IAQ Construction - Cost &amp; Forecast Revenue รายเดือน (25 โครงการ PO)</t>
   </si>
   <si>
-    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-26</t>
+    <t>ที่มา: dashboard IAQ Construction (Construction_Portfolio_Template Data base.xlsx) · งวด 40/40/20 · ณ 2026-10-28</t>
   </si>
   <si>
     <t>① Cost รายเดือน (฿)  —  จ่ายผู้รับเหมา 30/50/20 ตามวันที่จริง</t>
@@ -724,7 +724,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{434CEC48-D7C7-4DE5-B7EB-2042421ED20D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AB2448E-01A1-4B60-9E90-77C370476BCB}">
   <dimension ref="A1:AK62"/>
   <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>